<commit_message>
8/3, 8/4, 8/5 - Returns, Sales, Purchaces
</commit_message>
<xml_diff>
--- a/docs/Chiraath-Summary-Aug26.xlsx
+++ b/docs/Chiraath-Summary-Aug26.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/anooppremachandran/Desktop/CHIRAATH/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA8A2D1C-869A-5A48-BE38-6581203DE227}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{88CB7011-580A-8F42-9B00-0A7BBA060129}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" tabRatio="500" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Notes" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">INVENTORY!$A$1:$T$188</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">Purchases!$A$1:$D$32</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">Sales!$A$1:$I$296</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">Sales!$A$1:$I$301</definedName>
   </definedNames>
   <calcPr calcId="191029" iterateDelta="1E-4"/>
   <extLst>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3197" uniqueCount="1270">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3211" uniqueCount="1272">
   <si>
     <t>Notes:</t>
   </si>
@@ -3466,9 +3466,6 @@
     <t>CHR-87 Red Salwar with Elephant print, CHR-58 Wine Red Salwar (1000 advance, 1350 balance)</t>
   </si>
   <si>
-    <t>Renju, Jisha bank</t>
-  </si>
-  <si>
     <t>Urmila</t>
   </si>
   <si>
@@ -3491,9 +3488,6 @@
   </si>
   <si>
     <t>Gincy Jibi</t>
-  </si>
-  <si>
-    <t>Sheeba George, Soji Thomas, Jessy Joseph, Jeeja Anil ,Sanam, Geetha, Sushama Bhaskar, Divya Jacob, Baby Johny, Jayasree, Navya, Bindu Saji, Vanajakshi, Dison Jose, Akshitha, Bahuleyan, Urmila, Gincy Jibi, Razia Salim</t>
   </si>
   <si>
     <t>Green/maroon - Rajitha Teacher,  chikku green - Razia Salim, Rust Orange/Coffee Brown - Nishida, Chikku Maroon(1200) - Nishida, Komalavalli - Red/green, peacock blue/navy - returned, mustard/blue - girija(1200)</t>
@@ -3678,9 +3672,6 @@
     <t>CHR-111 white cotton salwar, Banarasi golden yellow blue</t>
   </si>
   <si>
-    <t>CHR-212 - Red, CHR-214 - Yellow/Blue Chanderi Silk, CHR-95 Chinon Silk</t>
-  </si>
-  <si>
     <t>Teena mathew - Paeach</t>
   </si>
   <si>
@@ -3843,9 +3834,6 @@
     <t>Parrot Green Banarasi - 6 pieces from bulk</t>
   </si>
   <si>
-    <t>1250 X 6</t>
-  </si>
-  <si>
     <t>Asha Sandran</t>
   </si>
   <si>
@@ -3861,19 +3849,37 @@
     <t>Prabha Chidambaram - Purple/Green</t>
   </si>
   <si>
-    <t>Maroon/Mustard, Green/Coffee Brown</t>
-  </si>
-  <si>
     <t>CHR-223 - Purple/Green, CHR-229 - Black</t>
   </si>
   <si>
-    <t>Rajan</t>
-  </si>
-  <si>
     <t>Blue, Wine</t>
   </si>
   <si>
     <t>Prabha Chidambaram - Green</t>
+  </si>
+  <si>
+    <t>Green/Coffee Brown</t>
+  </si>
+  <si>
+    <t>Prabha Chithambaram</t>
+  </si>
+  <si>
+    <t>Sheeba George, Soji Thomas, Jessy Joseph, Jeeja Anil ,Sanam, Geetha, Sushama Bhaskar, Divya Jacob, Baby Johny, Jayasree, Navya, Bindu Saji, Vanajakshi, Dison Jose, Akshitha, Bahuleyan, Urmila, Gincy Jibi, Razia Salim, Komalavalli</t>
+  </si>
+  <si>
+    <t>Asha Sharath (Haritha Karma Sena Bulk - 11 pieces)</t>
+  </si>
+  <si>
+    <t>Parrot Green Banarasi - 11 pieces from bulk</t>
+  </si>
+  <si>
+    <t>1250 X 6, 1250 X 11</t>
+  </si>
+  <si>
+    <t>Renju</t>
+  </si>
+  <si>
+    <t>CHR-212 - Red, CHR-214 - Yellow/Blue Chanderi Silk - 1380 advance for the returned saree, 920 pending</t>
   </si>
 </sst>
 </file>
@@ -4759,7 +4765,7 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>307</c:v>
+                  <c:v>317</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>96</c:v>
@@ -4862,7 +4868,7 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>216</c:v>
+                  <c:v>204</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>54</c:v>
@@ -5195,7 +5201,7 @@
                   <c:v>57128</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>160465.19666666666</c:v>
+                  <c:v>150163.43666666665</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>1062</c:v>
@@ -5531,7 +5537,7 @@
                   <c:v>102200</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0</c:v>
+                  <c:v>9387</c:v>
                 </c:pt>
                 <c:pt idx="8">
                   <c:v>0</c:v>
@@ -5688,10 +5694,10 @@
                   <c:v>72885</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>62696</c:v>
+                  <c:v>61746</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>9829</c:v>
+                  <c:v>26489</c:v>
                 </c:pt>
                 <c:pt idx="8">
                   <c:v>0</c:v>
@@ -6128,10 +6134,10 @@
                   <c:v>-26158</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>-39504</c:v>
+                  <c:v>-40454</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>9829</c:v>
+                  <c:v>17102</c:v>
                 </c:pt>
                 <c:pt idx="8">
                   <c:v>0</c:v>
@@ -6592,10 +6598,10 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="2"/>
                 <c:pt idx="0">
-                  <c:v>408</c:v>
+                  <c:v>418</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>273</c:v>
+                  <c:v>261</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -7767,7 +7773,7 @@
       </c>
       <c r="B3" s="8">
         <f>SUM(Purchases!C:C)</f>
-        <v>556347</v>
+        <v>565734</v>
       </c>
       <c r="E3" s="8" t="s">
         <v>42</v>
@@ -7782,7 +7788,7 @@
       </c>
       <c r="B4" s="10">
         <f>SUMIFS(Sales!C:C, Sales!I:I, "Completed")</f>
-        <v>485923</v>
+        <v>499953</v>
       </c>
       <c r="E4" s="9" t="str">
         <f>PartnerShares!A3</f>
@@ -7799,7 +7805,7 @@
       </c>
       <c r="B5" s="12">
         <f>SUM(Sales!C:C)</f>
-        <v>503653</v>
+        <v>516733</v>
       </c>
       <c r="E5" s="11" t="str">
         <f>PartnerShares!A4</f>
@@ -7816,7 +7822,7 @@
       </c>
       <c r="B6" s="10">
         <f>B4-B3</f>
-        <v>-70424</v>
+        <v>-65781</v>
       </c>
       <c r="E6" s="9" t="str">
         <f>PartnerShares!A5</f>
@@ -7851,7 +7857,7 @@
       </c>
       <c r="B10" s="13">
         <f>PartnerShares!H8</f>
-        <v>48677.66</v>
+        <v>54935.66</v>
       </c>
       <c r="C10" s="9"/>
     </row>
@@ -7861,7 +7867,7 @@
       </c>
       <c r="B11" s="14">
         <f>PartnerShares!H9</f>
-        <v>44228.67</v>
+        <v>41099.67</v>
       </c>
       <c r="C11" s="11"/>
     </row>
@@ -7871,7 +7877,7 @@
       </c>
       <c r="B12" s="13">
         <f>PartnerShares!H10</f>
-        <v>-92906.33</v>
+        <v>-96035.33</v>
       </c>
       <c r="C12" s="9"/>
     </row>
@@ -7910,15 +7916,15 @@
       </c>
       <c r="B18" s="10">
         <f>PartnerShares!B8</f>
-        <v>252430</v>
+        <v>261817</v>
       </c>
       <c r="C18" s="10">
         <f>PartnerShares!C8</f>
-        <v>185449</v>
+        <v>188578</v>
       </c>
       <c r="D18" s="10">
         <f>PartnerShares!D8</f>
-        <v>66981</v>
+        <v>73239</v>
       </c>
       <c r="E18" s="10">
         <f>IFERROR(SUMIFS(PartnerShares!$E$14:$E$500,PartnerShares!$D$14:$D$500,$A18,PartnerShares!$B$14:$B$500,"Contribution"),0)-IFERROR(SUMIFS(PartnerShares!$E$14:$E$500,PartnerShares!$C$14:$C$500,$A18,PartnerShares!$B$14:$B$500,"Contribution"),0)</f>
@@ -7926,11 +7932,11 @@
       </c>
       <c r="F18" s="13">
         <f>D18-E18</f>
-        <v>48677.66</v>
+        <v>54935.66</v>
       </c>
       <c r="G18" s="16" t="str">
         <f>IF(ROUND(F18,0)&gt;0,"Receive ₹"&amp;TEXT(ABS(F18),"#,##0"),IF(ROUND(F18,0)&lt;0,"Pay ₹"&amp;TEXT(ABS(F18),"#,##0"),"✓ Settled"))</f>
-        <v>Receive ₹48,678</v>
+        <v>Receive ₹54,936</v>
       </c>
     </row>
     <row r="19" spans="1:7" ht="13.5" customHeight="1">
@@ -7944,11 +7950,11 @@
       </c>
       <c r="C19" s="12">
         <f>PartnerShares!C9</f>
-        <v>185449</v>
+        <v>188578</v>
       </c>
       <c r="D19" s="12">
         <f>PartnerShares!D9</f>
-        <v>85868</v>
+        <v>82739</v>
       </c>
       <c r="E19" s="12">
         <f>IFERROR(SUMIFS(PartnerShares!$E$14:$E$500,PartnerShares!$D$14:$D$500,$A19,PartnerShares!$B$14:$B$500,"Contribution"),0)-IFERROR(SUMIFS(PartnerShares!$E$14:$E$500,PartnerShares!$C$14:$C$500,$A19,PartnerShares!$B$14:$B$500,"Contribution"),0)</f>
@@ -7956,11 +7962,11 @@
       </c>
       <c r="F19" s="14">
         <f>D19-E19</f>
-        <v>44228.67</v>
+        <v>41099.67</v>
       </c>
       <c r="G19" s="17" t="str">
         <f>IF(ROUND(F19,0)&gt;0,"Receive ₹"&amp;TEXT(ABS(F19),"#,##0"),IF(ROUND(F19,0)&lt;0,"Pay ₹"&amp;TEXT(ABS(F19),"#,##0"),"✓ Settled"))</f>
-        <v>Receive ₹44,229</v>
+        <v>Receive ₹41,100</v>
       </c>
     </row>
     <row r="20" spans="1:7" ht="13.5" customHeight="1">
@@ -7974,11 +7980,11 @@
       </c>
       <c r="C20" s="10">
         <f>PartnerShares!C10</f>
-        <v>185449</v>
+        <v>188578</v>
       </c>
       <c r="D20" s="10">
         <f>PartnerShares!D10</f>
-        <v>-152849</v>
+        <v>-155978</v>
       </c>
       <c r="E20" s="10">
         <f>IFERROR(SUMIFS(PartnerShares!$E$14:$E$500,PartnerShares!$D$14:$D$500,$A20,PartnerShares!$B$14:$B$500,"Contribution"),0)-IFERROR(SUMIFS(PartnerShares!$E$14:$E$500,PartnerShares!$C$14:$C$500,$A20,PartnerShares!$B$14:$B$500,"Contribution"),0)</f>
@@ -7986,11 +7992,11 @@
       </c>
       <c r="F20" s="13">
         <f>D20-E20</f>
-        <v>-92906.33</v>
+        <v>-96035.33</v>
       </c>
       <c r="G20" s="17" t="str">
         <f>IF(ROUND(F20,0)&gt;0,"Receive ₹"&amp;TEXT(ABS(F20),"#,##0"),IF(ROUND(F20,0)&lt;0,"Pay ₹"&amp;TEXT(ABS(F20),"#,##0"),"✓ Settled"))</f>
-        <v>Pay ₹92,906</v>
+        <v>Pay ₹96,035</v>
       </c>
     </row>
     <row r="24" spans="1:7" ht="15.75" customHeight="1">
@@ -8028,15 +8034,15 @@
       </c>
       <c r="B26" s="10">
         <f>'Cash Pool'!B4</f>
-        <v>416139</v>
+        <v>432799</v>
       </c>
       <c r="C26" s="10">
         <f>'Cash Pool'!D4</f>
-        <v>162006.72819999998</v>
+        <v>166684.3302</v>
       </c>
       <c r="D26" s="10">
         <f>'Cash Pool'!E4</f>
-        <v>254132.27180000002</v>
+        <v>266114.66980000003</v>
       </c>
       <c r="E26" s="10">
         <f>'Cash Pool'!F4</f>
@@ -8044,11 +8050,11 @@
       </c>
       <c r="F26" s="13">
         <f>'Cash Pool'!G4</f>
-        <v>116822.2458</v>
+        <v>128804.64380000002</v>
       </c>
       <c r="G26" s="17" t="str">
         <f>IF(ROUND(F26,0)&gt;0,"Pay ₹"&amp;TEXT(ABS(F26),"#,##0"),IF(ROUND(F26,0)&lt;0,"Receive ₹"&amp;TEXT(ABS(F26),"#,##0"),"✓ Settled"))</f>
-        <v>Pay ₹116,822</v>
+        <v>Pay ₹128,805</v>
       </c>
     </row>
     <row r="27" spans="1:7" ht="13.5" customHeight="1">
@@ -8062,11 +8068,11 @@
       </c>
       <c r="C27" s="12">
         <f>'Cash Pool'!D5</f>
-        <v>161909.5436</v>
+        <v>166584.33960000001</v>
       </c>
       <c r="D27" s="12">
         <f>'Cash Pool'!E5</f>
-        <v>-107285.5436</v>
+        <v>-111960.33960000001</v>
       </c>
       <c r="E27" s="12">
         <f>'Cash Pool'!F5</f>
@@ -8074,11 +8080,11 @@
       </c>
       <c r="F27" s="14">
         <f>'Cash Pool'!G5</f>
-        <v>-35698.501600000003</v>
+        <v>-40373.297600000005</v>
       </c>
       <c r="G27" s="18" t="str">
         <f>IF(ROUND(F27,0)&gt;0,"Pay ₹"&amp;TEXT(ABS(F27),"#,##0"),IF(ROUND(F27,0)&lt;0,"Receive ₹"&amp;TEXT(ABS(F27),"#,##0"),"✓ Settled"))</f>
-        <v>Receive ₹35,699</v>
+        <v>Receive ₹40,373</v>
       </c>
     </row>
     <row r="28" spans="1:7" ht="13.5" customHeight="1">
@@ -8092,11 +8098,11 @@
       </c>
       <c r="C28" s="10">
         <f>'Cash Pool'!D6</f>
-        <v>162006.72819999998</v>
+        <v>166684.3302</v>
       </c>
       <c r="D28" s="10">
         <f>'Cash Pool'!E6</f>
-        <v>-149476.72819999998</v>
+        <v>-154154.3302</v>
       </c>
       <c r="E28" s="10">
         <f>'Cash Pool'!F6</f>
@@ -8104,11 +8110,11 @@
       </c>
       <c r="F28" s="13">
         <f>'Cash Pool'!G6</f>
-        <v>-83753.744199999972</v>
+        <v>-88431.346199999985</v>
       </c>
       <c r="G28" s="16" t="str">
         <f>IF(ROUND(F28,0)&gt;0,"Pay ₹"&amp;TEXT(ABS(F28),"#,##0"),IF(ROUND(F28,0)&lt;0,"Receive ₹"&amp;TEXT(ABS(F28),"#,##0"),"✓ Settled"))</f>
-        <v>Receive ₹83,754</v>
+        <v>Receive ₹88,431</v>
       </c>
     </row>
     <row r="32" spans="1:7" ht="15.75" customHeight="1">
@@ -8220,7 +8226,7 @@
       </c>
       <c r="B3" s="20">
         <f ca="1">TODAY()</f>
-        <v>46236</v>
+        <v>46239</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="15" customHeight="1">
@@ -8229,14 +8235,14 @@
       </c>
       <c r="B5" s="21">
         <f>Summary!B3</f>
-        <v>556347</v>
+        <v>565734</v>
       </c>
       <c r="D5" s="19" t="s">
         <v>69</v>
       </c>
       <c r="E5" s="21">
         <f>Summary!B4</f>
-        <v>485923</v>
+        <v>499953</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="15" customHeight="1">
@@ -8245,14 +8251,14 @@
       </c>
       <c r="B6" s="21">
         <f>Summary!B6</f>
-        <v>-70424</v>
+        <v>-65781</v>
       </c>
       <c r="D6" s="19" t="s">
         <v>71</v>
       </c>
       <c r="E6" s="21">
         <f>SUMIFS(INVENTORY!K:K, INVENTORY!N:N, "&lt;&gt;Sold Out")</f>
-        <v>209034.39666666667</v>
+        <v>197482.63666666666</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="15.75" customHeight="1">
@@ -8304,7 +8310,7 @@
       </c>
       <c r="G10" s="21">
         <f>SUM(INVENTORY!F:F)</f>
-        <v>408</v>
+        <v>418</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="15" customHeight="1">
@@ -8328,7 +8334,7 @@
       </c>
       <c r="G11" s="27">
         <f>SUM(INVENTORY!G:G)</f>
-        <v>273</v>
+        <v>261</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="15" customHeight="1">
@@ -8409,11 +8415,11 @@
       </c>
       <c r="C16" s="21">
         <f>IFERROR(SUMPRODUCT((TEXT(Sales!$A$2:$A$994,"MMM")=$A16)*(YEAR(Sales!$A$2:$A$994)=$B$7)*Sales!$C$2:$C$994),0)</f>
-        <v>62696</v>
+        <v>61746</v>
       </c>
       <c r="D16" s="21">
         <f t="shared" si="0"/>
-        <v>-39504</v>
+        <v>-40454</v>
       </c>
     </row>
     <row r="17" spans="1:4" ht="15" customHeight="1">
@@ -8422,15 +8428,15 @@
       </c>
       <c r="B17" s="27">
         <f>IFERROR(SUMPRODUCT((TEXT(Purchases!$A$2:$A$998,"MMM")=$A17)*(YEAR(Purchases!$A$2:$A$998)=$B$7)*Purchases!$C$2:$C$998),0)</f>
-        <v>0</v>
+        <v>9387</v>
       </c>
       <c r="C17" s="27">
         <f>IFERROR(SUMPRODUCT((TEXT(Sales!$A$2:$A$994,"MMM")=$A17)*(YEAR(Sales!$A$2:$A$994)=$B$7)*Sales!$C$2:$C$994),0)</f>
-        <v>9829</v>
+        <v>26489</v>
       </c>
       <c r="D17" s="27">
         <f t="shared" si="0"/>
-        <v>9829</v>
+        <v>17102</v>
       </c>
     </row>
     <row r="18" spans="1:4" ht="15" customHeight="1">
@@ -8524,11 +8530,11 @@
       </c>
       <c r="G47" s="30">
         <f>SUMIF(INVENTORY!C:C, F47, INVENTORY!F:F)</f>
-        <v>307</v>
+        <v>317</v>
       </c>
       <c r="H47" s="30">
         <f>SUMIF(INVENTORY!C:C, F47, INVENTORY!G:G)</f>
-        <v>216</v>
+        <v>204</v>
       </c>
       <c r="J47" s="30" t="s">
         <v>96</v>
@@ -8555,7 +8561,7 @@
       </c>
       <c r="K48" s="31">
         <f t="array" ref="K48">SUMPRODUCT((INVENTORY!$C$2:$C$477=J48)*(INVENTORY!$D$2:$D$477)*(INVENTORY!$G$2:$G$477))</f>
-        <v>160465.19666666666</v>
+        <v>150163.43666666665</v>
       </c>
     </row>
     <row r="49" spans="5:12" ht="15" customHeight="1">
@@ -9998,7 +10004,7 @@
         <v>70</v>
       </c>
       <c r="D96" s="36" t="s">
-        <v>1147</v>
+        <v>1145</v>
       </c>
     </row>
     <row r="97" spans="1:4" ht="15" customHeight="1">
@@ -10012,7 +10018,7 @@
         <v>1375</v>
       </c>
       <c r="D97" s="39" t="s">
-        <v>1148</v>
+        <v>1146</v>
       </c>
     </row>
     <row r="98" spans="1:4" ht="15" customHeight="1">
@@ -10026,7 +10032,7 @@
         <v>189</v>
       </c>
       <c r="D98" s="36" t="s">
-        <v>1149</v>
+        <v>1147</v>
       </c>
     </row>
     <row r="99" spans="1:4" ht="15" customHeight="1">
@@ -10114,16 +10120,32 @@
       </c>
     </row>
     <row r="105" spans="1:4" ht="15" customHeight="1">
-      <c r="A105" s="38"/>
-      <c r="B105" s="39"/>
-      <c r="C105" s="40"/>
-      <c r="D105" s="39"/>
+      <c r="A105" s="38">
+        <v>46238</v>
+      </c>
+      <c r="B105" s="39" t="s">
+        <v>49</v>
+      </c>
+      <c r="C105" s="40">
+        <v>757</v>
+      </c>
+      <c r="D105" s="39" t="s">
+        <v>119</v>
+      </c>
     </row>
     <row r="106" spans="1:4" ht="15" customHeight="1">
-      <c r="A106" s="35"/>
-      <c r="B106" s="36"/>
-      <c r="C106" s="37"/>
-      <c r="D106" s="36"/>
+      <c r="A106" s="35">
+        <v>46239</v>
+      </c>
+      <c r="B106" s="36" t="s">
+        <v>49</v>
+      </c>
+      <c r="C106" s="37">
+        <v>8630</v>
+      </c>
+      <c r="D106" s="36" t="s">
+        <v>118</v>
+      </c>
     </row>
     <row r="107" spans="1:4" ht="15" customHeight="1">
       <c r="A107" s="38"/>
@@ -12198,6 +12220,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:I329"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="13"/>
   <cols>
@@ -12242,7 +12265,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="2" spans="1:9" ht="14">
+    <row r="2" spans="1:9" ht="14" hidden="1">
       <c r="A2" s="82">
         <v>45900</v>
       </c>
@@ -12265,7 +12288,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="3" spans="1:9" ht="14">
+    <row r="3" spans="1:9" ht="14" hidden="1">
       <c r="A3" s="84">
         <v>45900</v>
       </c>
@@ -12288,7 +12311,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="4" spans="1:9" ht="14">
+    <row r="4" spans="1:9" ht="14" hidden="1">
       <c r="A4" s="82">
         <v>45900</v>
       </c>
@@ -12311,7 +12334,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="5" spans="1:9" ht="14">
+    <row r="5" spans="1:9" ht="14" hidden="1">
       <c r="A5" s="84">
         <v>45900</v>
       </c>
@@ -12334,7 +12357,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="6" spans="1:9" ht="14">
+    <row r="6" spans="1:9" ht="14" hidden="1">
       <c r="A6" s="82">
         <v>45900</v>
       </c>
@@ -12357,7 +12380,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="7" spans="1:9" ht="14">
+    <row r="7" spans="1:9" ht="14" hidden="1">
       <c r="A7" s="84">
         <v>45900</v>
       </c>
@@ -12380,7 +12403,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="8" spans="1:9" ht="14">
+    <row r="8" spans="1:9" ht="14" hidden="1">
       <c r="A8" s="82">
         <v>45900</v>
       </c>
@@ -12403,7 +12426,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="9" spans="1:9" ht="14">
+    <row r="9" spans="1:9" ht="14" hidden="1">
       <c r="A9" s="84">
         <v>45901</v>
       </c>
@@ -12426,7 +12449,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="10" spans="1:9" ht="14">
+    <row r="10" spans="1:9" ht="14" hidden="1">
       <c r="A10" s="82">
         <v>45902</v>
       </c>
@@ -12449,7 +12472,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="11" spans="1:9" ht="14">
+    <row r="11" spans="1:9" ht="14" hidden="1">
       <c r="A11" s="84">
         <v>45903</v>
       </c>
@@ -12472,7 +12495,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="12" spans="1:9" ht="14">
+    <row r="12" spans="1:9" ht="14" hidden="1">
       <c r="A12" s="82">
         <v>45904</v>
       </c>
@@ -12495,7 +12518,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="13" spans="1:9" ht="14">
+    <row r="13" spans="1:9" ht="14" hidden="1">
       <c r="A13" s="84">
         <v>45905</v>
       </c>
@@ -12518,7 +12541,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="14" spans="1:9" ht="14">
+    <row r="14" spans="1:9" ht="14" hidden="1">
       <c r="A14" s="82">
         <v>45906</v>
       </c>
@@ -12541,7 +12564,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="15" spans="1:9" ht="14">
+    <row r="15" spans="1:9" ht="14" hidden="1">
       <c r="A15" s="84">
         <v>45907</v>
       </c>
@@ -12564,7 +12587,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="16" spans="1:9" ht="14">
+    <row r="16" spans="1:9" ht="14" hidden="1">
       <c r="A16" s="82">
         <v>45908</v>
       </c>
@@ -12587,7 +12610,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="17" spans="1:9" ht="14">
+    <row r="17" spans="1:9" ht="14" hidden="1">
       <c r="A17" s="84">
         <v>45909</v>
       </c>
@@ -12610,7 +12633,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="18" spans="1:9" ht="14">
+    <row r="18" spans="1:9" ht="14" hidden="1">
       <c r="A18" s="82">
         <v>45910</v>
       </c>
@@ -12633,7 +12656,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="19" spans="1:9" ht="14">
+    <row r="19" spans="1:9" ht="14" hidden="1">
       <c r="A19" s="84">
         <v>45911</v>
       </c>
@@ -12656,7 +12679,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="20" spans="1:9" ht="14">
+    <row r="20" spans="1:9" ht="14" hidden="1">
       <c r="A20" s="82">
         <v>45912</v>
       </c>
@@ -12679,7 +12702,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="21" spans="1:9" ht="14">
+    <row r="21" spans="1:9" ht="14" hidden="1">
       <c r="A21" s="84">
         <v>45913</v>
       </c>
@@ -12702,7 +12725,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="22" spans="1:9" ht="14">
+    <row r="22" spans="1:9" ht="14" hidden="1">
       <c r="A22" s="82">
         <v>45914</v>
       </c>
@@ -12725,7 +12748,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="23" spans="1:9" ht="14">
+    <row r="23" spans="1:9" ht="14" hidden="1">
       <c r="A23" s="84">
         <v>45915</v>
       </c>
@@ -12748,7 +12771,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="24" spans="1:9" ht="14">
+    <row r="24" spans="1:9" ht="14" hidden="1">
       <c r="A24" s="82">
         <v>45916</v>
       </c>
@@ -12771,7 +12794,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="25" spans="1:9" ht="14">
+    <row r="25" spans="1:9" ht="14" hidden="1">
       <c r="A25" s="84">
         <v>45917</v>
       </c>
@@ -12794,7 +12817,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="26" spans="1:9" ht="14">
+    <row r="26" spans="1:9" ht="14" hidden="1">
       <c r="A26" s="82">
         <v>45917</v>
       </c>
@@ -12817,7 +12840,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="27" spans="1:9" ht="14">
+    <row r="27" spans="1:9" ht="14" hidden="1">
       <c r="A27" s="84">
         <v>45918</v>
       </c>
@@ -12840,7 +12863,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="28" spans="1:9" ht="14">
+    <row r="28" spans="1:9" ht="14" hidden="1">
       <c r="A28" s="82">
         <v>45919</v>
       </c>
@@ -12863,7 +12886,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="29" spans="1:9" ht="14">
+    <row r="29" spans="1:9" ht="14" hidden="1">
       <c r="A29" s="84">
         <v>45920</v>
       </c>
@@ -12886,7 +12909,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="30" spans="1:9" ht="14">
+    <row r="30" spans="1:9" ht="14" hidden="1">
       <c r="A30" s="82">
         <v>45921</v>
       </c>
@@ -12909,7 +12932,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="31" spans="1:9" ht="14">
+    <row r="31" spans="1:9" ht="14" hidden="1">
       <c r="A31" s="84">
         <v>45922</v>
       </c>
@@ -12932,7 +12955,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="32" spans="1:9" ht="14">
+    <row r="32" spans="1:9" ht="14" hidden="1">
       <c r="A32" s="82">
         <v>45924</v>
       </c>
@@ -12955,7 +12978,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="33" spans="1:9" ht="14">
+    <row r="33" spans="1:9" ht="14" hidden="1">
       <c r="A33" s="84">
         <v>45924</v>
       </c>
@@ -12978,7 +13001,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="34" spans="1:9" ht="14">
+    <row r="34" spans="1:9" ht="14" hidden="1">
       <c r="A34" s="82">
         <v>45930</v>
       </c>
@@ -13001,7 +13024,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="35" spans="1:9" ht="14">
+    <row r="35" spans="1:9" ht="14" hidden="1">
       <c r="A35" s="84">
         <v>45933.931944444397</v>
       </c>
@@ -13024,7 +13047,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="36" spans="1:9" ht="14">
+    <row r="36" spans="1:9" ht="14" hidden="1">
       <c r="A36" s="82">
         <v>45934.931944386597</v>
       </c>
@@ -13047,7 +13070,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="37" spans="1:9" ht="14">
+    <row r="37" spans="1:9" ht="14" hidden="1">
       <c r="A37" s="84">
         <v>45935.931944386597</v>
       </c>
@@ -13070,7 +13093,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="38" spans="1:9" ht="14">
+    <row r="38" spans="1:9" ht="14" hidden="1">
       <c r="A38" s="82">
         <v>45939.931944444397</v>
       </c>
@@ -13093,7 +13116,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="39" spans="1:9" ht="14">
+    <row r="39" spans="1:9" ht="14" hidden="1">
       <c r="A39" s="84">
         <v>45939.931944444397</v>
       </c>
@@ -13116,7 +13139,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="40" spans="1:9" ht="14">
+    <row r="40" spans="1:9" ht="14" hidden="1">
       <c r="A40" s="82">
         <v>45945</v>
       </c>
@@ -13139,7 +13162,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="41" spans="1:9" ht="14">
+    <row r="41" spans="1:9" ht="14" hidden="1">
       <c r="A41" s="84">
         <v>45946</v>
       </c>
@@ -13162,7 +13185,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="42" spans="1:9" ht="14">
+    <row r="42" spans="1:9" ht="14" hidden="1">
       <c r="A42" s="82">
         <v>45946</v>
       </c>
@@ -13185,7 +13208,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="43" spans="1:9" ht="14">
+    <row r="43" spans="1:9" ht="14" hidden="1">
       <c r="A43" s="84">
         <v>45947</v>
       </c>
@@ -13208,7 +13231,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="44" spans="1:9" ht="14">
+    <row r="44" spans="1:9" ht="14" hidden="1">
       <c r="A44" s="82">
         <v>45948</v>
       </c>
@@ -13231,7 +13254,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="45" spans="1:9" ht="14">
+    <row r="45" spans="1:9" ht="14" hidden="1">
       <c r="A45" s="84">
         <v>45949</v>
       </c>
@@ -13254,7 +13277,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="46" spans="1:9" ht="14">
+    <row r="46" spans="1:9" ht="14" hidden="1">
       <c r="A46" s="82">
         <v>45950</v>
       </c>
@@ -13277,7 +13300,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="47" spans="1:9" ht="14">
+    <row r="47" spans="1:9" ht="14" hidden="1">
       <c r="A47" s="84">
         <v>45951</v>
       </c>
@@ -13300,7 +13323,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="48" spans="1:9" ht="14">
+    <row r="48" spans="1:9" ht="14" hidden="1">
       <c r="A48" s="82">
         <v>45964</v>
       </c>
@@ -13323,7 +13346,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="49" spans="1:9" ht="14">
+    <row r="49" spans="1:9" ht="14" hidden="1">
       <c r="A49" s="84">
         <v>45963</v>
       </c>
@@ -13346,7 +13369,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="50" spans="1:9" ht="14">
+    <row r="50" spans="1:9" ht="14" hidden="1">
       <c r="A50" s="82">
         <v>45982</v>
       </c>
@@ -13369,7 +13392,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="51" spans="1:9" ht="14">
+    <row r="51" spans="1:9" ht="14" hidden="1">
       <c r="A51" s="84">
         <v>45983</v>
       </c>
@@ -13392,7 +13415,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="52" spans="1:9" ht="14">
+    <row r="52" spans="1:9" ht="14" hidden="1">
       <c r="A52" s="82">
         <v>45984</v>
       </c>
@@ -13415,7 +13438,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="53" spans="1:9" ht="14">
+    <row r="53" spans="1:9" ht="14" hidden="1">
       <c r="A53" s="84">
         <v>45985</v>
       </c>
@@ -13438,7 +13461,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="54" spans="1:9" ht="13.5" customHeight="1">
+    <row r="54" spans="1:9" ht="13.5" hidden="1" customHeight="1">
       <c r="A54" s="82">
         <v>45986</v>
       </c>
@@ -13463,7 +13486,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="55" spans="1:9" ht="15.75" customHeight="1">
+    <row r="55" spans="1:9" ht="15.75" hidden="1" customHeight="1">
       <c r="A55" s="84">
         <v>45992</v>
       </c>
@@ -13488,7 +13511,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="56" spans="1:9" ht="13.5" customHeight="1">
+    <row r="56" spans="1:9" ht="13.5" hidden="1" customHeight="1">
       <c r="A56" s="82">
         <v>45992</v>
       </c>
@@ -13513,7 +13536,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="57" spans="1:9" ht="15.75" customHeight="1">
+    <row r="57" spans="1:9" ht="15.75" hidden="1" customHeight="1">
       <c r="A57" s="84">
         <v>45996</v>
       </c>
@@ -13538,7 +13561,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="58" spans="1:9" ht="42" customHeight="1">
+    <row r="58" spans="1:9" ht="42" hidden="1" customHeight="1">
       <c r="A58" s="82">
         <v>45996</v>
       </c>
@@ -13563,7 +13586,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="59" spans="1:9" ht="15.75" customHeight="1">
+    <row r="59" spans="1:9" ht="15.75" hidden="1" customHeight="1">
       <c r="A59" s="84">
         <v>45996</v>
       </c>
@@ -13588,7 +13611,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="60" spans="1:9" ht="13.5" customHeight="1">
+    <row r="60" spans="1:9" ht="13.5" hidden="1" customHeight="1">
       <c r="A60" s="82">
         <v>46007</v>
       </c>
@@ -13613,7 +13636,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="61" spans="1:9" ht="15.75" customHeight="1">
+    <row r="61" spans="1:9" ht="15.75" hidden="1" customHeight="1">
       <c r="A61" s="84">
         <v>46008</v>
       </c>
@@ -13640,7 +13663,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="62" spans="1:9" ht="13.5" customHeight="1">
+    <row r="62" spans="1:9" ht="13.5" hidden="1" customHeight="1">
       <c r="A62" s="82">
         <v>46008</v>
       </c>
@@ -13665,7 +13688,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="63" spans="1:9" ht="15.75" customHeight="1">
+    <row r="63" spans="1:9" ht="15.75" hidden="1" customHeight="1">
       <c r="A63" s="84">
         <v>46008</v>
       </c>
@@ -13690,7 +13713,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="64" spans="1:9" ht="15.75" customHeight="1">
+    <row r="64" spans="1:9" ht="15.75" hidden="1" customHeight="1">
       <c r="A64" s="84">
         <v>46008</v>
       </c>
@@ -13715,7 +13738,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="65" spans="1:9" ht="13.5" customHeight="1">
+    <row r="65" spans="1:9" ht="13.5" hidden="1" customHeight="1">
       <c r="A65" s="82">
         <v>46009</v>
       </c>
@@ -13740,7 +13763,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="66" spans="1:9" ht="15.75" customHeight="1">
+    <row r="66" spans="1:9" ht="15.75" hidden="1" customHeight="1">
       <c r="A66" s="84">
         <v>46010</v>
       </c>
@@ -13765,7 +13788,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="67" spans="1:9" ht="13.5" customHeight="1">
+    <row r="67" spans="1:9" ht="13.5" hidden="1" customHeight="1">
       <c r="A67" s="82">
         <v>46010</v>
       </c>
@@ -13792,7 +13815,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="68" spans="1:9" ht="31.5" customHeight="1">
+    <row r="68" spans="1:9" ht="31.5" hidden="1" customHeight="1">
       <c r="A68" s="84">
         <v>46011</v>
       </c>
@@ -13817,7 +13840,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="69" spans="1:9" ht="13.5" customHeight="1">
+    <row r="69" spans="1:9" ht="13.5" hidden="1" customHeight="1">
       <c r="A69" s="82">
         <v>46011</v>
       </c>
@@ -13842,7 +13865,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="70" spans="1:9" ht="13.5" customHeight="1">
+    <row r="70" spans="1:9" ht="13.5" hidden="1" customHeight="1">
       <c r="A70" s="82">
         <v>46011</v>
       </c>
@@ -13867,7 +13890,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="71" spans="1:9" ht="15.75" customHeight="1">
+    <row r="71" spans="1:9" ht="15.75" hidden="1" customHeight="1">
       <c r="A71" s="84">
         <v>46011</v>
       </c>
@@ -13892,7 +13915,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="72" spans="1:9" ht="27.75" customHeight="1">
+    <row r="72" spans="1:9" ht="27.75" hidden="1" customHeight="1">
       <c r="A72" s="82">
         <v>46011</v>
       </c>
@@ -13917,7 +13940,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="73" spans="1:9" ht="31.5" customHeight="1">
+    <row r="73" spans="1:9" ht="31.5" hidden="1" customHeight="1">
       <c r="A73" s="84">
         <v>46011</v>
       </c>
@@ -13942,7 +13965,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="74" spans="1:9" ht="13.5" customHeight="1">
+    <row r="74" spans="1:9" ht="13.5" hidden="1" customHeight="1">
       <c r="A74" s="82">
         <v>46013</v>
       </c>
@@ -13969,7 +13992,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="75" spans="1:9" ht="15.75" customHeight="1">
+    <row r="75" spans="1:9" ht="15.75" hidden="1" customHeight="1">
       <c r="A75" s="84">
         <v>46013</v>
       </c>
@@ -13994,7 +14017,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="76" spans="1:9" ht="15.75" customHeight="1">
+    <row r="76" spans="1:9" ht="15.75" hidden="1" customHeight="1">
       <c r="A76" s="84">
         <v>46017</v>
       </c>
@@ -14019,7 +14042,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="77" spans="1:9" ht="13.5" customHeight="1">
+    <row r="77" spans="1:9" ht="13.5" hidden="1" customHeight="1">
       <c r="A77" s="82">
         <v>46017</v>
       </c>
@@ -14044,7 +14067,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="78" spans="1:9" ht="15.75" customHeight="1">
+    <row r="78" spans="1:9" ht="15.75" hidden="1" customHeight="1">
       <c r="A78" s="84">
         <v>46017</v>
       </c>
@@ -14069,7 +14092,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="79" spans="1:9" ht="13.5" customHeight="1">
+    <row r="79" spans="1:9" ht="13.5" hidden="1" customHeight="1">
       <c r="A79" s="82">
         <v>46017</v>
       </c>
@@ -14094,7 +14117,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="80" spans="1:9" ht="15.75" customHeight="1">
+    <row r="80" spans="1:9" ht="15.75" hidden="1" customHeight="1">
       <c r="A80" s="84">
         <v>46020</v>
       </c>
@@ -14119,7 +14142,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="81" spans="1:9" ht="13.5" customHeight="1">
+    <row r="81" spans="1:9" ht="13.5" hidden="1" customHeight="1">
       <c r="A81" s="82">
         <v>46024</v>
       </c>
@@ -14144,7 +14167,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="82" spans="1:9" ht="15.75" customHeight="1">
+    <row r="82" spans="1:9" ht="15.75" hidden="1" customHeight="1">
       <c r="A82" s="84">
         <v>46024</v>
       </c>
@@ -14169,7 +14192,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="83" spans="1:9" ht="13.5" customHeight="1">
+    <row r="83" spans="1:9" ht="13.5" hidden="1" customHeight="1">
       <c r="A83" s="82">
         <v>46024</v>
       </c>
@@ -14194,7 +14217,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="84" spans="1:9" ht="15.75" customHeight="1">
+    <row r="84" spans="1:9" ht="15.75" hidden="1" customHeight="1">
       <c r="A84" s="84">
         <v>46024</v>
       </c>
@@ -14219,7 +14242,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="85" spans="1:9" ht="13.5" customHeight="1">
+    <row r="85" spans="1:9" ht="13.5" hidden="1" customHeight="1">
       <c r="A85" s="82">
         <v>46027</v>
       </c>
@@ -14244,7 +14267,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="86" spans="1:9" ht="13.5" customHeight="1">
+    <row r="86" spans="1:9" ht="13.5" hidden="1" customHeight="1">
       <c r="A86" s="82">
         <v>46028</v>
       </c>
@@ -14269,7 +14292,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="87" spans="1:9" ht="15.75" customHeight="1">
+    <row r="87" spans="1:9" ht="15.75" hidden="1" customHeight="1">
       <c r="A87" s="84">
         <v>46029</v>
       </c>
@@ -14294,7 +14317,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="88" spans="1:9" ht="13.5" customHeight="1">
+    <row r="88" spans="1:9" ht="13.5" hidden="1" customHeight="1">
       <c r="A88" s="82">
         <v>46032</v>
       </c>
@@ -14319,7 +14342,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="89" spans="1:9" ht="15.75" customHeight="1">
+    <row r="89" spans="1:9" ht="15.75" hidden="1" customHeight="1">
       <c r="A89" s="84">
         <v>46033</v>
       </c>
@@ -14344,7 +14367,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="90" spans="1:9" ht="13.5" customHeight="1">
+    <row r="90" spans="1:9" ht="13.5" hidden="1" customHeight="1">
       <c r="A90" s="82">
         <v>46033</v>
       </c>
@@ -14369,7 +14392,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="91" spans="1:9" ht="15.75" customHeight="1">
+    <row r="91" spans="1:9" ht="15.75" hidden="1" customHeight="1">
       <c r="A91" s="84">
         <v>46034</v>
       </c>
@@ -14394,7 +14417,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="92" spans="1:9" ht="27.75" customHeight="1">
+    <row r="92" spans="1:9" ht="27.75" hidden="1" customHeight="1">
       <c r="A92" s="82">
         <v>46034</v>
       </c>
@@ -14419,7 +14442,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="93" spans="1:9" ht="15.75" customHeight="1">
+    <row r="93" spans="1:9" ht="15.75" hidden="1" customHeight="1">
       <c r="A93" s="84">
         <v>46035</v>
       </c>
@@ -14444,7 +14467,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="94" spans="1:9" ht="13.5" customHeight="1">
+    <row r="94" spans="1:9" ht="13.5" hidden="1" customHeight="1">
       <c r="A94" s="82">
         <v>46036</v>
       </c>
@@ -14469,7 +14492,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="95" spans="1:9" ht="15.75" customHeight="1">
+    <row r="95" spans="1:9" ht="15.75" hidden="1" customHeight="1">
       <c r="A95" s="84">
         <v>46038</v>
       </c>
@@ -14494,7 +14517,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="96" spans="1:9" ht="13.5" customHeight="1">
+    <row r="96" spans="1:9" ht="13.5" hidden="1" customHeight="1">
       <c r="A96" s="82">
         <v>46038</v>
       </c>
@@ -14519,7 +14542,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="97" spans="1:9" ht="15.75" customHeight="1">
+    <row r="97" spans="1:9" ht="15.75" hidden="1" customHeight="1">
       <c r="A97" s="84">
         <v>46039</v>
       </c>
@@ -14544,7 +14567,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="98" spans="1:9" ht="13.5" customHeight="1">
+    <row r="98" spans="1:9" ht="13.5" hidden="1" customHeight="1">
       <c r="A98" s="82">
         <v>46040</v>
       </c>
@@ -14569,7 +14592,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="99" spans="1:9" ht="15.75" customHeight="1">
+    <row r="99" spans="1:9" ht="15.75" hidden="1" customHeight="1">
       <c r="A99" s="84">
         <v>46041</v>
       </c>
@@ -14594,7 +14617,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="100" spans="1:9" ht="13.5" customHeight="1">
+    <row r="100" spans="1:9" ht="13.5" hidden="1" customHeight="1">
       <c r="A100" s="82">
         <v>46042</v>
       </c>
@@ -14619,7 +14642,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="101" spans="1:9" ht="15.75" customHeight="1">
+    <row r="101" spans="1:9" ht="15.75" hidden="1" customHeight="1">
       <c r="A101" s="84">
         <v>46043</v>
       </c>
@@ -14644,7 +14667,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="102" spans="1:9" ht="13.5" customHeight="1">
+    <row r="102" spans="1:9" ht="13.5" hidden="1" customHeight="1">
       <c r="A102" s="82">
         <v>46046</v>
       </c>
@@ -14669,7 +14692,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="103" spans="1:9" ht="13.5" customHeight="1">
+    <row r="103" spans="1:9" ht="13.5" hidden="1" customHeight="1">
       <c r="A103" s="84">
         <v>46048</v>
       </c>
@@ -14694,7 +14717,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="104" spans="1:9" ht="13.5" customHeight="1">
+    <row r="104" spans="1:9" ht="13.5" hidden="1" customHeight="1">
       <c r="A104" s="82">
         <v>46048</v>
       </c>
@@ -14719,7 +14742,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="105" spans="1:9" ht="15.75" customHeight="1">
+    <row r="105" spans="1:9" ht="15.75" hidden="1" customHeight="1">
       <c r="A105" s="84">
         <v>46049</v>
       </c>
@@ -14744,7 +14767,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="106" spans="1:9" ht="13.5" customHeight="1">
+    <row r="106" spans="1:9" ht="13.5" hidden="1" customHeight="1">
       <c r="A106" s="82">
         <v>46049</v>
       </c>
@@ -14769,7 +14792,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="107" spans="1:9" ht="15.75" customHeight="1">
+    <row r="107" spans="1:9" ht="15.75" hidden="1" customHeight="1">
       <c r="A107" s="84">
         <v>46049</v>
       </c>
@@ -14794,7 +14817,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="108" spans="1:9" ht="13.5" customHeight="1">
+    <row r="108" spans="1:9" ht="13.5" hidden="1" customHeight="1">
       <c r="A108" s="82">
         <v>46050</v>
       </c>
@@ -14819,7 +14842,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="109" spans="1:9" ht="15.75" customHeight="1">
+    <row r="109" spans="1:9" ht="15.75" hidden="1" customHeight="1">
       <c r="A109" s="84">
         <v>46051</v>
       </c>
@@ -14844,7 +14867,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="110" spans="1:9" ht="13.5" customHeight="1">
+    <row r="110" spans="1:9" ht="13.5" hidden="1" customHeight="1">
       <c r="A110" s="82">
         <v>46051</v>
       </c>
@@ -14869,7 +14892,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="111" spans="1:9" ht="15.75" customHeight="1">
+    <row r="111" spans="1:9" ht="15.75" hidden="1" customHeight="1">
       <c r="A111" s="84">
         <v>46051</v>
       </c>
@@ -14894,7 +14917,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="112" spans="1:9" ht="27.75" customHeight="1">
+    <row r="112" spans="1:9" ht="27.75" hidden="1" customHeight="1">
       <c r="A112" s="82">
         <v>46054</v>
       </c>
@@ -14919,7 +14942,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="113" spans="1:9" ht="15.75" customHeight="1">
+    <row r="113" spans="1:9" ht="15.75" hidden="1" customHeight="1">
       <c r="A113" s="84">
         <v>46054</v>
       </c>
@@ -14944,7 +14967,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="114" spans="1:9" ht="13.5" customHeight="1">
+    <row r="114" spans="1:9" ht="13.5" hidden="1" customHeight="1">
       <c r="A114" s="82">
         <v>46055</v>
       </c>
@@ -14969,7 +14992,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="115" spans="1:9" ht="15.75" customHeight="1">
+    <row r="115" spans="1:9" ht="15.75" hidden="1" customHeight="1">
       <c r="A115" s="84">
         <v>46055</v>
       </c>
@@ -14994,7 +15017,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="116" spans="1:9" ht="13.5" customHeight="1">
+    <row r="116" spans="1:9" ht="13.5" hidden="1" customHeight="1">
       <c r="A116" s="82">
         <v>46060</v>
       </c>
@@ -15019,7 +15042,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="117" spans="1:9" ht="15.75" customHeight="1">
+    <row r="117" spans="1:9" ht="15.75" hidden="1" customHeight="1">
       <c r="A117" s="84">
         <v>46062</v>
       </c>
@@ -15044,7 +15067,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="118" spans="1:9" ht="13.5" customHeight="1">
+    <row r="118" spans="1:9" ht="13.5" hidden="1" customHeight="1">
       <c r="A118" s="82">
         <v>46065</v>
       </c>
@@ -15069,7 +15092,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="119" spans="1:9" ht="15.75" customHeight="1">
+    <row r="119" spans="1:9" ht="15.75" hidden="1" customHeight="1">
       <c r="A119" s="84">
         <v>46055</v>
       </c>
@@ -15094,7 +15117,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="120" spans="1:9" ht="27.75" customHeight="1">
+    <row r="120" spans="1:9" ht="27.75" hidden="1" customHeight="1">
       <c r="A120" s="82">
         <v>46070</v>
       </c>
@@ -15119,7 +15142,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="121" spans="1:9" ht="15.75" customHeight="1">
+    <row r="121" spans="1:9" ht="15.75" hidden="1" customHeight="1">
       <c r="A121" s="84">
         <v>46073</v>
       </c>
@@ -15144,7 +15167,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="122" spans="1:9" ht="13.5" customHeight="1">
+    <row r="122" spans="1:9" ht="13.5" hidden="1" customHeight="1">
       <c r="A122" s="82">
         <v>46074</v>
       </c>
@@ -15169,7 +15192,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="123" spans="1:9" ht="15.75" customHeight="1">
+    <row r="123" spans="1:9" ht="15.75" hidden="1" customHeight="1">
       <c r="A123" s="84">
         <v>46075</v>
       </c>
@@ -15194,7 +15217,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="124" spans="1:9" ht="13.5" customHeight="1">
+    <row r="124" spans="1:9" ht="13.5" hidden="1" customHeight="1">
       <c r="A124" s="82">
         <v>46075</v>
       </c>
@@ -15219,7 +15242,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="125" spans="1:9" ht="31.5" customHeight="1">
+    <row r="125" spans="1:9" ht="31.5" hidden="1" customHeight="1">
       <c r="A125" s="84">
         <v>46079</v>
       </c>
@@ -15244,7 +15267,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="126" spans="1:9" ht="13.5" customHeight="1">
+    <row r="126" spans="1:9" ht="13.5" hidden="1" customHeight="1">
       <c r="A126" s="82">
         <v>46079</v>
       </c>
@@ -15269,7 +15292,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="127" spans="1:9" ht="13.5" customHeight="1">
+    <row r="127" spans="1:9" ht="13.5" hidden="1" customHeight="1">
       <c r="A127" s="84">
         <v>46090</v>
       </c>
@@ -15294,7 +15317,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="128" spans="1:9" ht="13.5" customHeight="1">
+    <row r="128" spans="1:9" ht="13.5" hidden="1" customHeight="1">
       <c r="A128" s="82">
         <v>46090</v>
       </c>
@@ -15319,7 +15342,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="129" spans="1:9" ht="13.5" customHeight="1">
+    <row r="129" spans="1:9" ht="13.5" hidden="1" customHeight="1">
       <c r="A129" s="82">
         <v>46090</v>
       </c>
@@ -15344,7 +15367,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="130" spans="1:9" ht="15.75" customHeight="1">
+    <row r="130" spans="1:9" ht="15.75" hidden="1" customHeight="1">
       <c r="A130" s="84">
         <v>46091</v>
       </c>
@@ -15369,7 +15392,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="131" spans="1:9" ht="13.5" customHeight="1">
+    <row r="131" spans="1:9" ht="13.5" hidden="1" customHeight="1">
       <c r="A131" s="82">
         <v>46092</v>
       </c>
@@ -15394,7 +15417,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="132" spans="1:9" ht="15.75" customHeight="1">
+    <row r="132" spans="1:9" ht="15.75" hidden="1" customHeight="1">
       <c r="A132" s="84">
         <v>46092</v>
       </c>
@@ -15419,7 +15442,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="133" spans="1:9" ht="27.75" customHeight="1">
+    <row r="133" spans="1:9" ht="27.75" hidden="1" customHeight="1">
       <c r="A133" s="82">
         <v>46093</v>
       </c>
@@ -15444,7 +15467,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="134" spans="1:9" ht="15.75" customHeight="1">
+    <row r="134" spans="1:9" ht="15.75" hidden="1" customHeight="1">
       <c r="A134" s="84">
         <v>46093</v>
       </c>
@@ -15469,7 +15492,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="135" spans="1:9" ht="13.5" customHeight="1">
+    <row r="135" spans="1:9" ht="13.5" hidden="1" customHeight="1">
       <c r="A135" s="82">
         <v>46097</v>
       </c>
@@ -15494,7 +15517,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="136" spans="1:9" ht="15.75" customHeight="1">
+    <row r="136" spans="1:9" ht="15.75" hidden="1" customHeight="1">
       <c r="A136" s="84">
         <v>46097</v>
       </c>
@@ -15519,7 +15542,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="137" spans="1:9" ht="13.5" customHeight="1">
+    <row r="137" spans="1:9" ht="13.5" hidden="1" customHeight="1">
       <c r="A137" s="82">
         <v>46100</v>
       </c>
@@ -15544,7 +15567,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="138" spans="1:9" ht="15.75" customHeight="1">
+    <row r="138" spans="1:9" ht="15.75" hidden="1" customHeight="1">
       <c r="A138" s="84">
         <v>46104</v>
       </c>
@@ -15569,7 +15592,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="139" spans="1:9" ht="27.75" customHeight="1">
+    <row r="139" spans="1:9" ht="27.75" hidden="1" customHeight="1">
       <c r="A139" s="82">
         <v>46105</v>
       </c>
@@ -15594,7 +15617,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="140" spans="1:9" ht="31.5" customHeight="1">
+    <row r="140" spans="1:9" ht="31.5" hidden="1" customHeight="1">
       <c r="A140" s="84">
         <v>46113</v>
       </c>
@@ -15619,7 +15642,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="141" spans="1:9" ht="13.5" customHeight="1">
+    <row r="141" spans="1:9" ht="13.5" hidden="1" customHeight="1">
       <c r="A141" s="82">
         <v>46118</v>
       </c>
@@ -15644,7 +15667,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="142" spans="1:9" ht="15.75" customHeight="1">
+    <row r="142" spans="1:9" ht="15.75" hidden="1" customHeight="1">
       <c r="A142" s="84">
         <v>46119</v>
       </c>
@@ -15669,7 +15692,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="143" spans="1:9" ht="13.5" customHeight="1">
+    <row r="143" spans="1:9" ht="13.5" hidden="1" customHeight="1">
       <c r="A143" s="82">
         <v>46120</v>
       </c>
@@ -15694,7 +15717,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="144" spans="1:9" ht="15.75" customHeight="1">
+    <row r="144" spans="1:9" ht="15.75" hidden="1" customHeight="1">
       <c r="A144" s="84">
         <v>46120</v>
       </c>
@@ -15719,7 +15742,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="145" spans="1:9" ht="13.5" customHeight="1">
+    <row r="145" spans="1:9" ht="13.5" hidden="1" customHeight="1">
       <c r="A145" s="82">
         <v>46120</v>
       </c>
@@ -15744,7 +15767,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="146" spans="1:9" ht="31.5" customHeight="1">
+    <row r="146" spans="1:9" ht="31.5" hidden="1" customHeight="1">
       <c r="A146" s="84">
         <v>46122</v>
       </c>
@@ -15769,7 +15792,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="147" spans="1:9" ht="13.5" customHeight="1">
+    <row r="147" spans="1:9" ht="13.5" hidden="1" customHeight="1">
       <c r="A147" s="82">
         <v>46122</v>
       </c>
@@ -15794,7 +15817,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="148" spans="1:9" ht="15.75" customHeight="1">
+    <row r="148" spans="1:9" ht="15.75" hidden="1" customHeight="1">
       <c r="A148" s="84">
         <v>46122</v>
       </c>
@@ -15819,7 +15842,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="149" spans="1:9" ht="13.5" customHeight="1">
+    <row r="149" spans="1:9" ht="13.5" hidden="1" customHeight="1">
       <c r="A149" s="82">
         <v>46122</v>
       </c>
@@ -15844,7 +15867,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="150" spans="1:9" ht="15.75" customHeight="1">
+    <row r="150" spans="1:9" ht="15.75" hidden="1" customHeight="1">
       <c r="A150" s="84">
         <v>46125</v>
       </c>
@@ -15869,7 +15892,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="151" spans="1:9" ht="13.5" customHeight="1">
+    <row r="151" spans="1:9" ht="13.5" hidden="1" customHeight="1">
       <c r="A151" s="82">
         <v>46125</v>
       </c>
@@ -15894,7 +15917,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="152" spans="1:9" ht="15.75" customHeight="1">
+    <row r="152" spans="1:9" ht="15.75" hidden="1" customHeight="1">
       <c r="A152" s="84">
         <v>46125</v>
       </c>
@@ -15919,7 +15942,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="153" spans="1:9" ht="13.5" customHeight="1">
+    <row r="153" spans="1:9" ht="13.5" hidden="1" customHeight="1">
       <c r="A153" s="82">
         <v>46125</v>
       </c>
@@ -15944,7 +15967,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="154" spans="1:9" ht="15.75" customHeight="1">
+    <row r="154" spans="1:9" ht="15.75" hidden="1" customHeight="1">
       <c r="A154" s="84">
         <v>46126</v>
       </c>
@@ -15969,7 +15992,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="155" spans="1:9" ht="13.5" customHeight="1">
+    <row r="155" spans="1:9" ht="13.5" hidden="1" customHeight="1">
       <c r="A155" s="82">
         <v>46127</v>
       </c>
@@ -15994,7 +16017,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="156" spans="1:9" ht="15.75" customHeight="1">
+    <row r="156" spans="1:9" ht="15.75" hidden="1" customHeight="1">
       <c r="A156" s="84">
         <v>46129</v>
       </c>
@@ -16019,7 +16042,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="157" spans="1:9" ht="13.5" customHeight="1">
+    <row r="157" spans="1:9" ht="13.5" hidden="1" customHeight="1">
       <c r="A157" s="82">
         <v>46129</v>
       </c>
@@ -16044,7 +16067,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="158" spans="1:9" ht="15.75" customHeight="1">
+    <row r="158" spans="1:9" ht="15.75" hidden="1" customHeight="1">
       <c r="A158" s="84">
         <v>46129</v>
       </c>
@@ -16069,7 +16092,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="159" spans="1:9" ht="13.5" customHeight="1">
+    <row r="159" spans="1:9" ht="13.5" hidden="1" customHeight="1">
       <c r="A159" s="82">
         <v>46130</v>
       </c>
@@ -16094,7 +16117,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="160" spans="1:9" ht="15.75" customHeight="1">
+    <row r="160" spans="1:9" ht="15.75" hidden="1" customHeight="1">
       <c r="A160" s="84">
         <v>46131</v>
       </c>
@@ -16119,7 +16142,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="161" spans="1:9" ht="13.5" customHeight="1">
+    <row r="161" spans="1:9" ht="13.5" hidden="1" customHeight="1">
       <c r="A161" s="82">
         <v>46132</v>
       </c>
@@ -16144,7 +16167,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="162" spans="1:9" ht="42" customHeight="1">
+    <row r="162" spans="1:9" ht="42" hidden="1" customHeight="1">
       <c r="A162" s="84">
         <v>46132</v>
       </c>
@@ -16169,7 +16192,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="163" spans="1:9" ht="13.5" customHeight="1">
+    <row r="163" spans="1:9" ht="13.5" hidden="1" customHeight="1">
       <c r="A163" s="82">
         <v>46133</v>
       </c>
@@ -16194,7 +16217,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="164" spans="1:9" ht="13.5" customHeight="1">
+    <row r="164" spans="1:9" ht="13.5" hidden="1" customHeight="1">
       <c r="A164" s="84">
         <v>46133</v>
       </c>
@@ -16219,7 +16242,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="165" spans="1:9" ht="13.5" customHeight="1">
+    <row r="165" spans="1:9" ht="13.5" hidden="1" customHeight="1">
       <c r="A165" s="82">
         <v>46133</v>
       </c>
@@ -16244,7 +16267,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="166" spans="1:9" ht="13.5" customHeight="1">
+    <row r="166" spans="1:9" ht="13.5" hidden="1" customHeight="1">
       <c r="A166" s="84">
         <v>46134</v>
       </c>
@@ -16269,7 +16292,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="167" spans="1:9" ht="13.5" customHeight="1">
+    <row r="167" spans="1:9" ht="13.5" hidden="1" customHeight="1">
       <c r="A167" s="82">
         <v>46134</v>
       </c>
@@ -16294,7 +16317,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="168" spans="1:9" ht="13.5" customHeight="1">
+    <row r="168" spans="1:9" ht="13.5" hidden="1" customHeight="1">
       <c r="A168" s="82">
         <v>46134</v>
       </c>
@@ -16319,7 +16342,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="169" spans="1:9" ht="13.5" customHeight="1">
+    <row r="169" spans="1:9" ht="13.5" hidden="1" customHeight="1">
       <c r="A169" s="84">
         <v>46134</v>
       </c>
@@ -16344,7 +16367,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="170" spans="1:9" ht="13.5" customHeight="1">
+    <row r="170" spans="1:9" ht="13.5" hidden="1" customHeight="1">
       <c r="A170" s="82">
         <v>46134</v>
       </c>
@@ -16369,7 +16392,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="171" spans="1:9" ht="13.5" customHeight="1">
+    <row r="171" spans="1:9" ht="13.5" hidden="1" customHeight="1">
       <c r="A171" s="84">
         <v>46136</v>
       </c>
@@ -16394,7 +16417,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="172" spans="1:9" ht="13.5" customHeight="1">
+    <row r="172" spans="1:9" ht="13.5" hidden="1" customHeight="1">
       <c r="A172" s="82">
         <v>46138</v>
       </c>
@@ -16419,7 +16442,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="173" spans="1:9" ht="13.5" customHeight="1">
+    <row r="173" spans="1:9" ht="13.5" hidden="1" customHeight="1">
       <c r="A173" s="84">
         <v>46138</v>
       </c>
@@ -16444,7 +16467,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="174" spans="1:9" ht="13.5" customHeight="1">
+    <row r="174" spans="1:9" ht="13.5" hidden="1" customHeight="1">
       <c r="A174" s="82">
         <v>46139</v>
       </c>
@@ -16469,7 +16492,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="175" spans="1:9" ht="13.5" customHeight="1">
+    <row r="175" spans="1:9" ht="13.5" hidden="1" customHeight="1">
       <c r="A175" s="84">
         <v>46139</v>
       </c>
@@ -16494,7 +16517,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="176" spans="1:9" ht="13.5" customHeight="1">
+    <row r="176" spans="1:9" ht="13.5" hidden="1" customHeight="1">
       <c r="A176" s="82">
         <v>46139</v>
       </c>
@@ -16519,7 +16542,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="177" spans="1:9" ht="13.5" customHeight="1">
+    <row r="177" spans="1:9" ht="13.5" hidden="1" customHeight="1">
       <c r="A177" s="84">
         <v>46140</v>
       </c>
@@ -16544,7 +16567,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="178" spans="1:9" ht="13.5" customHeight="1">
+    <row r="178" spans="1:9" ht="13.5" hidden="1" customHeight="1">
       <c r="A178" s="82">
         <v>46140</v>
       </c>
@@ -16569,7 +16592,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="179" spans="1:9" ht="13.5" customHeight="1">
+    <row r="179" spans="1:9" ht="13.5" hidden="1" customHeight="1">
       <c r="A179" s="84">
         <v>46140</v>
       </c>
@@ -16594,7 +16617,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="180" spans="1:9" ht="13.5" customHeight="1">
+    <row r="180" spans="1:9" ht="13.5" hidden="1" customHeight="1">
       <c r="A180" s="82">
         <v>46140</v>
       </c>
@@ -16619,7 +16642,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="181" spans="1:9" ht="13.5" customHeight="1">
+    <row r="181" spans="1:9" ht="13.5" hidden="1" customHeight="1">
       <c r="A181" s="84">
         <v>46141</v>
       </c>
@@ -16644,7 +16667,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="182" spans="1:9" ht="13.5" customHeight="1">
+    <row r="182" spans="1:9" ht="13.5" hidden="1" customHeight="1">
       <c r="A182" s="82">
         <v>46141</v>
       </c>
@@ -16669,7 +16692,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="183" spans="1:9" ht="13.5" customHeight="1">
+    <row r="183" spans="1:9" ht="13.5" hidden="1" customHeight="1">
       <c r="A183" s="84">
         <v>46142</v>
       </c>
@@ -16694,7 +16717,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="184" spans="1:9" ht="13.5" customHeight="1">
+    <row r="184" spans="1:9" ht="13.5" hidden="1" customHeight="1">
       <c r="A184" s="82">
         <v>46142</v>
       </c>
@@ -16719,7 +16742,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="185" spans="1:9" ht="13.5" customHeight="1">
+    <row r="185" spans="1:9" ht="13.5" hidden="1" customHeight="1">
       <c r="A185" s="84">
         <v>46142</v>
       </c>
@@ -16744,7 +16767,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="186" spans="1:9" ht="13.5" customHeight="1">
+    <row r="186" spans="1:9" ht="13.5" hidden="1" customHeight="1">
       <c r="A186" s="84">
         <v>46144</v>
       </c>
@@ -16769,7 +16792,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="187" spans="1:9" ht="13.5" customHeight="1">
+    <row r="187" spans="1:9" ht="13.5" hidden="1" customHeight="1">
       <c r="A187" s="82">
         <v>46144</v>
       </c>
@@ -16794,7 +16817,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="188" spans="1:9" ht="13.5" customHeight="1">
+    <row r="188" spans="1:9" ht="13.5" hidden="1" customHeight="1">
       <c r="A188" s="84">
         <v>46145</v>
       </c>
@@ -16819,7 +16842,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="189" spans="1:9" ht="13.5" customHeight="1">
+    <row r="189" spans="1:9" ht="13.5" hidden="1" customHeight="1">
       <c r="A189" s="82">
         <v>46145</v>
       </c>
@@ -16844,7 +16867,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="190" spans="1:9" ht="13.5" customHeight="1">
+    <row r="190" spans="1:9" ht="13.5" hidden="1" customHeight="1">
       <c r="A190" s="84">
         <v>46145</v>
       </c>
@@ -16869,7 +16892,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="191" spans="1:9" ht="42" customHeight="1">
+    <row r="191" spans="1:9" ht="42" hidden="1" customHeight="1">
       <c r="A191" s="82">
         <v>46151</v>
       </c>
@@ -16894,7 +16917,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="192" spans="1:9" ht="27.75" customHeight="1">
+    <row r="192" spans="1:9" ht="27.75" hidden="1" customHeight="1">
       <c r="A192" s="84">
         <v>46152</v>
       </c>
@@ -16919,7 +16942,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="193" spans="1:9" ht="42" customHeight="1">
+    <row r="193" spans="1:9" ht="42" hidden="1" customHeight="1">
       <c r="A193" s="82">
         <v>46152</v>
       </c>
@@ -16944,7 +16967,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="194" spans="1:9" ht="27.75" customHeight="1">
+    <row r="194" spans="1:9" ht="27.75" hidden="1" customHeight="1">
       <c r="A194" s="84">
         <v>46151</v>
       </c>
@@ -16969,7 +16992,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="195" spans="1:9" ht="42" customHeight="1">
+    <row r="195" spans="1:9" ht="42" hidden="1" customHeight="1">
       <c r="A195" s="82">
         <v>46155</v>
       </c>
@@ -16994,7 +17017,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="196" spans="1:9" ht="42" customHeight="1">
+    <row r="196" spans="1:9" ht="42" hidden="1" customHeight="1">
       <c r="A196" s="84">
         <v>46155</v>
       </c>
@@ -17019,7 +17042,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="197" spans="1:9" ht="42" customHeight="1">
+    <row r="197" spans="1:9" ht="42" hidden="1" customHeight="1">
       <c r="A197" s="82">
         <v>46155</v>
       </c>
@@ -17044,7 +17067,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="198" spans="1:9" ht="42" customHeight="1">
+    <row r="198" spans="1:9" ht="42" hidden="1" customHeight="1">
       <c r="A198" s="84">
         <v>46168</v>
       </c>
@@ -17069,7 +17092,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="199" spans="1:9" ht="13.5" customHeight="1">
+    <row r="199" spans="1:9" ht="13.5" hidden="1" customHeight="1">
       <c r="A199" s="82">
         <v>46172</v>
       </c>
@@ -17094,7 +17117,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="200" spans="1:9" ht="27.75" customHeight="1">
+    <row r="200" spans="1:9" ht="27.75" hidden="1" customHeight="1">
       <c r="A200" s="84">
         <v>46173</v>
       </c>
@@ -17119,7 +17142,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="201" spans="1:9" ht="27.75" customHeight="1">
+    <row r="201" spans="1:9" ht="27.75" hidden="1" customHeight="1">
       <c r="A201" s="82">
         <v>46173</v>
       </c>
@@ -17144,7 +17167,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="202" spans="1:9" ht="13.5" customHeight="1">
+    <row r="202" spans="1:9" ht="13.5" hidden="1" customHeight="1">
       <c r="A202" s="84">
         <v>46173</v>
       </c>
@@ -17194,7 +17217,7 @@
         <v>356</v>
       </c>
     </row>
-    <row r="204" spans="1:9" ht="13.5" customHeight="1">
+    <row r="204" spans="1:9" ht="13.5" hidden="1" customHeight="1">
       <c r="A204" s="84">
         <v>46175</v>
       </c>
@@ -17219,7 +17242,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="205" spans="1:9" ht="13.5" customHeight="1">
+    <row r="205" spans="1:9" ht="13.5" hidden="1" customHeight="1">
       <c r="A205" s="82">
         <v>46175</v>
       </c>
@@ -17244,7 +17267,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="206" spans="1:9" ht="13.5" customHeight="1">
+    <row r="206" spans="1:9" ht="13.5" hidden="1" customHeight="1">
       <c r="A206" s="84">
         <v>46175</v>
       </c>
@@ -17269,7 +17292,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="207" spans="1:9" ht="13.5" customHeight="1">
+    <row r="207" spans="1:9" ht="13.5" hidden="1" customHeight="1">
       <c r="A207" s="82">
         <v>46175</v>
       </c>
@@ -17294,7 +17317,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="208" spans="1:9" ht="13.5" customHeight="1">
+    <row r="208" spans="1:9" ht="13.5" hidden="1" customHeight="1">
       <c r="A208" s="84">
         <v>46175</v>
       </c>
@@ -17319,7 +17342,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="209" spans="1:9" ht="13.5" customHeight="1">
+    <row r="209" spans="1:9" ht="13.5" hidden="1" customHeight="1">
       <c r="A209" s="82">
         <v>46176</v>
       </c>
@@ -17344,7 +17367,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="210" spans="1:9" ht="27.75" customHeight="1">
+    <row r="210" spans="1:9" ht="27.75" hidden="1" customHeight="1">
       <c r="A210" s="84">
         <v>46176</v>
       </c>
@@ -17369,7 +17392,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="211" spans="1:9" ht="13.5" customHeight="1">
+    <row r="211" spans="1:9" ht="13.5" hidden="1" customHeight="1">
       <c r="A211" s="82">
         <v>46176</v>
       </c>
@@ -17394,7 +17417,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="212" spans="1:9" ht="14">
+    <row r="212" spans="1:9" ht="14" hidden="1">
       <c r="A212" s="84">
         <v>46176</v>
       </c>
@@ -17419,7 +17442,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="213" spans="1:9" ht="13.5" customHeight="1">
+    <row r="213" spans="1:9" ht="13.5" hidden="1" customHeight="1">
       <c r="A213" s="82">
         <v>46176</v>
       </c>
@@ -17444,7 +17467,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="214" spans="1:9" ht="14">
+    <row r="214" spans="1:9" ht="14" hidden="1">
       <c r="A214" s="84">
         <v>46177</v>
       </c>
@@ -17469,7 +17492,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="215" spans="1:9" ht="13.5" customHeight="1">
+    <row r="215" spans="1:9" ht="13.5" hidden="1" customHeight="1">
       <c r="A215" s="82">
         <v>46187</v>
       </c>
@@ -17494,7 +17517,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="216" spans="1:9" ht="55.5" customHeight="1">
+    <row r="216" spans="1:9" ht="55.5" hidden="1" customHeight="1">
       <c r="A216" s="84">
         <v>46188</v>
       </c>
@@ -17519,7 +17542,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="217" spans="1:9" ht="13.5" customHeight="1">
+    <row r="217" spans="1:9" ht="13.5" hidden="1" customHeight="1">
       <c r="A217" s="84">
         <v>46191</v>
       </c>
@@ -17544,7 +17567,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="218" spans="1:9" ht="13.5" customHeight="1">
+    <row r="218" spans="1:9" ht="13.5" hidden="1" customHeight="1">
       <c r="A218" s="82">
         <v>46191</v>
       </c>
@@ -17569,7 +17592,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="219" spans="1:9" ht="13.5" customHeight="1">
+    <row r="219" spans="1:9" ht="13.5" hidden="1" customHeight="1">
       <c r="A219" s="84">
         <v>46191</v>
       </c>
@@ -17594,7 +17617,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="220" spans="1:9" ht="13.5" customHeight="1">
+    <row r="220" spans="1:9" ht="13.5" hidden="1" customHeight="1">
       <c r="A220" s="82">
         <v>46191</v>
       </c>
@@ -17619,7 +17642,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="221" spans="1:9" ht="13.5" customHeight="1">
+    <row r="221" spans="1:9" ht="13.5" hidden="1" customHeight="1">
       <c r="A221" s="84">
         <v>46191</v>
       </c>
@@ -17644,7 +17667,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="222" spans="1:9" ht="13.5" customHeight="1">
+    <row r="222" spans="1:9" ht="13.5" hidden="1" customHeight="1">
       <c r="A222" s="82">
         <v>46191</v>
       </c>
@@ -17669,7 +17692,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="223" spans="1:9" ht="13.5" customHeight="1">
+    <row r="223" spans="1:9" ht="13.5" hidden="1" customHeight="1">
       <c r="A223" s="84">
         <v>46191</v>
       </c>
@@ -17694,7 +17717,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="224" spans="1:9" ht="13.5" customHeight="1">
+    <row r="224" spans="1:9" ht="13.5" hidden="1" customHeight="1">
       <c r="A224" s="82">
         <v>46192</v>
       </c>
@@ -17719,7 +17742,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="225" spans="1:9" ht="13.5" customHeight="1">
+    <row r="225" spans="1:9" ht="13.5" hidden="1" customHeight="1">
       <c r="A225" s="84">
         <v>46192</v>
       </c>
@@ -17744,7 +17767,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="226" spans="1:9" ht="13.5" customHeight="1">
+    <row r="226" spans="1:9" ht="13.5" hidden="1" customHeight="1">
       <c r="A226" s="82">
         <v>46192</v>
       </c>
@@ -17769,7 +17792,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="227" spans="1:9" ht="13.5" customHeight="1">
+    <row r="227" spans="1:9" ht="13.5" hidden="1" customHeight="1">
       <c r="A227" s="84">
         <v>46192</v>
       </c>
@@ -17794,7 +17817,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="228" spans="1:9" ht="13.5" customHeight="1">
+    <row r="228" spans="1:9" ht="13.5" hidden="1" customHeight="1">
       <c r="A228" s="82">
         <v>46193</v>
       </c>
@@ -17819,7 +17842,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="229" spans="1:9" ht="13.5" customHeight="1">
+    <row r="229" spans="1:9" ht="13.5" hidden="1" customHeight="1">
       <c r="A229" s="84">
         <v>46193</v>
       </c>
@@ -17844,7 +17867,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="230" spans="1:9" ht="13.5" customHeight="1">
+    <row r="230" spans="1:9" ht="13.5" hidden="1" customHeight="1">
       <c r="A230" s="82">
         <v>46193</v>
       </c>
@@ -17869,7 +17892,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="231" spans="1:9" ht="13.5" customHeight="1">
+    <row r="231" spans="1:9" ht="13.5" hidden="1" customHeight="1">
       <c r="A231" s="84">
         <v>46193</v>
       </c>
@@ -17894,7 +17917,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="232" spans="1:9" ht="13.5" customHeight="1">
+    <row r="232" spans="1:9" ht="13.5" hidden="1" customHeight="1">
       <c r="A232" s="82">
         <v>46193</v>
       </c>
@@ -17919,7 +17942,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="233" spans="1:9" ht="13.5" customHeight="1">
+    <row r="233" spans="1:9" ht="13.5" hidden="1" customHeight="1">
       <c r="A233" s="84">
         <v>46193</v>
       </c>
@@ -17944,7 +17967,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="234" spans="1:9" ht="27.75" customHeight="1">
+    <row r="234" spans="1:9" ht="27.75" hidden="1" customHeight="1">
       <c r="A234" s="82">
         <v>46193</v>
       </c>
@@ -17969,7 +17992,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="235" spans="1:9" ht="13.5" customHeight="1">
+    <row r="235" spans="1:9" ht="13.5" hidden="1" customHeight="1">
       <c r="A235" s="84">
         <v>46194</v>
       </c>
@@ -17994,7 +18017,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="236" spans="1:9" ht="27.75" customHeight="1">
+    <row r="236" spans="1:9" ht="27.75" hidden="1" customHeight="1">
       <c r="A236" s="82">
         <v>46194</v>
       </c>
@@ -18019,7 +18042,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="237" spans="1:9" ht="13.5" customHeight="1">
+    <row r="237" spans="1:9" ht="13.5" hidden="1" customHeight="1">
       <c r="A237" s="84">
         <v>46196</v>
       </c>
@@ -18044,7 +18067,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="238" spans="1:9" ht="13.5" customHeight="1">
+    <row r="238" spans="1:9" ht="13.5" hidden="1" customHeight="1">
       <c r="A238" s="82">
         <v>46196</v>
       </c>
@@ -18069,7 +18092,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="239" spans="1:9" ht="13.5" customHeight="1">
+    <row r="239" spans="1:9" ht="13.5" hidden="1" customHeight="1">
       <c r="A239" s="84">
         <v>46196</v>
       </c>
@@ -18094,7 +18117,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="240" spans="1:9" ht="27.75" customHeight="1">
+    <row r="240" spans="1:9" ht="27.75" hidden="1" customHeight="1">
       <c r="A240" s="82">
         <v>46196</v>
       </c>
@@ -18119,7 +18142,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="241" spans="1:9" ht="13.5" customHeight="1">
+    <row r="241" spans="1:9" ht="13.5" hidden="1" customHeight="1">
       <c r="A241" s="84">
         <v>46197</v>
       </c>
@@ -18144,7 +18167,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="242" spans="1:9" ht="13.5" customHeight="1">
+    <row r="242" spans="1:9" ht="13.5" hidden="1" customHeight="1">
       <c r="A242" s="82">
         <v>46197</v>
       </c>
@@ -18169,7 +18192,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="243" spans="1:9" ht="13.5" customHeight="1">
+    <row r="243" spans="1:9" ht="13.5" hidden="1" customHeight="1">
       <c r="A243" s="84">
         <v>46197</v>
       </c>
@@ -18194,7 +18217,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="244" spans="1:9" ht="13.5" customHeight="1">
+    <row r="244" spans="1:9" ht="13.5" hidden="1" customHeight="1">
       <c r="A244" s="82">
         <v>46197</v>
       </c>
@@ -18219,7 +18242,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="245" spans="1:9" ht="13.5" customHeight="1">
+    <row r="245" spans="1:9" ht="13.5" hidden="1" customHeight="1">
       <c r="A245" s="84">
         <v>46198</v>
       </c>
@@ -18244,7 +18267,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="246" spans="1:9" ht="13.5" customHeight="1">
+    <row r="246" spans="1:9" ht="13.5" hidden="1" customHeight="1">
       <c r="A246" s="82">
         <v>46199</v>
       </c>
@@ -18269,7 +18292,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="247" spans="1:9" ht="13.5" customHeight="1">
+    <row r="247" spans="1:9" ht="13.5" hidden="1" customHeight="1">
       <c r="A247" s="84">
         <v>46199</v>
       </c>
@@ -18294,7 +18317,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="248" spans="1:9" ht="13.5" customHeight="1">
+    <row r="248" spans="1:9" ht="13.5" hidden="1" customHeight="1">
       <c r="A248" s="82">
         <v>46199</v>
       </c>
@@ -18319,7 +18342,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="249" spans="1:9" ht="14">
+    <row r="249" spans="1:9" ht="14" hidden="1">
       <c r="A249" s="84">
         <v>46200</v>
       </c>
@@ -18365,7 +18388,7 @@
         <v>356</v>
       </c>
     </row>
-    <row r="251" spans="1:9" ht="14">
+    <row r="251" spans="1:9" ht="14" hidden="1">
       <c r="A251" s="84">
         <v>46201</v>
       </c>
@@ -18390,7 +18413,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="252" spans="1:9" ht="14">
+    <row r="252" spans="1:9" ht="14" hidden="1">
       <c r="A252" s="82">
         <v>46201</v>
       </c>
@@ -18415,7 +18438,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="253" spans="1:9" ht="14">
+    <row r="253" spans="1:9" ht="14" hidden="1">
       <c r="A253" s="84">
         <v>46201</v>
       </c>
@@ -18440,7 +18463,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="254" spans="1:9" ht="14">
+    <row r="254" spans="1:9" ht="14" hidden="1">
       <c r="A254" s="82">
         <v>46201</v>
       </c>
@@ -18465,7 +18488,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="255" spans="1:9" ht="14">
+    <row r="255" spans="1:9" ht="14" hidden="1">
       <c r="A255" s="84">
         <v>46201</v>
       </c>
@@ -18490,7 +18513,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="256" spans="1:9" ht="14">
+    <row r="256" spans="1:9" ht="14" hidden="1">
       <c r="A256" s="82">
         <v>46203</v>
       </c>
@@ -18515,7 +18538,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="257" spans="1:9" ht="14">
+    <row r="257" spans="1:9" ht="14" hidden="1">
       <c r="A257" s="84">
         <v>46204</v>
       </c>
@@ -18540,7 +18563,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="258" spans="1:9" ht="14">
+    <row r="258" spans="1:9" ht="14" hidden="1">
       <c r="A258" s="82">
         <v>46205</v>
       </c>
@@ -18565,7 +18588,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="259" spans="1:9" ht="14">
+    <row r="259" spans="1:9" ht="14" hidden="1">
       <c r="A259" s="84">
         <v>46205</v>
       </c>
@@ -18590,7 +18613,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="260" spans="1:9" ht="14">
+    <row r="260" spans="1:9" ht="14" hidden="1">
       <c r="A260" s="82">
         <v>46205</v>
       </c>
@@ -18615,7 +18638,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="261" spans="1:9" ht="14">
+    <row r="261" spans="1:9" ht="14" hidden="1">
       <c r="A261" s="84">
         <v>46205</v>
       </c>
@@ -18634,13 +18657,13 @@
       <c r="F261" s="46"/>
       <c r="G261" s="46"/>
       <c r="H261" s="46" t="s">
-        <v>1203</v>
+        <v>1201</v>
       </c>
       <c r="I261" s="45" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="262" spans="1:9" ht="14">
+    <row r="262" spans="1:9" ht="14" hidden="1">
       <c r="A262" s="82">
         <v>46206</v>
       </c>
@@ -18665,7 +18688,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="263" spans="1:9" ht="14">
+    <row r="263" spans="1:9" ht="14" hidden="1">
       <c r="A263" s="84">
         <v>46206</v>
       </c>
@@ -18740,7 +18763,7 @@
         <v>356</v>
       </c>
     </row>
-    <row r="266" spans="1:9" ht="14">
+    <row r="266" spans="1:9" ht="14" hidden="1">
       <c r="A266" s="82">
         <v>46206</v>
       </c>
@@ -18765,7 +18788,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="267" spans="1:9" ht="14">
+    <row r="267" spans="1:9" ht="14" hidden="1">
       <c r="A267" s="84">
         <v>46207</v>
       </c>
@@ -18811,7 +18834,7 @@
         <v>356</v>
       </c>
     </row>
-    <row r="269" spans="1:9" ht="14">
+    <row r="269" spans="1:9" ht="14" hidden="1">
       <c r="A269" s="84">
         <v>46209</v>
       </c>
@@ -18836,12 +18859,12 @@
         <v>148</v>
       </c>
     </row>
-    <row r="270" spans="1:9" ht="14">
+    <row r="270" spans="1:9" ht="14" hidden="1">
       <c r="A270" s="82">
         <v>46210</v>
       </c>
       <c r="B270" s="44" t="s">
-        <v>1256</v>
+        <v>1253</v>
       </c>
       <c r="C270" s="83">
         <v>3200</v>
@@ -18861,7 +18884,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="271" spans="1:9" ht="14">
+    <row r="271" spans="1:9" ht="14" hidden="1">
       <c r="A271" s="84">
         <v>46211</v>
       </c>
@@ -18886,12 +18909,12 @@
         <v>148</v>
       </c>
     </row>
-    <row r="272" spans="1:9" ht="14">
+    <row r="272" spans="1:9" ht="14" hidden="1">
       <c r="A272" s="82">
         <v>46215</v>
       </c>
       <c r="B272" s="44" t="s">
-        <v>1135</v>
+        <v>1134</v>
       </c>
       <c r="C272" s="83">
         <v>1380</v>
@@ -18911,12 +18934,12 @@
         <v>148</v>
       </c>
     </row>
-    <row r="273" spans="1:9" ht="14">
+    <row r="273" spans="1:9" ht="14" hidden="1">
       <c r="A273" s="84">
         <v>46215</v>
       </c>
       <c r="B273" s="45" t="s">
-        <v>1136</v>
+        <v>1135</v>
       </c>
       <c r="C273" s="85">
         <v>699</v>
@@ -18936,7 +18959,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="274" spans="1:9" ht="14">
+    <row r="274" spans="1:9" ht="14" hidden="1">
       <c r="A274" s="82">
         <v>46215</v>
       </c>
@@ -18955,18 +18978,18 @@
       <c r="F274" s="44"/>
       <c r="G274" s="44"/>
       <c r="H274" s="44" t="s">
-        <v>1138</v>
+        <v>1137</v>
       </c>
       <c r="I274" s="44" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="275" spans="1:9" ht="14">
+    <row r="275" spans="1:9" ht="14" hidden="1">
       <c r="A275" s="84">
         <v>46216</v>
       </c>
       <c r="B275" s="45" t="s">
-        <v>1139</v>
+        <v>1138</v>
       </c>
       <c r="C275" s="85">
         <v>699</v>
@@ -18986,12 +19009,12 @@
         <v>148</v>
       </c>
     </row>
-    <row r="276" spans="1:9" ht="14">
+    <row r="276" spans="1:9" ht="14" hidden="1">
       <c r="A276" s="82">
         <v>46216</v>
       </c>
       <c r="B276" s="44" t="s">
-        <v>1141</v>
+        <v>1140</v>
       </c>
       <c r="C276" s="83">
         <v>3000</v>
@@ -19005,18 +19028,18 @@
       <c r="F276" s="44"/>
       <c r="G276" s="44"/>
       <c r="H276" s="44" t="s">
-        <v>1140</v>
+        <v>1139</v>
       </c>
       <c r="I276" s="44" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="277" spans="1:9" ht="14">
+    <row r="277" spans="1:9" ht="14" hidden="1">
       <c r="A277" s="84">
         <v>46219</v>
       </c>
       <c r="B277" s="45" t="s">
-        <v>1142</v>
+        <v>1141</v>
       </c>
       <c r="C277" s="85">
         <v>1380</v>
@@ -19036,7 +19059,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="278" spans="1:9" ht="14">
+    <row r="278" spans="1:9" ht="14" hidden="1">
       <c r="A278" s="82">
         <v>46219</v>
       </c>
@@ -19061,7 +19084,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="279" spans="1:9" ht="14">
+    <row r="279" spans="1:9" ht="14" hidden="1">
       <c r="A279" s="84">
         <v>46219</v>
       </c>
@@ -19080,13 +19103,13 @@
       <c r="F279" s="46"/>
       <c r="G279" s="46"/>
       <c r="H279" s="46" t="s">
-        <v>1146</v>
+        <v>1144</v>
       </c>
       <c r="I279" s="45" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="280" spans="1:9" ht="14">
+    <row r="280" spans="1:9" ht="14" hidden="1">
       <c r="A280" s="82">
         <v>46219</v>
       </c>
@@ -19105,13 +19128,13 @@
       <c r="F280" s="44"/>
       <c r="G280" s="44"/>
       <c r="H280" s="44" t="s">
-        <v>1152</v>
+        <v>1150</v>
       </c>
       <c r="I280" s="44" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="281" spans="1:9" ht="14">
+    <row r="281" spans="1:9" ht="14" hidden="1">
       <c r="A281" s="84">
         <v>46219</v>
       </c>
@@ -19130,18 +19153,18 @@
       <c r="F281" s="46"/>
       <c r="G281" s="46"/>
       <c r="H281" s="46" t="s">
-        <v>1157</v>
+        <v>1155</v>
       </c>
       <c r="I281" s="45" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="282" spans="1:9" ht="14">
+    <row r="282" spans="1:9" ht="14" hidden="1">
       <c r="A282" s="82">
         <v>46220</v>
       </c>
       <c r="B282" s="44" t="s">
-        <v>1167</v>
+        <v>1165</v>
       </c>
       <c r="C282" s="83">
         <v>1500</v>
@@ -19155,18 +19178,18 @@
       <c r="F282" s="44"/>
       <c r="G282" s="44"/>
       <c r="H282" s="44" t="s">
-        <v>1168</v>
+        <v>1166</v>
       </c>
       <c r="I282" s="44" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="283" spans="1:9" ht="14">
+    <row r="283" spans="1:9" ht="14" hidden="1">
       <c r="A283" s="84">
         <v>46221</v>
       </c>
       <c r="B283" s="45" t="s">
-        <v>1171</v>
+        <v>1169</v>
       </c>
       <c r="C283" s="85">
         <v>1100</v>
@@ -19180,18 +19203,18 @@
       <c r="F283" s="46"/>
       <c r="G283" s="46"/>
       <c r="H283" s="46" t="s">
-        <v>1172</v>
+        <v>1170</v>
       </c>
       <c r="I283" s="45" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="284" spans="1:9" ht="14">
+    <row r="284" spans="1:9" ht="14" hidden="1">
       <c r="A284" s="82">
         <v>46222</v>
       </c>
       <c r="B284" s="44" t="s">
-        <v>1173</v>
+        <v>1171</v>
       </c>
       <c r="C284" s="83">
         <v>850</v>
@@ -19205,18 +19228,18 @@
       <c r="F284" s="44"/>
       <c r="G284" s="44"/>
       <c r="H284" s="44" t="s">
-        <v>1174</v>
+        <v>1172</v>
       </c>
       <c r="I284" s="44" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="285" spans="1:9" ht="14">
+    <row r="285" spans="1:9" ht="14" hidden="1">
       <c r="A285" s="84">
         <v>46222</v>
       </c>
       <c r="B285" s="45" t="s">
-        <v>1175</v>
+        <v>1173</v>
       </c>
       <c r="C285" s="85">
         <v>1250</v>
@@ -19230,18 +19253,18 @@
       <c r="F285" s="46"/>
       <c r="G285" s="46"/>
       <c r="H285" s="46" t="s">
-        <v>1176</v>
+        <v>1174</v>
       </c>
       <c r="I285" s="45" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="286" spans="1:9" ht="14">
+    <row r="286" spans="1:9" ht="14" hidden="1">
       <c r="A286" s="82">
         <v>46222</v>
       </c>
       <c r="B286" s="44" t="s">
-        <v>1178</v>
+        <v>1176</v>
       </c>
       <c r="C286" s="83">
         <v>700</v>
@@ -19261,12 +19284,12 @@
         <v>148</v>
       </c>
     </row>
-    <row r="287" spans="1:9" ht="14">
+    <row r="287" spans="1:9" ht="14" hidden="1">
       <c r="A287" s="84">
         <v>46222</v>
       </c>
       <c r="B287" s="45" t="s">
-        <v>1179</v>
+        <v>1177</v>
       </c>
       <c r="C287" s="85">
         <v>699</v>
@@ -19286,12 +19309,12 @@
         <v>148</v>
       </c>
     </row>
-    <row r="288" spans="1:9" ht="14">
+    <row r="288" spans="1:9" ht="14" hidden="1">
       <c r="A288" s="82">
         <v>46223</v>
       </c>
       <c r="B288" s="44" t="s">
-        <v>1182</v>
+        <v>1180</v>
       </c>
       <c r="C288" s="83">
         <v>1380</v>
@@ -19305,18 +19328,18 @@
       <c r="F288" s="44"/>
       <c r="G288" s="44"/>
       <c r="H288" s="44" t="s">
-        <v>1183</v>
+        <v>1181</v>
       </c>
       <c r="I288" s="44" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="289" spans="1:9" ht="14">
+    <row r="289" spans="1:9" ht="14" hidden="1">
       <c r="A289" s="84">
         <v>46224</v>
       </c>
       <c r="B289" s="45" t="s">
-        <v>1185</v>
+        <v>1183</v>
       </c>
       <c r="C289" s="85">
         <v>1380</v>
@@ -19330,18 +19353,18 @@
       <c r="F289" s="46"/>
       <c r="G289" s="46"/>
       <c r="H289" s="46" t="s">
-        <v>1188</v>
+        <v>1186</v>
       </c>
       <c r="I289" s="45" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="290" spans="1:9" ht="14">
+    <row r="290" spans="1:9" ht="14" hidden="1">
       <c r="A290" s="82">
         <v>46224</v>
       </c>
       <c r="B290" s="44" t="s">
-        <v>1184</v>
+        <v>1182</v>
       </c>
       <c r="C290" s="83">
         <v>1380</v>
@@ -19355,13 +19378,13 @@
       <c r="F290" s="44"/>
       <c r="G290" s="44"/>
       <c r="H290" s="44" t="s">
-        <v>1189</v>
+        <v>1187</v>
       </c>
       <c r="I290" s="44" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="291" spans="1:9" ht="14">
+    <row r="291" spans="1:9" ht="14" hidden="1">
       <c r="A291" s="82">
         <v>46228</v>
       </c>
@@ -19380,7 +19403,7 @@
       <c r="F291" s="44"/>
       <c r="G291" s="44"/>
       <c r="H291" s="44" t="s">
-        <v>1192</v>
+        <v>1190</v>
       </c>
       <c r="I291" s="44" t="s">
         <v>148</v>
@@ -19391,7 +19414,7 @@
         <v>46229</v>
       </c>
       <c r="B292" s="45" t="s">
-        <v>1195</v>
+        <v>1193</v>
       </c>
       <c r="C292" s="85">
         <v>1900</v>
@@ -19401,7 +19424,7 @@
       <c r="F292" s="46"/>
       <c r="G292" s="46"/>
       <c r="H292" s="46" t="s">
-        <v>1254</v>
+        <v>1251</v>
       </c>
       <c r="I292" s="45" t="s">
         <v>356</v>
@@ -19422,7 +19445,7 @@
       <c r="F293" s="44"/>
       <c r="G293" s="44"/>
       <c r="H293" s="44" t="s">
-        <v>1255</v>
+        <v>1252</v>
       </c>
       <c r="I293" s="44" t="s">
         <v>356</v>
@@ -19436,14 +19459,14 @@
         <v>1109</v>
       </c>
       <c r="C294" s="85">
-        <v>3250</v>
+        <v>2300</v>
       </c>
       <c r="D294" s="45"/>
       <c r="E294" s="45"/>
       <c r="F294" s="46"/>
       <c r="G294" s="46"/>
       <c r="H294" s="46" t="s">
-        <v>1204</v>
+        <v>1271</v>
       </c>
       <c r="I294" s="45" t="s">
         <v>356</v>
@@ -19454,7 +19477,7 @@
         <v>46229</v>
       </c>
       <c r="B295" s="44" t="s">
-        <v>1207</v>
+        <v>1204</v>
       </c>
       <c r="C295" s="83">
         <v>1550</v>
@@ -19464,18 +19487,18 @@
       <c r="F295" s="44"/>
       <c r="G295" s="44"/>
       <c r="H295" s="44" t="s">
-        <v>1208</v>
+        <v>1205</v>
       </c>
       <c r="I295" s="44" t="s">
         <v>356</v>
       </c>
     </row>
-    <row r="296" spans="1:9" ht="14">
+    <row r="296" spans="1:9" ht="14" hidden="1">
       <c r="A296" s="84">
         <v>46235</v>
       </c>
       <c r="B296" s="45" t="s">
-        <v>1260</v>
+        <v>1256</v>
       </c>
       <c r="C296" s="85">
         <v>1450</v>
@@ -19489,18 +19512,18 @@
       <c r="F296" s="46"/>
       <c r="G296" s="46"/>
       <c r="H296" s="46" t="s">
-        <v>1253</v>
+        <v>1250</v>
       </c>
       <c r="I296" s="45" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="297" spans="1:9" ht="28">
+    <row r="297" spans="1:9" ht="28" hidden="1">
       <c r="A297" s="82">
         <v>46236</v>
       </c>
       <c r="B297" s="44" t="s">
-        <v>1257</v>
+        <v>1254</v>
       </c>
       <c r="C297" s="83">
         <v>6900</v>
@@ -19514,18 +19537,18 @@
       <c r="F297" s="44"/>
       <c r="G297" s="44"/>
       <c r="H297" s="44" t="s">
-        <v>1258</v>
+        <v>1255</v>
       </c>
       <c r="I297" s="44" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="298" spans="1:9" ht="14">
+    <row r="298" spans="1:9" ht="14" hidden="1">
       <c r="A298" s="84">
         <v>46236</v>
       </c>
       <c r="B298" s="45" t="s">
-        <v>1263</v>
+        <v>1259</v>
       </c>
       <c r="C298" s="85">
         <v>1479</v>
@@ -19539,15 +19562,19 @@
       <c r="F298" s="46"/>
       <c r="G298" s="46"/>
       <c r="H298" s="46" t="s">
-        <v>1262</v>
+        <v>1258</v>
       </c>
       <c r="I298" s="45" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="299" spans="1:9" ht="14">
-      <c r="A299" s="82"/>
-      <c r="B299" s="44"/>
+    <row r="299" spans="1:9" ht="14" hidden="1">
+      <c r="A299" s="82">
+        <v>46236</v>
+      </c>
+      <c r="B299" s="44" t="s">
+        <v>1265</v>
+      </c>
       <c r="C299" s="83">
         <v>2630</v>
       </c>
@@ -19555,38 +19582,66 @@
         <v>162</v>
       </c>
       <c r="E299" s="44" t="s">
-        <v>1267</v>
+        <v>49</v>
       </c>
       <c r="F299" s="44"/>
       <c r="G299" s="44"/>
       <c r="H299" s="44" t="s">
-        <v>1266</v>
+        <v>1261</v>
       </c>
       <c r="I299" s="44" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="300" spans="1:9">
-      <c r="A300" s="84"/>
-      <c r="B300" s="45"/>
-      <c r="C300" s="85"/>
-      <c r="D300" s="45"/>
-      <c r="E300" s="45"/>
+    <row r="300" spans="1:9" ht="14" hidden="1">
+      <c r="A300" s="84">
+        <v>46238</v>
+      </c>
+      <c r="B300" s="45" t="s">
+        <v>1106</v>
+      </c>
+      <c r="C300" s="85">
+        <v>1380</v>
+      </c>
+      <c r="D300" s="45" t="s">
+        <v>162</v>
+      </c>
+      <c r="E300" s="45" t="s">
+        <v>49</v>
+      </c>
       <c r="F300" s="46"/>
       <c r="G300" s="46"/>
-      <c r="H300" s="46"/>
-      <c r="I300" s="45"/>
-    </row>
-    <row r="301" spans="1:9">
-      <c r="A301" s="82"/>
-      <c r="B301" s="44"/>
-      <c r="C301" s="83"/>
-      <c r="D301" s="44"/>
-      <c r="E301" s="44"/>
+      <c r="H300" s="46" t="s">
+        <v>272</v>
+      </c>
+      <c r="I300" s="45" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="301" spans="1:9" ht="28" hidden="1">
+      <c r="A301" s="82">
+        <v>46238</v>
+      </c>
+      <c r="B301" s="44" t="s">
+        <v>1267</v>
+      </c>
+      <c r="C301" s="83">
+        <v>12650</v>
+      </c>
+      <c r="D301" s="44" t="s">
+        <v>162</v>
+      </c>
+      <c r="E301" s="44" t="s">
+        <v>49</v>
+      </c>
       <c r="F301" s="44"/>
       <c r="G301" s="44"/>
-      <c r="H301" s="44"/>
-      <c r="I301" s="44"/>
+      <c r="H301" s="44" t="s">
+        <v>1268</v>
+      </c>
+      <c r="I301" s="44" t="s">
+        <v>148</v>
+      </c>
     </row>
     <row r="302" spans="1:9">
       <c r="A302" s="84"/>
@@ -19897,7 +19952,13 @@
       <c r="I329" s="44"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I296" xr:uid="{00000000-0009-0000-0000-000004000000}"/>
+  <autoFilter ref="A1:I301" xr:uid="{00000000-0009-0000-0000-000004000000}">
+    <filterColumn colId="8">
+      <filters>
+        <filter val="Pending"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G2:G1258" xr:uid="{00000000-0002-0000-0400-000000000000}">
       <formula1>"Ordered,Pending,Completed,Cancelled"</formula1>
@@ -28324,7 +28385,7 @@
         <v>472</v>
       </c>
       <c r="L93" s="55" t="s">
-        <v>1186</v>
+        <v>1184</v>
       </c>
       <c r="M93" s="55"/>
       <c r="N93" s="52" t="s">
@@ -28460,10 +28521,10 @@
         <v>1450</v>
       </c>
       <c r="F96" s="53">
+        <v>0</v>
+      </c>
+      <c r="G96" s="53">
         <v>1</v>
-      </c>
-      <c r="G96" s="53">
-        <v>0</v>
       </c>
       <c r="H96" s="52">
         <f t="shared" si="4"/>
@@ -28475,15 +28536,13 @@
       </c>
       <c r="J96" s="52">
         <f t="shared" si="5"/>
-        <v>1250</v>
+        <v>0</v>
       </c>
       <c r="K96" s="52">
         <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="L96" s="52" t="s">
-        <v>1109</v>
-      </c>
+        <v>1250</v>
+      </c>
+      <c r="L96" s="52"/>
       <c r="M96" s="52"/>
       <c r="N96" s="52" t="s">
         <v>504</v>
@@ -29764,7 +29823,7 @@
         <v>3351.6266666666638</v>
       </c>
       <c r="L120" s="52" t="s">
-        <v>1180</v>
+        <v>1178</v>
       </c>
       <c r="M120" s="52" t="s">
         <v>49</v>
@@ -29774,7 +29833,7 @@
       </c>
       <c r="O120" s="52"/>
       <c r="P120" s="52" t="s">
-        <v>1181</v>
+        <v>1179</v>
       </c>
       <c r="Q120" s="52"/>
       <c r="R120" s="52"/>
@@ -31854,7 +31913,7 @@
         <v>0</v>
       </c>
       <c r="L147" s="55" t="s">
-        <v>1177</v>
+        <v>1175</v>
       </c>
       <c r="M147" s="55"/>
       <c r="N147" s="55" t="s">
@@ -31906,7 +31965,7 @@
         <v>1004</v>
       </c>
       <c r="L148" s="52" t="s">
-        <v>1150</v>
+        <v>1148</v>
       </c>
       <c r="M148" s="52"/>
       <c r="N148" s="52" t="s">
@@ -31958,7 +32017,7 @@
         <v>0</v>
       </c>
       <c r="L149" s="55" t="s">
-        <v>1151</v>
+        <v>1149</v>
       </c>
       <c r="M149" s="55"/>
       <c r="N149" s="55" t="s">
@@ -32280,7 +32339,7 @@
         <v>949</v>
       </c>
       <c r="L155" s="55" t="s">
-        <v>1137</v>
+        <v>1136</v>
       </c>
       <c r="M155" s="55"/>
       <c r="N155" s="55" t="s">
@@ -32756,7 +32815,7 @@
         <v>0</v>
       </c>
       <c r="L164" s="52" t="s">
-        <v>1156</v>
+        <v>1154</v>
       </c>
       <c r="M164" s="52"/>
       <c r="N164" s="52" t="s">
@@ -33215,11 +33274,11 @@
         <v>1</v>
       </c>
       <c r="G173" s="64">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H173" s="63">
         <f t="shared" si="11"/>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I173" s="63">
         <f>IF(D173&lt;&gt;"",D173,IFERROR(E173/(IFERROR(SUM(Sales!C:C),0))*(IFERROR(SUM(Purchases!C:C),0)),0))</f>
@@ -33231,14 +33290,14 @@
       </c>
       <c r="K173" s="63">
         <f t="shared" si="10"/>
-        <v>803.26</v>
+        <v>0</v>
       </c>
       <c r="L173" s="55" t="s">
         <v>416</v>
       </c>
       <c r="M173" s="55"/>
       <c r="N173" s="55" t="s">
-        <v>589</v>
+        <v>504</v>
       </c>
       <c r="O173" s="55"/>
       <c r="P173" s="55"/>
@@ -33765,7 +33824,7 @@
         <v>1676</v>
       </c>
       <c r="L183" s="55" t="s">
-        <v>1196</v>
+        <v>1194</v>
       </c>
       <c r="M183" s="55"/>
       <c r="N183" s="55" t="s">
@@ -33795,10 +33854,10 @@
         <v>1380</v>
       </c>
       <c r="F184" s="66">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="G184" s="66">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H184" s="65">
         <f t="shared" ref="H184:H226" si="12">F184+IF(LEN(G184)=0,0,G184)</f>
@@ -33810,18 +33869,18 @@
       </c>
       <c r="J184" s="65">
         <f t="shared" si="9"/>
-        <v>16929</v>
+        <v>17820</v>
       </c>
       <c r="K184" s="65">
         <f t="shared" si="10"/>
-        <v>891</v>
+        <v>0</v>
       </c>
       <c r="L184" s="52" t="s">
-        <v>1143</v>
+        <v>1266</v>
       </c>
       <c r="M184" s="52"/>
       <c r="N184" s="52" t="s">
-        <v>589</v>
+        <v>504</v>
       </c>
       <c r="O184" s="52"/>
       <c r="P184" s="52"/>
@@ -33999,10 +34058,10 @@
         <v>1380</v>
       </c>
       <c r="F188" s="66">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G188" s="66">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H188" s="65">
         <f t="shared" si="12"/>
@@ -34014,18 +34073,18 @@
       </c>
       <c r="J188" s="65">
         <f t="shared" si="9"/>
-        <v>1782</v>
+        <v>891</v>
       </c>
       <c r="K188" s="65">
         <f t="shared" si="10"/>
-        <v>0</v>
+        <v>891</v>
       </c>
       <c r="L188" s="52" t="s">
-        <v>1134</v>
+        <v>1270</v>
       </c>
       <c r="M188" s="52"/>
       <c r="N188" s="52" t="s">
-        <v>504</v>
+        <v>589</v>
       </c>
       <c r="O188" s="52"/>
       <c r="P188" s="52"/>
@@ -34073,7 +34132,7 @@
         <v>1782</v>
       </c>
       <c r="L189" s="55" t="s">
-        <v>1144</v>
+        <v>1142</v>
       </c>
       <c r="M189" s="55"/>
       <c r="N189" s="55" t="s">
@@ -34081,7 +34140,7 @@
       </c>
       <c r="O189" s="55"/>
       <c r="P189" s="55" t="s">
-        <v>1145</v>
+        <v>1143</v>
       </c>
       <c r="Q189" s="55"/>
       <c r="R189" s="55"/>
@@ -34127,7 +34186,7 @@
         <v>0</v>
       </c>
       <c r="L190" s="52" t="s">
-        <v>1187</v>
+        <v>1185</v>
       </c>
       <c r="M190" s="52"/>
       <c r="N190" s="47" t="s">
@@ -34424,14 +34483,14 @@
         <v>3985</v>
       </c>
       <c r="L196" s="52" t="s">
-        <v>1154</v>
+        <v>1152</v>
       </c>
       <c r="M196" s="52"/>
       <c r="N196" s="47" t="s">
         <v>589</v>
       </c>
       <c r="P196" s="47" t="s">
-        <v>1155</v>
+        <v>1153</v>
       </c>
       <c r="S196" s="47"/>
       <c r="T196" s="47"/>
@@ -34573,14 +34632,14 @@
         <v>1401</v>
       </c>
       <c r="L199" s="55" t="s">
-        <v>1205</v>
+        <v>1202</v>
       </c>
       <c r="M199" s="55"/>
       <c r="N199" s="47" t="s">
         <v>589</v>
       </c>
       <c r="P199" s="47" t="s">
-        <v>1206</v>
+        <v>1203</v>
       </c>
       <c r="S199" s="47"/>
       <c r="T199" s="47"/>
@@ -34726,14 +34785,14 @@
         <v>940</v>
       </c>
       <c r="L202" s="52" t="s">
-        <v>1169</v>
+        <v>1167</v>
       </c>
       <c r="M202" s="52"/>
       <c r="N202" s="47" t="s">
         <v>589</v>
       </c>
       <c r="P202" s="47" t="s">
-        <v>1170</v>
+        <v>1168</v>
       </c>
       <c r="S202" s="47"/>
       <c r="T202" s="47"/>
@@ -35208,10 +35267,10 @@
         <v>1380</v>
       </c>
       <c r="F212" s="66">
-        <v>6</v>
+        <v>17</v>
       </c>
       <c r="G212" s="66">
-        <v>26</v>
+        <v>15</v>
       </c>
       <c r="H212" s="65">
         <f t="shared" si="12"/>
@@ -35223,14 +35282,14 @@
       </c>
       <c r="J212" s="65">
         <f t="shared" si="13"/>
-        <v>5349</v>
+        <v>15155.5</v>
       </c>
       <c r="K212" s="65">
         <f t="shared" si="14"/>
-        <v>23179</v>
+        <v>13372.5</v>
       </c>
       <c r="L212" s="52" t="s">
-        <v>1259</v>
+        <v>1269</v>
       </c>
       <c r="M212" s="52"/>
       <c r="N212" s="47" t="s">
@@ -35244,7 +35303,7 @@
         <v>1036</v>
       </c>
       <c r="B213" s="52" t="s">
-        <v>1153</v>
+        <v>1151</v>
       </c>
       <c r="C213" s="52" t="s">
         <v>95</v>
@@ -35278,14 +35337,14 @@
         <v>3330</v>
       </c>
       <c r="L213" s="55" t="s">
-        <v>1201</v>
+        <v>1199</v>
       </c>
       <c r="M213" s="55"/>
       <c r="N213" s="47" t="s">
         <v>589</v>
       </c>
       <c r="P213" s="47" t="s">
-        <v>1202</v>
+        <v>1200</v>
       </c>
       <c r="S213" s="47"/>
       <c r="T213" s="47"/>
@@ -35295,7 +35354,7 @@
         <v>1037</v>
       </c>
       <c r="B214" s="52" t="s">
-        <v>1158</v>
+        <v>1156</v>
       </c>
       <c r="C214" s="52" t="s">
         <v>95</v>
@@ -35334,7 +35393,7 @@
         <v>678</v>
       </c>
       <c r="P214" s="47" t="s">
-        <v>1159</v>
+        <v>1157</v>
       </c>
       <c r="S214" s="47"/>
       <c r="T214" s="47"/>
@@ -35344,7 +35403,7 @@
         <v>1038</v>
       </c>
       <c r="B215" s="55" t="s">
-        <v>1160</v>
+        <v>1158</v>
       </c>
       <c r="C215" s="55" t="s">
         <v>95</v>
@@ -35378,14 +35437,14 @@
         <v>2976</v>
       </c>
       <c r="L215" s="55" t="s">
-        <v>1261</v>
+        <v>1257</v>
       </c>
       <c r="M215" s="55"/>
       <c r="N215" s="47" t="s">
         <v>589</v>
       </c>
       <c r="P215" s="47" t="s">
-        <v>1161</v>
+        <v>1159</v>
       </c>
       <c r="S215" s="47"/>
       <c r="T215" s="47"/>
@@ -35429,14 +35488,14 @@
         <v>2880</v>
       </c>
       <c r="L216" s="52" t="s">
-        <v>1199</v>
+        <v>1197</v>
       </c>
       <c r="M216" s="52"/>
       <c r="N216" s="47" t="s">
         <v>589</v>
       </c>
       <c r="P216" s="47" t="s">
-        <v>1200</v>
+        <v>1198</v>
       </c>
       <c r="S216" s="47"/>
       <c r="T216" s="47"/>
@@ -35446,7 +35505,7 @@
         <v>1040</v>
       </c>
       <c r="B217" s="55" t="s">
-        <v>1162</v>
+        <v>1160</v>
       </c>
       <c r="C217" s="55" t="s">
         <v>95</v>
@@ -35485,7 +35544,7 @@
         <v>678</v>
       </c>
       <c r="P217" s="47" t="s">
-        <v>1163</v>
+        <v>1161</v>
       </c>
       <c r="S217" s="47"/>
       <c r="T217" s="47"/>
@@ -35495,7 +35554,7 @@
         <v>1041</v>
       </c>
       <c r="B218" s="52" t="s">
-        <v>1164</v>
+        <v>1162</v>
       </c>
       <c r="C218" s="52" t="s">
         <v>95</v>
@@ -35529,14 +35588,14 @@
         <v>828</v>
       </c>
       <c r="L218" s="52" t="s">
-        <v>1197</v>
+        <v>1195</v>
       </c>
       <c r="M218" s="52"/>
       <c r="N218" s="47" t="s">
         <v>589</v>
       </c>
       <c r="P218" s="47" t="s">
-        <v>1198</v>
+        <v>1196</v>
       </c>
       <c r="S218" s="47"/>
       <c r="T218" s="47"/>
@@ -35546,7 +35605,7 @@
         <v>1042</v>
       </c>
       <c r="B219" s="55" t="s">
-        <v>1165</v>
+        <v>1163</v>
       </c>
       <c r="C219" s="55" t="s">
         <v>95</v>
@@ -35580,14 +35639,14 @@
         <v>2283</v>
       </c>
       <c r="L219" s="55" t="s">
-        <v>1210</v>
+        <v>1207</v>
       </c>
       <c r="M219" s="55"/>
       <c r="N219" s="47" t="s">
         <v>678</v>
       </c>
       <c r="P219" s="47" t="s">
-        <v>1209</v>
+        <v>1206</v>
       </c>
       <c r="S219" s="47"/>
       <c r="T219" s="47"/>
@@ -35597,7 +35656,7 @@
         <v>1043</v>
       </c>
       <c r="B220" s="52" t="s">
-        <v>1166</v>
+        <v>1164</v>
       </c>
       <c r="C220" s="52" t="s">
         <v>95</v>
@@ -35631,14 +35690,14 @@
         <v>3805</v>
       </c>
       <c r="L220" s="52" t="s">
-        <v>1193</v>
+        <v>1191</v>
       </c>
       <c r="M220" s="52"/>
       <c r="N220" s="47" t="s">
         <v>589</v>
       </c>
       <c r="P220" s="47" t="s">
-        <v>1194</v>
+        <v>1192</v>
       </c>
       <c r="S220" s="47"/>
       <c r="T220" s="47"/>
@@ -35648,7 +35707,7 @@
         <v>1044</v>
       </c>
       <c r="B221" s="55" t="s">
-        <v>1190</v>
+        <v>1188</v>
       </c>
       <c r="C221" s="55" t="s">
         <v>95</v>
@@ -35687,7 +35746,7 @@
         <v>678</v>
       </c>
       <c r="P221" s="47" t="s">
-        <v>1191</v>
+        <v>1189</v>
       </c>
       <c r="S221" s="47"/>
       <c r="T221" s="47"/>
@@ -35697,7 +35756,7 @@
         <v>1045</v>
       </c>
       <c r="B222" s="52" t="s">
-        <v>1211</v>
+        <v>1208</v>
       </c>
       <c r="C222" s="52" t="s">
         <v>96</v>
@@ -35736,7 +35795,7 @@
         <v>678</v>
       </c>
       <c r="P222" s="86" t="s">
-        <v>1238</v>
+        <v>1235</v>
       </c>
       <c r="S222" s="47"/>
       <c r="T222" s="47"/>
@@ -35746,7 +35805,7 @@
         <v>1046</v>
       </c>
       <c r="B223" s="55" t="s">
-        <v>1212</v>
+        <v>1209</v>
       </c>
       <c r="C223" s="55" t="s">
         <v>95</v>
@@ -35785,7 +35844,7 @@
         <v>678</v>
       </c>
       <c r="P223" s="86" t="s">
-        <v>1239</v>
+        <v>1236</v>
       </c>
       <c r="S223" s="47"/>
       <c r="T223" s="47"/>
@@ -35795,7 +35854,7 @@
         <v>1047</v>
       </c>
       <c r="B224" s="52" t="s">
-        <v>1213</v>
+        <v>1210</v>
       </c>
       <c r="C224" s="52" t="s">
         <v>95</v>
@@ -35810,11 +35869,11 @@
         <v>1</v>
       </c>
       <c r="G224" s="66">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H224" s="65">
         <f t="shared" si="12"/>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I224" s="65">
         <f>IF(D224&lt;&gt;"",D224,IFERROR(E224/(IFERROR(SUM(Sales!C:C),0))*(IFERROR(SUM(Purchases!C:C),0)),0))</f>
@@ -35826,17 +35885,17 @@
       </c>
       <c r="K224" s="65">
         <f t="shared" si="14"/>
-        <v>1884</v>
+        <v>942</v>
       </c>
       <c r="L224" s="52" t="s">
-        <v>1264</v>
+        <v>1260</v>
       </c>
       <c r="M224" s="52"/>
       <c r="N224" s="47" t="s">
         <v>589</v>
       </c>
       <c r="P224" s="86" t="s">
-        <v>1265</v>
+        <v>1264</v>
       </c>
       <c r="S224" s="47"/>
       <c r="T224" s="47"/>
@@ -35846,7 +35905,7 @@
         <v>1048</v>
       </c>
       <c r="B225" s="55" t="s">
-        <v>1214</v>
+        <v>1211</v>
       </c>
       <c r="C225" s="55" t="s">
         <v>95</v>
@@ -35885,7 +35944,7 @@
         <v>678</v>
       </c>
       <c r="P225" s="86" t="s">
-        <v>1240</v>
+        <v>1237</v>
       </c>
       <c r="S225" s="47"/>
       <c r="T225" s="47"/>
@@ -35895,7 +35954,7 @@
         <v>1049</v>
       </c>
       <c r="B226" s="52" t="s">
-        <v>1215</v>
+        <v>1212</v>
       </c>
       <c r="C226" s="52" t="s">
         <v>95</v>
@@ -35934,17 +35993,17 @@
         <v>678</v>
       </c>
       <c r="P226" s="86" t="s">
-        <v>1241</v>
+        <v>1238</v>
       </c>
       <c r="S226" s="47"/>
       <c r="T226" s="47"/>
     </row>
     <row r="227" spans="1:20" ht="17">
       <c r="A227" s="52" t="s">
-        <v>1226</v>
+        <v>1223</v>
       </c>
       <c r="B227" s="55" t="s">
-        <v>1216</v>
+        <v>1213</v>
       </c>
       <c r="C227" s="55" t="s">
         <v>95</v>
@@ -35983,17 +36042,17 @@
         <v>678</v>
       </c>
       <c r="P227" s="86" t="s">
-        <v>1242</v>
+        <v>1239</v>
       </c>
       <c r="S227" s="47"/>
       <c r="T227" s="47"/>
     </row>
     <row r="228" spans="1:20" ht="17">
       <c r="A228" s="55" t="s">
-        <v>1227</v>
+        <v>1224</v>
       </c>
       <c r="B228" s="52" t="s">
-        <v>1217</v>
+        <v>1214</v>
       </c>
       <c r="C228" s="52" t="s">
         <v>95</v>
@@ -36032,17 +36091,17 @@
         <v>678</v>
       </c>
       <c r="P228" s="86" t="s">
-        <v>1243</v>
+        <v>1240</v>
       </c>
       <c r="S228" s="47"/>
       <c r="T228" s="47"/>
     </row>
     <row r="229" spans="1:20" ht="17">
       <c r="A229" s="52" t="s">
-        <v>1228</v>
+        <v>1225</v>
       </c>
       <c r="B229" s="55" t="s">
-        <v>1218</v>
+        <v>1215</v>
       </c>
       <c r="C229" s="55" t="s">
         <v>95</v>
@@ -36081,17 +36140,17 @@
         <v>678</v>
       </c>
       <c r="P229" s="86" t="s">
-        <v>1244</v>
+        <v>1241</v>
       </c>
       <c r="S229" s="47"/>
       <c r="T229" s="47"/>
     </row>
     <row r="230" spans="1:20" ht="17">
       <c r="A230" s="55" t="s">
-        <v>1229</v>
+        <v>1226</v>
       </c>
       <c r="B230" s="52" t="s">
-        <v>1219</v>
+        <v>1216</v>
       </c>
       <c r="C230" s="52" t="s">
         <v>95</v>
@@ -36125,24 +36184,24 @@
         <v>1564</v>
       </c>
       <c r="L230" s="52" t="s">
-        <v>1269</v>
+        <v>1263</v>
       </c>
       <c r="M230" s="52"/>
       <c r="N230" s="47" t="s">
         <v>589</v>
       </c>
       <c r="P230" s="86" t="s">
-        <v>1268</v>
+        <v>1262</v>
       </c>
       <c r="S230" s="47"/>
       <c r="T230" s="47"/>
     </row>
     <row r="231" spans="1:20" ht="17">
       <c r="A231" s="52" t="s">
-        <v>1230</v>
+        <v>1227</v>
       </c>
       <c r="B231" s="55" t="s">
-        <v>1218</v>
+        <v>1215</v>
       </c>
       <c r="C231" s="55" t="s">
         <v>95</v>
@@ -36181,17 +36240,17 @@
         <v>678</v>
       </c>
       <c r="P231" s="86" t="s">
-        <v>1245</v>
+        <v>1242</v>
       </c>
       <c r="S231" s="47"/>
       <c r="T231" s="47"/>
     </row>
     <row r="232" spans="1:20" ht="17">
       <c r="A232" s="52" t="s">
-        <v>1231</v>
+        <v>1228</v>
       </c>
       <c r="B232" s="52" t="s">
-        <v>1220</v>
+        <v>1217</v>
       </c>
       <c r="C232" s="52" t="s">
         <v>95</v>
@@ -36230,17 +36289,17 @@
         <v>678</v>
       </c>
       <c r="P232" s="86" t="s">
-        <v>1191</v>
+        <v>1189</v>
       </c>
       <c r="S232" s="47"/>
       <c r="T232" s="47"/>
     </row>
     <row r="233" spans="1:20" ht="17">
       <c r="A233" s="55" t="s">
-        <v>1232</v>
+        <v>1229</v>
       </c>
       <c r="B233" s="55" t="s">
-        <v>1221</v>
+        <v>1218</v>
       </c>
       <c r="C233" s="55" t="s">
         <v>95</v>
@@ -36274,24 +36333,24 @@
         <v>0</v>
       </c>
       <c r="L233" s="55" t="s">
-        <v>1252</v>
+        <v>1249</v>
       </c>
       <c r="M233" s="55"/>
       <c r="N233" s="47" t="s">
         <v>504</v>
       </c>
       <c r="P233" s="86" t="s">
-        <v>1246</v>
+        <v>1243</v>
       </c>
       <c r="S233" s="47"/>
       <c r="T233" s="47"/>
     </row>
     <row r="234" spans="1:20" ht="17">
       <c r="A234" s="52" t="s">
-        <v>1233</v>
+        <v>1230</v>
       </c>
       <c r="B234" s="52" t="s">
-        <v>1222</v>
+        <v>1219</v>
       </c>
       <c r="C234" s="52" t="s">
         <v>95</v>
@@ -36309,8 +36368,7 @@
         <v>5</v>
       </c>
       <c r="H234" s="65">
-        <f t="shared" si="15"/>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I234" s="65">
         <f>IF(D234&lt;&gt;"",D234,IFERROR(E234/(IFERROR(SUM(Sales!C:C),0))*(IFERROR(SUM(Purchases!C:C),0)),0))</f>
@@ -36330,17 +36388,17 @@
         <v>678</v>
       </c>
       <c r="P234" s="86" t="s">
-        <v>1247</v>
+        <v>1244</v>
       </c>
       <c r="S234" s="47"/>
       <c r="T234" s="47"/>
     </row>
     <row r="235" spans="1:20" ht="17">
       <c r="A235" s="55" t="s">
-        <v>1234</v>
+        <v>1231</v>
       </c>
       <c r="B235" s="55" t="s">
-        <v>1223</v>
+        <v>1220</v>
       </c>
       <c r="C235" s="55" t="s">
         <v>95</v>
@@ -36379,14 +36437,14 @@
         <v>678</v>
       </c>
       <c r="P235" s="86" t="s">
-        <v>1248</v>
+        <v>1245</v>
       </c>
       <c r="S235" s="47"/>
       <c r="T235" s="47"/>
     </row>
     <row r="236" spans="1:20" ht="17">
       <c r="A236" s="52" t="s">
-        <v>1235</v>
+        <v>1232</v>
       </c>
       <c r="B236" s="52" t="s">
         <v>510</v>
@@ -36428,17 +36486,17 @@
         <v>678</v>
       </c>
       <c r="P236" s="86" t="s">
-        <v>1249</v>
+        <v>1246</v>
       </c>
       <c r="S236" s="47"/>
       <c r="T236" s="47"/>
     </row>
     <row r="237" spans="1:20" ht="17">
       <c r="A237" s="52" t="s">
-        <v>1236</v>
+        <v>1233</v>
       </c>
       <c r="B237" s="55" t="s">
-        <v>1224</v>
+        <v>1221</v>
       </c>
       <c r="C237" s="55" t="s">
         <v>95</v>
@@ -36477,17 +36535,17 @@
         <v>678</v>
       </c>
       <c r="P237" s="86" t="s">
-        <v>1250</v>
+        <v>1247</v>
       </c>
       <c r="S237" s="47"/>
       <c r="T237" s="47"/>
     </row>
     <row r="238" spans="1:20" ht="17">
       <c r="A238" s="55" t="s">
-        <v>1237</v>
+        <v>1234</v>
       </c>
       <c r="B238" s="52" t="s">
-        <v>1225</v>
+        <v>1222</v>
       </c>
       <c r="C238" s="52" t="s">
         <v>95</v>
@@ -36526,7 +36584,7 @@
         <v>678</v>
       </c>
       <c r="P238" s="86" t="s">
-        <v>1251</v>
+        <v>1248</v>
       </c>
       <c r="S238" s="47"/>
       <c r="T238" s="47"/>
@@ -40448,15 +40506,15 @@
       </c>
       <c r="B8" s="9">
         <f>IFERROR(SUMIF(Purchases!$B:$B,$A8,Purchases!$C:$C),0)</f>
-        <v>252430</v>
+        <v>261817</v>
       </c>
       <c r="C8" s="9">
         <f>SUM($B$8:$B$10)/3</f>
-        <v>185449</v>
+        <v>188578</v>
       </c>
       <c r="D8" s="9">
         <f>B8-C8</f>
-        <v>66981</v>
+        <v>73239</v>
       </c>
       <c r="E8" s="9">
         <f>IF(Summary!$B$6&gt;0, Summary!$B$6*VLOOKUP($A8,$A$3:$B$5,2,FALSE()),0)</f>
@@ -40464,7 +40522,7 @@
       </c>
       <c r="F8" s="9">
         <f>D8+E8</f>
-        <v>66981</v>
+        <v>73239</v>
       </c>
       <c r="G8" s="9">
         <f>IFERROR(SUMIFS($E$13:$E$499,$D$13:$D$499,$A8,$B$13:$B$499,"Contribution"),0)+IFERROR(SUMIFS($E$13:$E$499,$D$13:$D$499,$A8,$B$13:$B$499,"Profit"),0)-IFERROR(SUMIFS($E$13:$E$499,$C$13:$C$499,$A8,$B$13:$B$499,"Contribution"),0)-IFERROR(SUMIFS($E$13:$E$499,$C$13:$C$499,$A8,$B$13:$B$499,"Profit"),0)</f>
@@ -40472,7 +40530,7 @@
       </c>
       <c r="H8" s="73">
         <f>F8-G8</f>
-        <v>48677.66</v>
+        <v>54935.66</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="13.5" customHeight="1">
@@ -40485,11 +40543,11 @@
       </c>
       <c r="C9" s="11">
         <f>SUM($B$8:$B$10)/3</f>
-        <v>185449</v>
+        <v>188578</v>
       </c>
       <c r="D9" s="11">
         <f>B9-C9</f>
-        <v>85868</v>
+        <v>82739</v>
       </c>
       <c r="E9" s="11">
         <f>IF(Summary!$B$6&gt;0, Summary!$B$6*VLOOKUP($A9,$A$3:$B$5,2,FALSE()),0)</f>
@@ -40497,7 +40555,7 @@
       </c>
       <c r="F9" s="11">
         <f>D9+E9</f>
-        <v>85868</v>
+        <v>82739</v>
       </c>
       <c r="G9" s="11">
         <f>IFERROR(SUMIFS($E$13:$E$499,$D$13:$D$499,$A9,$B$13:$B$499,"Contribution"),0)+IFERROR(SUMIFS($E$13:$E$499,$D$13:$D$499,$A9,$B$13:$B$499,"Profit"),0)-IFERROR(SUMIFS($E$13:$E$499,$C$13:$C$499,$A9,$B$13:$B$499,"Contribution"),0)-IFERROR(SUMIFS($E$13:$E$499,$C$13:$C$499,$A9,$B$13:$B$499,"Profit"),0)</f>
@@ -40505,7 +40563,7 @@
       </c>
       <c r="H9" s="74">
         <f>F9-G9</f>
-        <v>44228.67</v>
+        <v>41099.67</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="13.5" customHeight="1">
@@ -40518,11 +40576,11 @@
       </c>
       <c r="C10" s="9">
         <f>SUM($B$8:$B$10)/3</f>
-        <v>185449</v>
+        <v>188578</v>
       </c>
       <c r="D10" s="9">
         <f>B10-C10</f>
-        <v>-152849</v>
+        <v>-155978</v>
       </c>
       <c r="E10" s="9">
         <f>IF(Summary!$B$6&gt;0, Summary!$B$6*VLOOKUP($A10,$A$3:$B$5,2,FALSE()),0)</f>
@@ -40530,7 +40588,7 @@
       </c>
       <c r="F10" s="9">
         <f>D10+E10</f>
-        <v>-152849</v>
+        <v>-155978</v>
       </c>
       <c r="G10" s="9">
         <f>IFERROR(SUMIFS($E$13:$E$499,$D$13:$D$499,$A10,$B$13:$B$499,"Contribution"),0)+IFERROR(SUMIFS($E$13:$E$499,$D$13:$D$499,$A10,$B$13:$B$499,"Profit"),0)-IFERROR(SUMIFS($E$13:$E$499,$C$13:$C$499,$A10,$B$13:$B$499,"Contribution"),0)-IFERROR(SUMIFS($E$13:$E$499,$C$13:$C$499,$A10,$B$13:$B$499,"Profit"),0)</f>
@@ -40538,7 +40596,7 @@
       </c>
       <c r="H10" s="73">
         <f>F10-G10</f>
-        <v>-92906.33</v>
+        <v>-96035.33</v>
       </c>
     </row>
     <row r="12" spans="1:8" s="75" customFormat="1" ht="15.75" customHeight="1">
@@ -40955,7 +41013,7 @@
       </c>
       <c r="B4" s="9">
         <f>IFERROR(SUMIFS(Sales!$C:$C,Sales!$E:$E,$A4,Sales!$I:$I,"Completed"),0)</f>
-        <v>416139</v>
+        <v>432799</v>
       </c>
       <c r="C4" s="9">
         <f>VLOOKUP($A4,PartnerShares!$A$3:$B$5,2,FALSE())</f>
@@ -40963,11 +41021,11 @@
       </c>
       <c r="D4" s="9">
         <f>Summary!$B$4*C4</f>
-        <v>162006.72819999998</v>
+        <v>166684.3302</v>
       </c>
       <c r="E4" s="9">
         <f>B4-D4</f>
-        <v>254132.27180000002</v>
+        <v>266114.66980000003</v>
       </c>
       <c r="F4" s="9">
         <f>IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$D$13:$D$499,$A4,PartnerShares!$B$13:$B$499,"Cash"),0)-IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$C$13:$C$499,$A4,PartnerShares!$B$13:$B$499,"Cash"),0)</f>
@@ -40975,7 +41033,7 @@
       </c>
       <c r="G4" s="73">
         <f>E4+F4</f>
-        <v>116822.2458</v>
+        <v>128804.64380000002</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="13.5" customHeight="1">
@@ -40992,11 +41050,11 @@
       </c>
       <c r="D5" s="11">
         <f>Summary!$B$4*C5</f>
-        <v>161909.5436</v>
+        <v>166584.33960000001</v>
       </c>
       <c r="E5" s="11">
         <f>B5-D5</f>
-        <v>-107285.5436</v>
+        <v>-111960.33960000001</v>
       </c>
       <c r="F5" s="11">
         <f>IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$D$13:$D$499,$A5,PartnerShares!$B$13:$B$499,"Cash"),0)-IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$C$13:$C$499,$A5,PartnerShares!$B$13:$B$499,"Cash"),0)</f>
@@ -41004,7 +41062,7 @@
       </c>
       <c r="G5" s="74">
         <f>E5+F5</f>
-        <v>-35698.501600000003</v>
+        <v>-40373.297600000005</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="13.5" customHeight="1">
@@ -41021,11 +41079,11 @@
       </c>
       <c r="D6" s="9">
         <f>Summary!$B$4*C6</f>
-        <v>162006.72819999998</v>
+        <v>166684.3302</v>
       </c>
       <c r="E6" s="9">
         <f>B6-D6</f>
-        <v>-149476.72819999998</v>
+        <v>-154154.3302</v>
       </c>
       <c r="F6" s="9">
         <f>IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$D$13:$D$499,$A6,PartnerShares!$B$13:$B$499,"Cash"),0)-IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$C$13:$C$499,$A6,PartnerShares!$B$13:$B$499,"Cash"),0)</f>
@@ -41033,7 +41091,7 @@
       </c>
       <c r="G6" s="73">
         <f>E6+F6</f>
-        <v>-83753.744199999972</v>
+        <v>-88431.346199999985</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="13.5" customHeight="1">

</xml_diff>

<commit_message>
8/23 & 8/24 sales
</commit_message>
<xml_diff>
--- a/docs/Chiraath-Summary-Aug26.xlsx
+++ b/docs/Chiraath-Summary-Aug26.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/anooppremachandran/Desktop/CHIRAATH/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F5DA603-7CD1-944E-ACA5-37C93750C159}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63805685-D5E2-F64D-8AAE-58F5C469B1FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" tabRatio="500" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Notes" sheetId="1" r:id="rId1"/>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3356" uniqueCount="1331">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3381" uniqueCount="1339">
   <si>
     <t>Notes:</t>
   </si>
@@ -3094,12 +3094,6 @@
     <t>Matka Saree Collections</t>
   </si>
   <si>
-    <t>Navya - Black Orange</t>
-  </si>
-  <si>
-    <t>Black/pink, black/orange, violet/bottle green</t>
-  </si>
-  <si>
     <t>CHR-205</t>
   </si>
   <si>
@@ -3326,12 +3320,6 @@
   </si>
   <si>
     <t>CHR-165 (Chocolate Brown)</t>
-  </si>
-  <si>
-    <t>Chocolate Brown - Albert</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Violet, Bottle Green  </t>
   </si>
   <si>
     <t>Irene Anna Reji</t>
@@ -3601,9 +3589,6 @@
     <t>Cream/gold with leaves, cream/gold with flowers</t>
   </si>
   <si>
-    <t>Shylaja - Green and maroon with golden design</t>
-  </si>
-  <si>
     <t>Green and maroon, deep purple and dark green, blue and dark green, rose pink and olive green, Red</t>
   </si>
   <si>
@@ -3715,9 +3700,6 @@
     <t>Brown</t>
   </si>
   <si>
-    <t>Black, Wine</t>
-  </si>
-  <si>
     <t>Jet Black</t>
   </si>
   <si>
@@ -3898,9 +3880,6 @@
     <t>Sruthi (1300) - L, Bank of baroda customer - M, Niroop - XL</t>
   </si>
   <si>
-    <t>CHR-212 - Purple, CHR-215 - Green and Maroon with golden design - 1000 advance, 750 pending</t>
-  </si>
-  <si>
     <t>CHR-153 (XXL)-Cotton whine 3 piece salwar, CHR-155 (XXL) -Cotton black 3 piece salwar, CHR-51(XXL)-Mul cotton floral salwar  - 1000 advance, 1500 pending</t>
   </si>
   <si>
@@ -3914,12 +3893,6 @@
   </si>
   <si>
     <t>CHR-235-Silk Saree - Yellow/Black</t>
-  </si>
-  <si>
-    <t>Dr.Reshna - Yellow/Black</t>
-  </si>
-  <si>
-    <t>Pink with Silver Butas, Black/Red, Wine/Green</t>
   </si>
   <si>
     <t>Nisha Shaju</t>
@@ -4025,12 +3998,6 @@
     <t>CHR-182 (Yellow Linen Saree with Lotus, CHR-217 cream/gold with stars and paisley &amp; cream/gold with flowers, CHR-212 Green elephant print - 1600 advance, 1150 - pending</t>
   </si>
   <si>
-    <t>Latha - Red, Shylaja - Purple, Jisha - Red, Bank staff - Green</t>
-  </si>
-  <si>
-    <t>Yellow/Orange(4), Blue</t>
-  </si>
-  <si>
     <t>Green/maroon - Rajitha Teacher,  chikku green - Razia Salim, Rust Orange/Coffee Brown - Nishida, Chikku Maroon(1200) - Nishida, Komalavalli - Red/green, peacock blue/navy - returned, mustard/blue - girija(1200), Suma - Golden yellow &amp; green triangle</t>
   </si>
   <si>
@@ -4056,6 +4023,63 @@
   </si>
   <si>
     <t>CHR-186 - Banarasi Silk (Golden Yellow Green)</t>
+  </si>
+  <si>
+    <t>Courier charges</t>
+  </si>
+  <si>
+    <t>Chocolate Brown - Albert, Green - Said</t>
+  </si>
+  <si>
+    <t>Violet</t>
+  </si>
+  <si>
+    <t>CHR-165 - Checked Green, CHR-204 - Black/Pink</t>
+  </si>
+  <si>
+    <t>Navya - Black Orange, Saida - Black Pink</t>
+  </si>
+  <si>
+    <t>Violet/bottle green</t>
+  </si>
+  <si>
+    <t>CHR-212 Yellow/Orange</t>
+  </si>
+  <si>
+    <t>Latha - Red, Shylaja - Purple, Jisha - Red, Bank staff - Green, Rajna - Yellow/Orange</t>
+  </si>
+  <si>
+    <t>Yellow/Orange(2), Blue</t>
+  </si>
+  <si>
+    <t>CHR-212 - Purple, CHR-235 - Black Red - 1000 advance, 750 pending</t>
+  </si>
+  <si>
+    <t>Dr.Reshna - Yellow/Black, Shylaja - Black/Red</t>
+  </si>
+  <si>
+    <t>Pink with Silver Butas,  Wine/Green</t>
+  </si>
+  <si>
+    <t>Tennish</t>
+  </si>
+  <si>
+    <t>CHR-225 Black Tusshar</t>
+  </si>
+  <si>
+    <t>Tennish - Black Tussar</t>
+  </si>
+  <si>
+    <t>Wine</t>
+  </si>
+  <si>
+    <t>Hima BS</t>
+  </si>
+  <si>
+    <t>120 count mul cotton</t>
+  </si>
+  <si>
+    <t>Hima B S</t>
   </si>
 </sst>
 </file>
@@ -4941,7 +4965,7 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>350</c:v>
+                  <c:v>355</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>99</c:v>
@@ -5044,7 +5068,7 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>179</c:v>
+                  <c:v>173</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>51</c:v>
@@ -5377,7 +5401,7 @@
                   <c:v>53945</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>127271.14666666667</c:v>
+                  <c:v>122683.14666666667</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>1062</c:v>
@@ -5870,10 +5894,10 @@
                   <c:v>72885</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>63426</c:v>
+                  <c:v>63906</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>65478</c:v>
+                  <c:v>72908</c:v>
                 </c:pt>
                 <c:pt idx="8">
                   <c:v>0</c:v>
@@ -6310,10 +6334,10 @@
                   <c:v>-26158</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>-38774</c:v>
+                  <c:v>-38294</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>55017</c:v>
+                  <c:v>62447</c:v>
                 </c:pt>
                 <c:pt idx="8">
                   <c:v>0</c:v>
@@ -6774,10 +6798,10 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="2"/>
                 <c:pt idx="0">
-                  <c:v>454</c:v>
+                  <c:v>459</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>275</c:v>
+                  <c:v>269</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -7964,7 +7988,7 @@
       </c>
       <c r="B4" s="10">
         <f>SUMIFS(Sales!C:C, Sales!I:I, "Completed")</f>
-        <v>537362</v>
+        <v>541092</v>
       </c>
       <c r="E4" s="9" t="str">
         <f>PartnerShares!A3</f>
@@ -7981,7 +8005,7 @@
       </c>
       <c r="B5" s="12">
         <f>SUM(Sales!C:C)</f>
-        <v>557402</v>
+        <v>565312</v>
       </c>
       <c r="E5" s="11" t="str">
         <f>PartnerShares!A4</f>
@@ -7998,7 +8022,7 @@
       </c>
       <c r="B6" s="10">
         <f>B4-B3</f>
-        <v>-29446</v>
+        <v>-25716</v>
       </c>
       <c r="E6" s="9" t="str">
         <f>PartnerShares!A5</f>
@@ -8210,15 +8234,15 @@
       </c>
       <c r="B26" s="10">
         <f>'Cash Pool'!B4</f>
-        <v>469208</v>
+        <v>472938</v>
       </c>
       <c r="C26" s="10">
         <f>'Cash Pool'!D4</f>
-        <v>179156.4908</v>
+        <v>180400.07279999999</v>
       </c>
       <c r="D26" s="10">
         <f>'Cash Pool'!E4</f>
-        <v>290051.50919999997</v>
+        <v>292537.92720000003</v>
       </c>
       <c r="E26" s="10">
         <f>'Cash Pool'!F4</f>
@@ -8226,11 +8250,11 @@
       </c>
       <c r="F26" s="13">
         <f>'Cash Pool'!G4</f>
-        <v>152741.48319999996</v>
+        <v>155227.90120000002</v>
       </c>
       <c r="G26" s="17" t="str">
         <f>IF(ROUND(F26,0)&gt;0,"Pay ₹"&amp;TEXT(ABS(F26),"#,##0"),IF(ROUND(F26,0)&lt;0,"Receive ₹"&amp;TEXT(ABS(F26),"#,##0"),"✓ Settled"))</f>
-        <v>Pay ₹152,741</v>
+        <v>Pay ₹155,228</v>
       </c>
     </row>
     <row r="27" spans="1:7" ht="13.5" customHeight="1">
@@ -8244,11 +8268,11 @@
       </c>
       <c r="C27" s="12">
         <f>'Cash Pool'!D5</f>
-        <v>179049.0184</v>
+        <v>180291.85440000001</v>
       </c>
       <c r="D27" s="12">
         <f>'Cash Pool'!E5</f>
-        <v>-124425.0184</v>
+        <v>-125667.85440000001</v>
       </c>
       <c r="E27" s="12">
         <f>'Cash Pool'!F5</f>
@@ -8256,11 +8280,11 @@
       </c>
       <c r="F27" s="14">
         <f>'Cash Pool'!G5</f>
-        <v>-52837.9764</v>
+        <v>-54080.81240000001</v>
       </c>
       <c r="G27" s="18" t="str">
         <f>IF(ROUND(F27,0)&gt;0,"Pay ₹"&amp;TEXT(ABS(F27),"#,##0"),IF(ROUND(F27,0)&lt;0,"Receive ₹"&amp;TEXT(ABS(F27),"#,##0"),"✓ Settled"))</f>
-        <v>Receive ₹52,838</v>
+        <v>Receive ₹54,081</v>
       </c>
     </row>
     <row r="28" spans="1:7" ht="13.5" customHeight="1">
@@ -8274,11 +8298,11 @@
       </c>
       <c r="C28" s="10">
         <f>'Cash Pool'!D6</f>
-        <v>179156.4908</v>
+        <v>180400.07279999999</v>
       </c>
       <c r="D28" s="10">
         <f>'Cash Pool'!E6</f>
-        <v>-166626.4908</v>
+        <v>-167870.07279999999</v>
       </c>
       <c r="E28" s="10">
         <f>'Cash Pool'!F6</f>
@@ -8286,11 +8310,11 @@
       </c>
       <c r="F28" s="13">
         <f>'Cash Pool'!G6</f>
-        <v>-100903.50679999999</v>
+        <v>-102147.08879999998</v>
       </c>
       <c r="G28" s="16" t="str">
         <f>IF(ROUND(F28,0)&gt;0,"Pay ₹"&amp;TEXT(ABS(F28),"#,##0"),IF(ROUND(F28,0)&lt;0,"Receive ₹"&amp;TEXT(ABS(F28),"#,##0"),"✓ Settled"))</f>
-        <v>Receive ₹100,904</v>
+        <v>Receive ₹102,147</v>
       </c>
     </row>
     <row r="32" spans="1:7" ht="15.75" customHeight="1">
@@ -8402,7 +8426,7 @@
       </c>
       <c r="B3" s="20">
         <f ca="1">TODAY()</f>
-        <v>46253</v>
+        <v>46261</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="15" customHeight="1">
@@ -8418,7 +8442,7 @@
       </c>
       <c r="E5" s="21">
         <f>Summary!B4</f>
-        <v>537362</v>
+        <v>541092</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="15" customHeight="1">
@@ -8427,14 +8451,14 @@
       </c>
       <c r="B6" s="21">
         <f>Summary!B6</f>
-        <v>-29446</v>
+        <v>-25716</v>
       </c>
       <c r="D6" s="19" t="s">
         <v>71</v>
       </c>
       <c r="E6" s="21">
         <f>SUMIFS(INVENTORY!K:K, INVENTORY!N:N, "&lt;&gt;Sold Out")</f>
-        <v>171407.34666666665</v>
+        <v>168031.34666666665</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="15.75" customHeight="1">
@@ -8486,7 +8510,7 @@
       </c>
       <c r="G10" s="21">
         <f>SUM(INVENTORY!F:F)</f>
-        <v>454</v>
+        <v>459</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="15" customHeight="1">
@@ -8510,7 +8534,7 @@
       </c>
       <c r="G11" s="27">
         <f>SUM(INVENTORY!G:G)</f>
-        <v>275</v>
+        <v>269</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="15" customHeight="1">
@@ -8591,11 +8615,11 @@
       </c>
       <c r="C16" s="21">
         <f>IFERROR(SUMPRODUCT((TEXT(Sales!$A$2:$A$993,"MMM")=$A16)*(YEAR(Sales!$A$2:$A$993)=$B$7)*Sales!$C$2:$C$993),0)</f>
-        <v>63426</v>
+        <v>63906</v>
       </c>
       <c r="D16" s="21">
         <f t="shared" si="0"/>
-        <v>-38774</v>
+        <v>-38294</v>
       </c>
     </row>
     <row r="17" spans="1:4" ht="15" customHeight="1">
@@ -8608,11 +8632,11 @@
       </c>
       <c r="C17" s="27">
         <f>IFERROR(SUMPRODUCT((TEXT(Sales!$A$2:$A$993,"MMM")=$A17)*(YEAR(Sales!$A$2:$A$993)=$B$7)*Sales!$C$2:$C$993),0)</f>
-        <v>65478</v>
+        <v>72908</v>
       </c>
       <c r="D17" s="27">
         <f t="shared" si="0"/>
-        <v>55017</v>
+        <v>62447</v>
       </c>
     </row>
     <row r="18" spans="1:4" ht="15" customHeight="1">
@@ -8706,11 +8730,11 @@
       </c>
       <c r="G47" s="30">
         <f>SUMIF(INVENTORY!C:C, F47, INVENTORY!F:F)</f>
-        <v>350</v>
+        <v>355</v>
       </c>
       <c r="H47" s="30">
         <f>SUMIF(INVENTORY!C:C, F47, INVENTORY!G:G)</f>
-        <v>179</v>
+        <v>173</v>
       </c>
       <c r="J47" s="30" t="s">
         <v>96</v>
@@ -8737,7 +8761,7 @@
       </c>
       <c r="K48" s="31">
         <f t="array" ref="K48">SUMPRODUCT((INVENTORY!$C$2:$C$476=J48)*(INVENTORY!$D$2:$D$476)*(INVENTORY!$G$2:$G$476))</f>
-        <v>127271.14666666667</v>
+        <v>122683.14666666667</v>
       </c>
     </row>
     <row r="49" spans="5:12" ht="15" customHeight="1">
@@ -10110,7 +10134,7 @@
         <v>28526</v>
       </c>
       <c r="D91" s="39" t="s">
-        <v>1098</v>
+        <v>1094</v>
       </c>
     </row>
     <row r="92" spans="1:4" ht="15" customHeight="1">
@@ -10180,7 +10204,7 @@
         <v>70</v>
       </c>
       <c r="D96" s="36" t="s">
-        <v>1128</v>
+        <v>1124</v>
       </c>
     </row>
     <row r="97" spans="1:4" ht="15" customHeight="1">
@@ -10194,7 +10218,7 @@
         <v>1375</v>
       </c>
       <c r="D97" s="39" t="s">
-        <v>1129</v>
+        <v>1125</v>
       </c>
     </row>
     <row r="98" spans="1:4" ht="15" customHeight="1">
@@ -10208,7 +10232,7 @@
         <v>189</v>
       </c>
       <c r="D98" s="36" t="s">
-        <v>1130</v>
+        <v>1126</v>
       </c>
     </row>
     <row r="99" spans="1:4" ht="15" customHeight="1">
@@ -10334,7 +10358,7 @@
         <v>570</v>
       </c>
       <c r="D107" s="39" t="s">
-        <v>1288</v>
+        <v>1279</v>
       </c>
     </row>
     <row r="108" spans="1:4" ht="15" customHeight="1">
@@ -10362,7 +10386,7 @@
         <v>320</v>
       </c>
       <c r="D109" s="39" t="s">
-        <v>1288</v>
+        <v>1279</v>
       </c>
     </row>
     <row r="110" spans="1:4" ht="15" customHeight="1">
@@ -17735,7 +17759,7 @@
       <c r="F216" s="46"/>
       <c r="G216" s="46"/>
       <c r="H216" s="46" t="s">
-        <v>1085</v>
+        <v>1083</v>
       </c>
       <c r="I216" s="45" t="s">
         <v>148</v>
@@ -18560,7 +18584,7 @@
       <c r="F249" s="46"/>
       <c r="G249" s="46"/>
       <c r="H249" s="46" t="s">
-        <v>1071</v>
+        <v>1069</v>
       </c>
       <c r="I249" s="45" t="s">
         <v>148</v>
@@ -18581,7 +18605,7 @@
       <c r="F250" s="44"/>
       <c r="G250" s="44"/>
       <c r="H250" s="44" t="s">
-        <v>1073</v>
+        <v>1071</v>
       </c>
       <c r="I250" s="44" t="s">
         <v>356</v>
@@ -18592,7 +18616,7 @@
         <v>46201</v>
       </c>
       <c r="B251" s="45" t="s">
-        <v>1086</v>
+        <v>1084</v>
       </c>
       <c r="C251" s="85">
         <v>1380</v>
@@ -18617,7 +18641,7 @@
         <v>46201</v>
       </c>
       <c r="B252" s="44" t="s">
-        <v>1074</v>
+        <v>1072</v>
       </c>
       <c r="C252" s="83">
         <v>699</v>
@@ -18631,7 +18655,7 @@
       <c r="F252" s="44"/>
       <c r="G252" s="44"/>
       <c r="H252" s="44" t="s">
-        <v>1075</v>
+        <v>1073</v>
       </c>
       <c r="I252" s="44" t="s">
         <v>148</v>
@@ -18642,7 +18666,7 @@
         <v>46201</v>
       </c>
       <c r="B253" s="45" t="s">
-        <v>1076</v>
+        <v>1074</v>
       </c>
       <c r="C253" s="85">
         <v>699</v>
@@ -18656,7 +18680,7 @@
       <c r="F253" s="46"/>
       <c r="G253" s="46"/>
       <c r="H253" s="46" t="s">
-        <v>1077</v>
+        <v>1075</v>
       </c>
       <c r="I253" s="45" t="s">
         <v>148</v>
@@ -18667,7 +18691,7 @@
         <v>46201</v>
       </c>
       <c r="B254" s="44" t="s">
-        <v>1078</v>
+        <v>1076</v>
       </c>
       <c r="C254" s="83">
         <v>699</v>
@@ -18681,7 +18705,7 @@
       <c r="F254" s="44"/>
       <c r="G254" s="44"/>
       <c r="H254" s="44" t="s">
-        <v>1079</v>
+        <v>1077</v>
       </c>
       <c r="I254" s="44" t="s">
         <v>148</v>
@@ -18706,7 +18730,7 @@
       <c r="F255" s="46"/>
       <c r="G255" s="46"/>
       <c r="H255" s="46" t="s">
-        <v>1080</v>
+        <v>1078</v>
       </c>
       <c r="I255" s="45" t="s">
         <v>148</v>
@@ -18717,7 +18741,7 @@
         <v>46203</v>
       </c>
       <c r="B256" s="44" t="s">
-        <v>1087</v>
+        <v>1085</v>
       </c>
       <c r="C256" s="83">
         <v>950</v>
@@ -18731,7 +18755,7 @@
       <c r="F256" s="44"/>
       <c r="G256" s="44"/>
       <c r="H256" s="44" t="s">
-        <v>1088</v>
+        <v>1086</v>
       </c>
       <c r="I256" s="44" t="s">
         <v>148</v>
@@ -18742,7 +18766,7 @@
         <v>46204</v>
       </c>
       <c r="B257" s="45" t="s">
-        <v>1091</v>
+        <v>1087</v>
       </c>
       <c r="C257" s="85">
         <v>699</v>
@@ -18756,7 +18780,7 @@
       <c r="F257" s="46"/>
       <c r="G257" s="46"/>
       <c r="H257" s="46" t="s">
-        <v>1092</v>
+        <v>1088</v>
       </c>
       <c r="I257" s="45" t="s">
         <v>148</v>
@@ -18767,7 +18791,7 @@
         <v>46205</v>
       </c>
       <c r="B258" s="44" t="s">
-        <v>1093</v>
+        <v>1089</v>
       </c>
       <c r="C258" s="83">
         <v>1500</v>
@@ -18781,7 +18805,7 @@
       <c r="F258" s="44"/>
       <c r="G258" s="44"/>
       <c r="H258" s="44" t="s">
-        <v>1094</v>
+        <v>1090</v>
       </c>
       <c r="I258" s="44" t="s">
         <v>148</v>
@@ -18792,7 +18816,7 @@
         <v>46205</v>
       </c>
       <c r="B259" s="45" t="s">
-        <v>1093</v>
+        <v>1089</v>
       </c>
       <c r="C259" s="85">
         <v>1200</v>
@@ -18806,7 +18830,7 @@
       <c r="F259" s="46"/>
       <c r="G259" s="46"/>
       <c r="H259" s="46" t="s">
-        <v>1095</v>
+        <v>1091</v>
       </c>
       <c r="I259" s="45" t="s">
         <v>148</v>
@@ -18817,7 +18841,7 @@
         <v>46205</v>
       </c>
       <c r="B260" s="44" t="s">
-        <v>1097</v>
+        <v>1093</v>
       </c>
       <c r="C260" s="83">
         <v>1500</v>
@@ -18831,7 +18855,7 @@
       <c r="F260" s="44"/>
       <c r="G260" s="44"/>
       <c r="H260" s="44" t="s">
-        <v>1096</v>
+        <v>1092</v>
       </c>
       <c r="I260" s="44" t="s">
         <v>148</v>
@@ -18842,7 +18866,7 @@
         <v>46205</v>
       </c>
       <c r="B261" s="45" t="s">
-        <v>1100</v>
+        <v>1096</v>
       </c>
       <c r="C261" s="85">
         <v>2600</v>
@@ -18856,7 +18880,7 @@
       <c r="F261" s="46"/>
       <c r="G261" s="46"/>
       <c r="H261" s="46" t="s">
-        <v>1181</v>
+        <v>1176</v>
       </c>
       <c r="I261" s="45" t="s">
         <v>148</v>
@@ -18867,7 +18891,7 @@
         <v>46206</v>
       </c>
       <c r="B262" s="44" t="s">
-        <v>1102</v>
+        <v>1098</v>
       </c>
       <c r="C262" s="83">
         <v>1380</v>
@@ -18892,7 +18916,7 @@
         <v>46206</v>
       </c>
       <c r="B263" s="45" t="s">
-        <v>1103</v>
+        <v>1099</v>
       </c>
       <c r="C263" s="85">
         <v>1380</v>
@@ -18917,7 +18941,7 @@
         <v>46206</v>
       </c>
       <c r="B264" s="44" t="s">
-        <v>1113</v>
+        <v>1109</v>
       </c>
       <c r="C264" s="83">
         <v>2500</v>
@@ -18931,7 +18955,7 @@
       <c r="F264" s="44"/>
       <c r="G264" s="44"/>
       <c r="H264" s="44" t="s">
-        <v>1279</v>
+        <v>1272</v>
       </c>
       <c r="I264" s="44" t="s">
         <v>356</v>
@@ -18942,7 +18966,7 @@
         <v>46206</v>
       </c>
       <c r="B265" s="45" t="s">
-        <v>1106</v>
+        <v>1102</v>
       </c>
       <c r="C265" s="85">
         <v>1300</v>
@@ -18956,7 +18980,7 @@
       <c r="F265" s="46"/>
       <c r="G265" s="46"/>
       <c r="H265" s="46" t="s">
-        <v>1118</v>
+        <v>1114</v>
       </c>
       <c r="I265" s="45" t="s">
         <v>356</v>
@@ -18967,7 +18991,7 @@
         <v>46206</v>
       </c>
       <c r="B266" s="44" t="s">
-        <v>1097</v>
+        <v>1093</v>
       </c>
       <c r="C266" s="83">
         <v>1380</v>
@@ -18981,7 +19005,7 @@
       <c r="F266" s="44"/>
       <c r="G266" s="44"/>
       <c r="H266" s="44" t="s">
-        <v>1107</v>
+        <v>1103</v>
       </c>
       <c r="I266" s="44" t="s">
         <v>148</v>
@@ -19006,7 +19030,7 @@
       <c r="F267" s="46"/>
       <c r="G267" s="46"/>
       <c r="H267" s="46" t="s">
-        <v>1108</v>
+        <v>1104</v>
       </c>
       <c r="I267" s="45" t="s">
         <v>148</v>
@@ -19017,7 +19041,7 @@
         <v>46208</v>
       </c>
       <c r="B268" s="44" t="s">
-        <v>1309</v>
+        <v>1300</v>
       </c>
       <c r="C268" s="83">
         <v>2350</v>
@@ -19027,7 +19051,7 @@
       <c r="F268" s="44"/>
       <c r="G268" s="44"/>
       <c r="H268" s="44" t="s">
-        <v>1310</v>
+        <v>1301</v>
       </c>
       <c r="I268" s="44" t="s">
         <v>356</v>
@@ -19038,7 +19062,7 @@
         <v>46209</v>
       </c>
       <c r="B269" s="45" t="s">
-        <v>1111</v>
+        <v>1107</v>
       </c>
       <c r="C269" s="85">
         <v>1100</v>
@@ -19052,7 +19076,7 @@
       <c r="F269" s="46"/>
       <c r="G269" s="46"/>
       <c r="H269" s="46" t="s">
-        <v>1112</v>
+        <v>1108</v>
       </c>
       <c r="I269" s="45" t="s">
         <v>148</v>
@@ -19063,7 +19087,7 @@
         <v>46210</v>
       </c>
       <c r="B270" s="44" t="s">
-        <v>1312</v>
+        <v>1303</v>
       </c>
       <c r="C270" s="83">
         <v>3200</v>
@@ -19077,7 +19101,7 @@
       <c r="F270" s="44"/>
       <c r="G270" s="44"/>
       <c r="H270" s="44" t="s">
-        <v>1115</v>
+        <v>1111</v>
       </c>
       <c r="I270" s="44" t="s">
         <v>148</v>
@@ -19088,7 +19112,7 @@
         <v>46211</v>
       </c>
       <c r="B271" s="45" t="s">
-        <v>1116</v>
+        <v>1112</v>
       </c>
       <c r="C271" s="85">
         <v>1380</v>
@@ -19102,7 +19126,7 @@
       <c r="F271" s="46"/>
       <c r="G271" s="46"/>
       <c r="H271" s="46" t="s">
-        <v>1117</v>
+        <v>1113</v>
       </c>
       <c r="I271" s="45" t="s">
         <v>148</v>
@@ -19113,7 +19137,7 @@
         <v>46215</v>
       </c>
       <c r="B272" s="44" t="s">
-        <v>1119</v>
+        <v>1115</v>
       </c>
       <c r="C272" s="83">
         <v>1380</v>
@@ -19138,7 +19162,7 @@
         <v>46215</v>
       </c>
       <c r="B273" s="45" t="s">
-        <v>1120</v>
+        <v>1116</v>
       </c>
       <c r="C273" s="85">
         <v>699</v>
@@ -19152,7 +19176,7 @@
       <c r="F273" s="46"/>
       <c r="G273" s="46"/>
       <c r="H273" s="46" t="s">
-        <v>1092</v>
+        <v>1088</v>
       </c>
       <c r="I273" s="45" t="s">
         <v>148</v>
@@ -19177,7 +19201,7 @@
       <c r="F274" s="44"/>
       <c r="G274" s="44"/>
       <c r="H274" s="44" t="s">
-        <v>1122</v>
+        <v>1118</v>
       </c>
       <c r="I274" s="44" t="s">
         <v>148</v>
@@ -19188,7 +19212,7 @@
         <v>46216</v>
       </c>
       <c r="B275" s="45" t="s">
-        <v>1123</v>
+        <v>1119</v>
       </c>
       <c r="C275" s="85">
         <v>699</v>
@@ -19202,7 +19226,7 @@
       <c r="F275" s="46"/>
       <c r="G275" s="46"/>
       <c r="H275" s="46" t="s">
-        <v>1092</v>
+        <v>1088</v>
       </c>
       <c r="I275" s="45" t="s">
         <v>148</v>
@@ -19213,7 +19237,7 @@
         <v>46216</v>
       </c>
       <c r="B276" s="44" t="s">
-        <v>1125</v>
+        <v>1121</v>
       </c>
       <c r="C276" s="83">
         <v>3000</v>
@@ -19227,7 +19251,7 @@
       <c r="F276" s="44"/>
       <c r="G276" s="44"/>
       <c r="H276" s="44" t="s">
-        <v>1124</v>
+        <v>1120</v>
       </c>
       <c r="I276" s="44" t="s">
         <v>148</v>
@@ -19238,7 +19262,7 @@
         <v>46219</v>
       </c>
       <c r="B277" s="45" t="s">
-        <v>1126</v>
+        <v>1122</v>
       </c>
       <c r="C277" s="85">
         <v>1380</v>
@@ -19302,7 +19326,7 @@
       <c r="F279" s="46"/>
       <c r="G279" s="46"/>
       <c r="H279" s="46" t="s">
-        <v>1127</v>
+        <v>1123</v>
       </c>
       <c r="I279" s="45" t="s">
         <v>148</v>
@@ -19327,7 +19351,7 @@
       <c r="F280" s="44"/>
       <c r="G280" s="44"/>
       <c r="H280" s="44" t="s">
-        <v>1133</v>
+        <v>1129</v>
       </c>
       <c r="I280" s="44" t="s">
         <v>148</v>
@@ -19352,7 +19376,7 @@
       <c r="F281" s="46"/>
       <c r="G281" s="46"/>
       <c r="H281" s="46" t="s">
-        <v>1137</v>
+        <v>1133</v>
       </c>
       <c r="I281" s="45" t="s">
         <v>148</v>
@@ -19363,7 +19387,7 @@
         <v>46220</v>
       </c>
       <c r="B282" s="44" t="s">
-        <v>1147</v>
+        <v>1143</v>
       </c>
       <c r="C282" s="83">
         <v>1500</v>
@@ -19377,7 +19401,7 @@
       <c r="F282" s="44"/>
       <c r="G282" s="44"/>
       <c r="H282" s="44" t="s">
-        <v>1148</v>
+        <v>1144</v>
       </c>
       <c r="I282" s="44" t="s">
         <v>148</v>
@@ -19388,7 +19412,7 @@
         <v>46221</v>
       </c>
       <c r="B283" s="45" t="s">
-        <v>1151</v>
+        <v>1147</v>
       </c>
       <c r="C283" s="85">
         <v>1100</v>
@@ -19402,7 +19426,7 @@
       <c r="F283" s="46"/>
       <c r="G283" s="46"/>
       <c r="H283" s="46" t="s">
-        <v>1152</v>
+        <v>1148</v>
       </c>
       <c r="I283" s="45" t="s">
         <v>148</v>
@@ -19413,7 +19437,7 @@
         <v>46222</v>
       </c>
       <c r="B284" s="44" t="s">
-        <v>1153</v>
+        <v>1149</v>
       </c>
       <c r="C284" s="83">
         <v>850</v>
@@ -19427,7 +19451,7 @@
       <c r="F284" s="44"/>
       <c r="G284" s="44"/>
       <c r="H284" s="44" t="s">
-        <v>1154</v>
+        <v>1150</v>
       </c>
       <c r="I284" s="44" t="s">
         <v>148</v>
@@ -19438,7 +19462,7 @@
         <v>46222</v>
       </c>
       <c r="B285" s="45" t="s">
-        <v>1155</v>
+        <v>1151</v>
       </c>
       <c r="C285" s="85">
         <v>1250</v>
@@ -19452,7 +19476,7 @@
       <c r="F285" s="46"/>
       <c r="G285" s="46"/>
       <c r="H285" s="46" t="s">
-        <v>1156</v>
+        <v>1152</v>
       </c>
       <c r="I285" s="45" t="s">
         <v>148</v>
@@ -19463,7 +19487,7 @@
         <v>46222</v>
       </c>
       <c r="B286" s="44" t="s">
-        <v>1158</v>
+        <v>1154</v>
       </c>
       <c r="C286" s="83">
         <v>700</v>
@@ -19488,7 +19512,7 @@
         <v>46222</v>
       </c>
       <c r="B287" s="45" t="s">
-        <v>1159</v>
+        <v>1155</v>
       </c>
       <c r="C287" s="85">
         <v>699</v>
@@ -19513,7 +19537,7 @@
         <v>46223</v>
       </c>
       <c r="B288" s="44" t="s">
-        <v>1162</v>
+        <v>1158</v>
       </c>
       <c r="C288" s="83">
         <v>1380</v>
@@ -19527,7 +19551,7 @@
       <c r="F288" s="44"/>
       <c r="G288" s="44"/>
       <c r="H288" s="44" t="s">
-        <v>1163</v>
+        <v>1159</v>
       </c>
       <c r="I288" s="44" t="s">
         <v>148</v>
@@ -19538,7 +19562,7 @@
         <v>46224</v>
       </c>
       <c r="B289" s="45" t="s">
-        <v>1165</v>
+        <v>1161</v>
       </c>
       <c r="C289" s="85">
         <v>1380</v>
@@ -19552,7 +19576,7 @@
       <c r="F289" s="46"/>
       <c r="G289" s="46"/>
       <c r="H289" s="46" t="s">
-        <v>1168</v>
+        <v>1164</v>
       </c>
       <c r="I289" s="45" t="s">
         <v>148</v>
@@ -19563,7 +19587,7 @@
         <v>46224</v>
       </c>
       <c r="B290" s="44" t="s">
-        <v>1164</v>
+        <v>1160</v>
       </c>
       <c r="C290" s="83">
         <v>1380</v>
@@ -19577,7 +19601,7 @@
       <c r="F290" s="44"/>
       <c r="G290" s="44"/>
       <c r="H290" s="44" t="s">
-        <v>1169</v>
+        <v>1165</v>
       </c>
       <c r="I290" s="44" t="s">
         <v>148</v>
@@ -19602,7 +19626,7 @@
       <c r="F291" s="44"/>
       <c r="G291" s="44"/>
       <c r="H291" s="44" t="s">
-        <v>1172</v>
+        <v>1168</v>
       </c>
       <c r="I291" s="44" t="s">
         <v>148</v>
@@ -19613,7 +19637,7 @@
         <v>46229</v>
       </c>
       <c r="B292" s="45" t="s">
-        <v>1175</v>
+        <v>1171</v>
       </c>
       <c r="C292" s="85">
         <v>2750</v>
@@ -19623,7 +19647,7 @@
       <c r="F292" s="46"/>
       <c r="G292" s="46"/>
       <c r="H292" s="46" t="s">
-        <v>1319</v>
+        <v>1310</v>
       </c>
       <c r="I292" s="45" t="s">
         <v>356</v>
@@ -19637,14 +19661,14 @@
         <v>293</v>
       </c>
       <c r="C293" s="83">
-        <v>1750</v>
+        <v>2230</v>
       </c>
       <c r="D293" s="44"/>
       <c r="E293" s="44"/>
       <c r="F293" s="44"/>
       <c r="G293" s="44"/>
       <c r="H293" s="44" t="s">
-        <v>1278</v>
+        <v>1329</v>
       </c>
       <c r="I293" s="44" t="s">
         <v>356</v>
@@ -19655,7 +19679,7 @@
         <v>46229</v>
       </c>
       <c r="B294" s="45" t="s">
-        <v>1100</v>
+        <v>1096</v>
       </c>
       <c r="C294" s="85">
         <v>2230</v>
@@ -19669,7 +19693,7 @@
       <c r="F294" s="46"/>
       <c r="G294" s="46"/>
       <c r="H294" s="46" t="s">
-        <v>1318</v>
+        <v>1309</v>
       </c>
       <c r="I294" s="45" t="s">
         <v>148</v>
@@ -19680,13 +19704,13 @@
         <v>46229</v>
       </c>
       <c r="B295" s="44" t="s">
-        <v>1184</v>
+        <v>1179</v>
       </c>
       <c r="C295" s="83">
         <v>3700</v>
       </c>
       <c r="D295" s="44" t="s">
-        <v>1307</v>
+        <v>1298</v>
       </c>
       <c r="E295" s="44" t="s">
         <v>49</v>
@@ -19694,7 +19718,7 @@
       <c r="F295" s="44"/>
       <c r="G295" s="44"/>
       <c r="H295" s="44" t="s">
-        <v>1308</v>
+        <v>1299</v>
       </c>
       <c r="I295" s="44" t="s">
         <v>148</v>
@@ -19705,7 +19729,7 @@
         <v>46235</v>
       </c>
       <c r="B296" s="45" t="s">
-        <v>1226</v>
+        <v>1220</v>
       </c>
       <c r="C296" s="85">
         <v>1450</v>
@@ -19719,7 +19743,7 @@
       <c r="F296" s="46"/>
       <c r="G296" s="46"/>
       <c r="H296" s="46" t="s">
-        <v>1225</v>
+        <v>1219</v>
       </c>
       <c r="I296" s="45" t="s">
         <v>148</v>
@@ -19730,7 +19754,7 @@
         <v>46236</v>
       </c>
       <c r="B297" s="44" t="s">
-        <v>1312</v>
+        <v>1303</v>
       </c>
       <c r="C297" s="83">
         <v>6900</v>
@@ -19744,7 +19768,7 @@
       <c r="F297" s="44"/>
       <c r="G297" s="44"/>
       <c r="H297" s="44" t="s">
-        <v>1314</v>
+        <v>1305</v>
       </c>
       <c r="I297" s="44" t="s">
         <v>148</v>
@@ -19755,7 +19779,7 @@
         <v>46236</v>
       </c>
       <c r="B298" s="45" t="s">
-        <v>1229</v>
+        <v>1223</v>
       </c>
       <c r="C298" s="85">
         <v>1479</v>
@@ -19769,7 +19793,7 @@
       <c r="F298" s="46"/>
       <c r="G298" s="46"/>
       <c r="H298" s="46" t="s">
-        <v>1228</v>
+        <v>1222</v>
       </c>
       <c r="I298" s="45" t="s">
         <v>148</v>
@@ -19780,7 +19804,7 @@
         <v>46236</v>
       </c>
       <c r="B299" s="44" t="s">
-        <v>1233</v>
+        <v>1227</v>
       </c>
       <c r="C299" s="83">
         <v>2630</v>
@@ -19794,7 +19818,7 @@
       <c r="F299" s="44"/>
       <c r="G299" s="44"/>
       <c r="H299" s="44" t="s">
-        <v>1231</v>
+        <v>1225</v>
       </c>
       <c r="I299" s="44" t="s">
         <v>148</v>
@@ -19805,7 +19829,7 @@
         <v>46238</v>
       </c>
       <c r="B300" s="45" t="s">
-        <v>1097</v>
+        <v>1093</v>
       </c>
       <c r="C300" s="85">
         <v>1380</v>
@@ -19830,7 +19854,7 @@
         <v>46238</v>
       </c>
       <c r="B301" s="44" t="s">
-        <v>1312</v>
+        <v>1303</v>
       </c>
       <c r="C301" s="83">
         <v>12650</v>
@@ -19844,7 +19868,7 @@
       <c r="F301" s="44"/>
       <c r="G301" s="44"/>
       <c r="H301" s="44" t="s">
-        <v>1315</v>
+        <v>1306</v>
       </c>
       <c r="I301" s="44" t="s">
         <v>148</v>
@@ -19855,7 +19879,7 @@
         <v>46240</v>
       </c>
       <c r="B302" s="45" t="s">
-        <v>1229</v>
+        <v>1223</v>
       </c>
       <c r="C302" s="85">
         <v>1000</v>
@@ -19865,7 +19889,7 @@
       <c r="F302" s="46"/>
       <c r="G302" s="46"/>
       <c r="H302" s="46" t="s">
-        <v>1238</v>
+        <v>1232</v>
       </c>
       <c r="I302" s="45" t="s">
         <v>148</v>
@@ -19886,7 +19910,7 @@
       <c r="F303" s="44"/>
       <c r="G303" s="44"/>
       <c r="H303" s="44" t="s">
-        <v>1306</v>
+        <v>1297</v>
       </c>
       <c r="I303" s="44" t="s">
         <v>356</v>
@@ -19897,7 +19921,7 @@
         <v>46243</v>
       </c>
       <c r="B304" s="45" t="s">
-        <v>1280</v>
+        <v>1273</v>
       </c>
       <c r="C304" s="85">
         <v>1380</v>
@@ -19907,7 +19931,7 @@
       <c r="F304" s="46"/>
       <c r="G304" s="46"/>
       <c r="H304" s="46" t="s">
-        <v>1281</v>
+        <v>1274</v>
       </c>
       <c r="I304" s="45" t="s">
         <v>356</v>
@@ -19918,7 +19942,7 @@
         <v>46243</v>
       </c>
       <c r="B305" s="44" t="s">
-        <v>1282</v>
+        <v>1275</v>
       </c>
       <c r="C305" s="83">
         <v>1380</v>
@@ -19932,7 +19956,7 @@
       <c r="F305" s="44"/>
       <c r="G305" s="44"/>
       <c r="H305" s="44" t="s">
-        <v>1283</v>
+        <v>1276</v>
       </c>
       <c r="I305" s="44" t="s">
         <v>148</v>
@@ -19943,7 +19967,7 @@
         <v>46243</v>
       </c>
       <c r="B306" s="45" t="s">
-        <v>1286</v>
+        <v>1277</v>
       </c>
       <c r="C306" s="85">
         <v>1250</v>
@@ -19957,7 +19981,7 @@
       <c r="F306" s="46"/>
       <c r="G306" s="46"/>
       <c r="H306" s="46" t="s">
-        <v>1287</v>
+        <v>1278</v>
       </c>
       <c r="I306" s="45" t="s">
         <v>148</v>
@@ -19968,7 +19992,7 @@
         <v>46243</v>
       </c>
       <c r="B307" s="44" t="s">
-        <v>1312</v>
+        <v>1303</v>
       </c>
       <c r="C307" s="83">
         <v>5750</v>
@@ -19982,7 +20006,7 @@
       <c r="F307" s="44"/>
       <c r="G307" s="44"/>
       <c r="H307" s="44" t="s">
-        <v>1313</v>
+        <v>1304</v>
       </c>
       <c r="I307" s="44" t="s">
         <v>148</v>
@@ -19993,7 +20017,7 @@
         <v>46248</v>
       </c>
       <c r="B308" s="44" t="s">
-        <v>1290</v>
+        <v>1281</v>
       </c>
       <c r="C308" s="83">
         <v>1380</v>
@@ -20007,7 +20031,7 @@
       <c r="F308" s="44"/>
       <c r="G308" s="44"/>
       <c r="H308" s="44" t="s">
-        <v>1291</v>
+        <v>1282</v>
       </c>
       <c r="I308" s="44" t="s">
         <v>148</v>
@@ -20018,7 +20042,7 @@
         <v>46248</v>
       </c>
       <c r="B309" s="45" t="s">
-        <v>1292</v>
+        <v>1283</v>
       </c>
       <c r="C309" s="85">
         <v>1380</v>
@@ -20032,7 +20056,7 @@
       <c r="F309" s="46"/>
       <c r="G309" s="46"/>
       <c r="H309" s="46" t="s">
-        <v>1293</v>
+        <v>1284</v>
       </c>
       <c r="I309" s="45" t="s">
         <v>148</v>
@@ -20057,7 +20081,7 @@
       <c r="F310" s="44"/>
       <c r="G310" s="44"/>
       <c r="H310" s="44" t="s">
-        <v>1303</v>
+        <v>1294</v>
       </c>
       <c r="I310" s="44" t="s">
         <v>148</v>
@@ -20082,7 +20106,7 @@
       <c r="F311" s="46"/>
       <c r="G311" s="46"/>
       <c r="H311" s="46" t="s">
-        <v>1295</v>
+        <v>1286</v>
       </c>
       <c r="I311" s="45" t="s">
         <v>148</v>
@@ -20093,7 +20117,7 @@
         <v>46250</v>
       </c>
       <c r="B312" s="44" t="s">
-        <v>1298</v>
+        <v>1289</v>
       </c>
       <c r="C312" s="83">
         <v>2250</v>
@@ -20107,7 +20131,7 @@
       <c r="F312" s="44"/>
       <c r="G312" s="44"/>
       <c r="H312" s="44" t="s">
-        <v>1300</v>
+        <v>1291</v>
       </c>
       <c r="I312" s="44" t="s">
         <v>148</v>
@@ -20118,7 +20142,7 @@
         <v>46252</v>
       </c>
       <c r="B313" s="45" t="s">
-        <v>1312</v>
+        <v>1303</v>
       </c>
       <c r="C313" s="85">
         <v>5750</v>
@@ -20132,7 +20156,7 @@
       <c r="F313" s="46"/>
       <c r="G313" s="46"/>
       <c r="H313" s="46" t="s">
-        <v>1313</v>
+        <v>1304</v>
       </c>
       <c r="I313" s="45" t="s">
         <v>148</v>
@@ -20143,7 +20167,7 @@
         <v>46252</v>
       </c>
       <c r="B314" s="44" t="s">
-        <v>1316</v>
+        <v>1307</v>
       </c>
       <c r="C314" s="83">
         <v>1380</v>
@@ -20157,7 +20181,7 @@
       <c r="F314" s="44"/>
       <c r="G314" s="44"/>
       <c r="H314" s="44" t="s">
-        <v>1330</v>
+        <v>1319</v>
       </c>
       <c r="I314" s="44" t="s">
         <v>148</v>
@@ -20168,7 +20192,7 @@
         <v>46252</v>
       </c>
       <c r="B315" s="45" t="s">
-        <v>1312</v>
+        <v>1303</v>
       </c>
       <c r="C315" s="85">
         <v>5750</v>
@@ -20182,7 +20206,7 @@
       <c r="F315" s="46"/>
       <c r="G315" s="46"/>
       <c r="H315" s="46" t="s">
-        <v>1313</v>
+        <v>1304</v>
       </c>
       <c r="I315" s="45" t="s">
         <v>148</v>
@@ -20193,7 +20217,7 @@
         <v>46252</v>
       </c>
       <c r="B316" s="44" t="s">
-        <v>1323</v>
+        <v>1312</v>
       </c>
       <c r="C316" s="83">
         <v>1380</v>
@@ -20203,7 +20227,7 @@
       <c r="F316" s="44"/>
       <c r="G316" s="44"/>
       <c r="H316" s="44" t="s">
-        <v>1324</v>
+        <v>1313</v>
       </c>
       <c r="I316" s="44" t="s">
         <v>356</v>
@@ -20214,7 +20238,7 @@
         <v>46252</v>
       </c>
       <c r="B317" s="45" t="s">
-        <v>1326</v>
+        <v>1315</v>
       </c>
       <c r="C317" s="85">
         <v>1250</v>
@@ -20228,66 +20252,134 @@
       <c r="F317" s="46"/>
       <c r="G317" s="46"/>
       <c r="H317" s="46" t="s">
-        <v>1327</v>
+        <v>1316</v>
       </c>
       <c r="I317" s="45" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="318" spans="1:9">
-      <c r="A318" s="82"/>
-      <c r="B318" s="44"/>
-      <c r="C318" s="83"/>
-      <c r="D318" s="44"/>
-      <c r="E318" s="44"/>
+    <row r="318" spans="1:9" ht="14">
+      <c r="A318" s="82">
+        <v>46257</v>
+      </c>
+      <c r="B318" s="44" t="s">
+        <v>1303</v>
+      </c>
+      <c r="C318" s="83">
+        <v>1780</v>
+      </c>
+      <c r="D318" s="44" t="s">
+        <v>162</v>
+      </c>
+      <c r="E318" s="44" t="s">
+        <v>49</v>
+      </c>
       <c r="F318" s="44"/>
       <c r="G318" s="44"/>
-      <c r="H318" s="44"/>
-      <c r="I318" s="44"/>
-    </row>
-    <row r="319" spans="1:9">
-      <c r="A319" s="84"/>
-      <c r="B319" s="45"/>
-      <c r="C319" s="85"/>
-      <c r="D319" s="45"/>
+      <c r="H318" s="44" t="s">
+        <v>1320</v>
+      </c>
+      <c r="I318" s="44" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="319" spans="1:9" ht="14">
+      <c r="A319" s="84">
+        <v>46257</v>
+      </c>
+      <c r="B319" s="45" t="s">
+        <v>175</v>
+      </c>
+      <c r="C319" s="85">
+        <v>2200</v>
+      </c>
+      <c r="D319" s="45" t="s">
+        <v>162</v>
+      </c>
       <c r="E319" s="45"/>
       <c r="F319" s="46"/>
       <c r="G319" s="46"/>
-      <c r="H319" s="46"/>
-      <c r="I319" s="45"/>
-    </row>
-    <row r="320" spans="1:9">
-      <c r="A320" s="82"/>
-      <c r="B320" s="44"/>
-      <c r="C320" s="83"/>
-      <c r="D320" s="44"/>
-      <c r="E320" s="44"/>
+      <c r="H319" s="46" t="s">
+        <v>1323</v>
+      </c>
+      <c r="I319" s="45" t="s">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="320" spans="1:9" ht="14">
+      <c r="A320" s="82">
+        <v>46257</v>
+      </c>
+      <c r="B320" s="44" t="s">
+        <v>49</v>
+      </c>
+      <c r="C320" s="83">
+        <v>700</v>
+      </c>
+      <c r="D320" s="44" t="s">
+        <v>162</v>
+      </c>
+      <c r="E320" s="44" t="s">
+        <v>49</v>
+      </c>
       <c r="F320" s="44"/>
       <c r="G320" s="44"/>
-      <c r="H320" s="44"/>
-      <c r="I320" s="44"/>
-    </row>
-    <row r="321" spans="1:9">
-      <c r="A321" s="84"/>
-      <c r="B321" s="45"/>
-      <c r="C321" s="85"/>
-      <c r="D321" s="45"/>
-      <c r="E321" s="45"/>
+      <c r="H320" s="44" t="s">
+        <v>1326</v>
+      </c>
+      <c r="I320" s="44" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="321" spans="1:9" ht="14">
+      <c r="A321" s="84">
+        <v>46257</v>
+      </c>
+      <c r="B321" s="45" t="s">
+        <v>1332</v>
+      </c>
+      <c r="C321" s="85">
+        <v>1500</v>
+      </c>
+      <c r="D321" s="45" t="s">
+        <v>162</v>
+      </c>
+      <c r="E321" s="45" t="s">
+        <v>49</v>
+      </c>
       <c r="F321" s="46"/>
       <c r="G321" s="46"/>
-      <c r="H321" s="46"/>
-      <c r="I321" s="45"/>
-    </row>
-    <row r="322" spans="1:9">
-      <c r="A322" s="82"/>
-      <c r="B322" s="44"/>
-      <c r="C322" s="83"/>
-      <c r="D322" s="44"/>
-      <c r="E322" s="44"/>
+      <c r="H321" s="46" t="s">
+        <v>1333</v>
+      </c>
+      <c r="I321" s="45" t="s">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="322" spans="1:9" ht="14">
+      <c r="A322" s="82">
+        <v>46258</v>
+      </c>
+      <c r="B322" s="44" t="s">
+        <v>1336</v>
+      </c>
+      <c r="C322" s="83">
+        <v>1250</v>
+      </c>
+      <c r="D322" s="44" t="s">
+        <v>162</v>
+      </c>
+      <c r="E322" s="44" t="s">
+        <v>49</v>
+      </c>
       <c r="F322" s="44"/>
       <c r="G322" s="44"/>
-      <c r="H322" s="44"/>
-      <c r="I322" s="44"/>
+      <c r="H322" s="44" t="s">
+        <v>1337</v>
+      </c>
+      <c r="I322" s="44" t="s">
+        <v>148</v>
+      </c>
     </row>
     <row r="323" spans="1:9">
       <c r="A323" s="84"/>
@@ -26977,7 +27069,7 @@
         <v>0</v>
       </c>
       <c r="L59" s="55" t="s">
-        <v>1277</v>
+        <v>1271</v>
       </c>
       <c r="M59" s="55"/>
       <c r="N59" s="55" t="s">
@@ -28521,7 +28613,7 @@
         <v>0</v>
       </c>
       <c r="L88" s="52" t="s">
-        <v>1114</v>
+        <v>1110</v>
       </c>
       <c r="M88" s="52"/>
       <c r="N88" s="52" t="s">
@@ -28781,7 +28873,7 @@
         <v>472</v>
       </c>
       <c r="L93" s="55" t="s">
-        <v>1166</v>
+        <v>1162</v>
       </c>
       <c r="M93" s="55"/>
       <c r="N93" s="52" t="s">
@@ -29797,7 +29889,7 @@
         <v>0</v>
       </c>
       <c r="L112" s="52" t="s">
-        <v>1100</v>
+        <v>1096</v>
       </c>
       <c r="M112" s="52"/>
       <c r="N112" s="52" t="s">
@@ -30219,7 +30311,7 @@
         <v>3351.6266666666638</v>
       </c>
       <c r="L120" s="52" t="s">
-        <v>1160</v>
+        <v>1156</v>
       </c>
       <c r="M120" s="52" t="s">
         <v>49</v>
@@ -30229,7 +30321,7 @@
       </c>
       <c r="O120" s="52"/>
       <c r="P120" s="52" t="s">
-        <v>1161</v>
+        <v>1157</v>
       </c>
       <c r="Q120" s="52"/>
       <c r="R120" s="52"/>
@@ -31327,7 +31419,7 @@
         <v>0</v>
       </c>
       <c r="L128" s="52" t="s">
-        <v>1072</v>
+        <v>1070</v>
       </c>
       <c r="M128" s="52"/>
       <c r="N128" s="52" t="s">
@@ -32309,7 +32401,7 @@
         <v>0</v>
       </c>
       <c r="L147" s="55" t="s">
-        <v>1157</v>
+        <v>1153</v>
       </c>
       <c r="M147" s="55"/>
       <c r="N147" s="55" t="s">
@@ -32361,7 +32453,7 @@
         <v>1004</v>
       </c>
       <c r="L148" s="52" t="s">
-        <v>1131</v>
+        <v>1127</v>
       </c>
       <c r="M148" s="52"/>
       <c r="N148" s="52" t="s">
@@ -32413,7 +32505,7 @@
         <v>0</v>
       </c>
       <c r="L149" s="55" t="s">
-        <v>1132</v>
+        <v>1128</v>
       </c>
       <c r="M149" s="55"/>
       <c r="N149" s="55" t="s">
@@ -32681,14 +32773,14 @@
         <v>949</v>
       </c>
       <c r="L154" s="52" t="s">
-        <v>1104</v>
+        <v>1100</v>
       </c>
       <c r="M154" s="52"/>
       <c r="N154" s="52" t="s">
         <v>589</v>
       </c>
       <c r="O154" s="52" t="s">
-        <v>1101</v>
+        <v>1097</v>
       </c>
       <c r="P154" s="52"/>
       <c r="Q154" s="52"/>
@@ -32735,14 +32827,14 @@
         <v>949</v>
       </c>
       <c r="L155" s="55" t="s">
-        <v>1121</v>
+        <v>1117</v>
       </c>
       <c r="M155" s="55"/>
       <c r="N155" s="55" t="s">
         <v>589</v>
       </c>
       <c r="O155" s="55" t="s">
-        <v>1101</v>
+        <v>1097</v>
       </c>
       <c r="P155" s="55"/>
       <c r="Q155" s="55"/>
@@ -32789,7 +32881,7 @@
         <v>1900</v>
       </c>
       <c r="L156" s="52" t="s">
-        <v>1105</v>
+        <v>1101</v>
       </c>
       <c r="M156" s="52"/>
       <c r="N156" s="52" t="s">
@@ -33211,7 +33303,7 @@
         <v>0</v>
       </c>
       <c r="L164" s="52" t="s">
-        <v>1136</v>
+        <v>1132</v>
       </c>
       <c r="M164" s="52"/>
       <c r="N164" s="52" t="s">
@@ -33295,10 +33387,10 @@
         <v>950</v>
       </c>
       <c r="F166" s="66">
+        <v>2</v>
+      </c>
+      <c r="G166" s="66">
         <v>1</v>
-      </c>
-      <c r="G166" s="66">
-        <v>2</v>
       </c>
       <c r="H166" s="65">
         <f t="shared" si="11"/>
@@ -33310,22 +33402,22 @@
       </c>
       <c r="J166" s="65">
         <f t="shared" si="9"/>
-        <v>606</v>
+        <v>1212</v>
       </c>
       <c r="K166" s="65">
         <f t="shared" si="10"/>
-        <v>1212</v>
+        <v>606</v>
       </c>
       <c r="L166" s="52" t="s">
-        <v>1089</v>
+        <v>1321</v>
       </c>
       <c r="M166" s="52"/>
       <c r="N166" s="52" t="s">
-        <v>504</v>
+        <v>589</v>
       </c>
       <c r="O166" s="52"/>
       <c r="P166" s="52" t="s">
-        <v>1090</v>
+        <v>1322</v>
       </c>
       <c r="Q166" s="52"/>
       <c r="R166" s="52"/>
@@ -33637,7 +33729,7 @@
         <v>0</v>
       </c>
       <c r="L172" s="52" t="s">
-        <v>1267</v>
+        <v>1261</v>
       </c>
       <c r="M172" s="52"/>
       <c r="N172" s="52" t="s">
@@ -33793,7 +33885,7 @@
         <v>2793</v>
       </c>
       <c r="L175" s="55" t="s">
-        <v>1299</v>
+        <v>1290</v>
       </c>
       <c r="M175" s="55"/>
       <c r="N175" s="55" t="s">
@@ -33801,7 +33893,7 @@
       </c>
       <c r="O175" s="55"/>
       <c r="P175" s="55" t="s">
-        <v>1297</v>
+        <v>1288</v>
       </c>
       <c r="Q175" s="55"/>
       <c r="R175" s="55"/>
@@ -34113,14 +34205,14 @@
         <v>1019</v>
       </c>
       <c r="L181" s="55" t="s">
-        <v>1311</v>
+        <v>1302</v>
       </c>
       <c r="M181" s="55"/>
       <c r="N181" s="55" t="s">
         <v>589</v>
       </c>
       <c r="O181" s="55" t="s">
-        <v>1276</v>
+        <v>1270</v>
       </c>
       <c r="P181" s="55" t="s">
         <v>954</v>
@@ -34220,7 +34312,7 @@
         <v>1676</v>
       </c>
       <c r="L183" s="55" t="s">
-        <v>1176</v>
+        <v>1172</v>
       </c>
       <c r="M183" s="55"/>
       <c r="N183" s="55" t="s">
@@ -34272,7 +34364,7 @@
         <v>0</v>
       </c>
       <c r="L184" s="52" t="s">
-        <v>1234</v>
+        <v>1228</v>
       </c>
       <c r="M184" s="52"/>
       <c r="N184" s="52" t="s">
@@ -34426,7 +34518,7 @@
         <v>891</v>
       </c>
       <c r="L187" s="55" t="s">
-        <v>1316</v>
+        <v>1307</v>
       </c>
       <c r="M187" s="55"/>
       <c r="N187" s="55" t="s">
@@ -34478,7 +34570,7 @@
         <v>891</v>
       </c>
       <c r="L188" s="52" t="s">
-        <v>1235</v>
+        <v>1229</v>
       </c>
       <c r="M188" s="52"/>
       <c r="N188" s="52" t="s">
@@ -34530,7 +34622,7 @@
         <v>891</v>
       </c>
       <c r="L189" s="55" t="s">
-        <v>1322</v>
+        <v>1311</v>
       </c>
       <c r="M189" s="55"/>
       <c r="N189" s="55" t="s">
@@ -34538,7 +34630,7 @@
       </c>
       <c r="O189" s="55"/>
       <c r="P189" s="55" t="s">
-        <v>1325</v>
+        <v>1314</v>
       </c>
       <c r="Q189" s="55"/>
       <c r="R189" s="55"/>
@@ -34584,7 +34676,7 @@
         <v>0</v>
       </c>
       <c r="L190" s="52" t="s">
-        <v>1167</v>
+        <v>1163</v>
       </c>
       <c r="M190" s="52"/>
       <c r="N190" s="47" t="s">
@@ -34681,14 +34773,14 @@
         <v>1616</v>
       </c>
       <c r="L192" s="52" t="s">
-        <v>1081</v>
+        <v>1079</v>
       </c>
       <c r="M192" s="52"/>
       <c r="N192" s="47" t="s">
         <v>589</v>
       </c>
       <c r="P192" s="47" t="s">
-        <v>1082</v>
+        <v>1080</v>
       </c>
       <c r="S192" s="47"/>
       <c r="T192" s="47"/>
@@ -34747,7 +34839,7 @@
         <v>982</v>
       </c>
       <c r="B194" s="52" t="s">
-        <v>1302</v>
+        <v>1293</v>
       </c>
       <c r="C194" s="52" t="s">
         <v>95</v>
@@ -34781,14 +34873,14 @@
         <v>6320</v>
       </c>
       <c r="L194" s="52" t="s">
-        <v>1135</v>
+        <v>1131</v>
       </c>
       <c r="M194" s="52"/>
       <c r="N194" s="47" t="s">
         <v>589</v>
       </c>
       <c r="P194" s="47" t="s">
-        <v>1301</v>
+        <v>1292</v>
       </c>
       <c r="S194" s="47"/>
       <c r="T194" s="47"/>
@@ -34981,14 +35073,14 @@
         <v>1401</v>
       </c>
       <c r="L198" s="55" t="s">
-        <v>1182</v>
+        <v>1177</v>
       </c>
       <c r="M198" s="55"/>
       <c r="N198" s="47" t="s">
         <v>589</v>
       </c>
       <c r="P198" s="47" t="s">
-        <v>1183</v>
+        <v>1178</v>
       </c>
       <c r="S198" s="47"/>
       <c r="T198" s="47"/>
@@ -35032,14 +35124,14 @@
         <v>1732</v>
       </c>
       <c r="L199" s="52" t="s">
-        <v>1328</v>
+        <v>1317</v>
       </c>
       <c r="M199" s="52"/>
       <c r="N199" s="47" t="s">
         <v>589</v>
       </c>
       <c r="P199" s="47" t="s">
-        <v>1329</v>
+        <v>1318</v>
       </c>
       <c r="S199" s="47"/>
       <c r="T199" s="47"/>
@@ -35134,14 +35226,14 @@
         <v>940</v>
       </c>
       <c r="L201" s="52" t="s">
-        <v>1149</v>
+        <v>1145</v>
       </c>
       <c r="M201" s="52"/>
       <c r="N201" s="47" t="s">
         <v>589</v>
       </c>
       <c r="P201" s="47" t="s">
-        <v>1150</v>
+        <v>1146</v>
       </c>
       <c r="S201" s="47"/>
       <c r="T201" s="47"/>
@@ -35236,14 +35328,14 @@
         <v>880</v>
       </c>
       <c r="L203" s="52" t="s">
-        <v>1110</v>
+        <v>1106</v>
       </c>
       <c r="M203" s="52"/>
       <c r="N203" s="47" t="s">
         <v>589</v>
       </c>
       <c r="P203" s="47" t="s">
-        <v>1109</v>
+        <v>1105</v>
       </c>
       <c r="S203" s="47"/>
       <c r="T203" s="47"/>
@@ -35265,10 +35357,10 @@
         <v>1250</v>
       </c>
       <c r="F204" s="64">
+        <v>2</v>
+      </c>
+      <c r="G204" s="64">
         <v>1</v>
-      </c>
-      <c r="G204" s="64">
-        <v>2</v>
       </c>
       <c r="H204" s="63">
         <f t="shared" si="12"/>
@@ -35280,31 +35372,31 @@
       </c>
       <c r="J204" s="63">
         <f t="shared" si="13"/>
-        <v>761</v>
+        <v>1522</v>
       </c>
       <c r="K204" s="63">
         <f t="shared" si="14"/>
-        <v>1522</v>
+        <v>761</v>
       </c>
       <c r="L204" s="55" t="s">
-        <v>1011</v>
+        <v>1324</v>
       </c>
       <c r="M204" s="55"/>
       <c r="N204" s="47" t="s">
-        <v>678</v>
+        <v>589</v>
       </c>
       <c r="P204" s="47" t="s">
-        <v>1012</v>
+        <v>1325</v>
       </c>
       <c r="S204" s="47"/>
       <c r="T204" s="47"/>
     </row>
     <row r="205" spans="1:20" ht="15" customHeight="1">
       <c r="A205" s="52" t="s">
-        <v>1013</v>
+        <v>1011</v>
       </c>
       <c r="B205" s="52" t="s">
-        <v>1014</v>
+        <v>1012</v>
       </c>
       <c r="C205" s="52" t="s">
         <v>95</v>
@@ -35345,17 +35437,17 @@
         <v>504</v>
       </c>
       <c r="P205" s="47" t="s">
-        <v>1015</v>
+        <v>1013</v>
       </c>
       <c r="S205" s="47"/>
       <c r="T205" s="47"/>
     </row>
     <row r="206" spans="1:20" ht="15" customHeight="1">
       <c r="A206" s="55" t="s">
-        <v>1016</v>
+        <v>1014</v>
       </c>
       <c r="B206" s="55" t="s">
-        <v>1017</v>
+        <v>1015</v>
       </c>
       <c r="C206" s="55" t="s">
         <v>95</v>
@@ -35389,24 +35481,24 @@
         <v>3312</v>
       </c>
       <c r="L206" s="55" t="s">
-        <v>1018</v>
+        <v>1016</v>
       </c>
       <c r="M206" s="55"/>
       <c r="N206" s="47" t="s">
         <v>589</v>
       </c>
       <c r="P206" s="47" t="s">
-        <v>1019</v>
+        <v>1017</v>
       </c>
       <c r="S206" s="47"/>
       <c r="T206" s="47"/>
     </row>
     <row r="207" spans="1:20" ht="30" customHeight="1">
       <c r="A207" s="52" t="s">
-        <v>1020</v>
+        <v>1018</v>
       </c>
       <c r="B207" s="52" t="s">
-        <v>1021</v>
+        <v>1019</v>
       </c>
       <c r="C207" s="52" t="s">
         <v>95</v>
@@ -35445,17 +35537,17 @@
         <v>678</v>
       </c>
       <c r="P207" s="47" t="s">
-        <v>1022</v>
+        <v>1020</v>
       </c>
       <c r="S207" s="47"/>
       <c r="T207" s="47"/>
     </row>
     <row r="208" spans="1:20" ht="15" customHeight="1">
       <c r="A208" s="55" t="s">
-        <v>1023</v>
+        <v>1021</v>
       </c>
       <c r="B208" s="52" t="s">
-        <v>1024</v>
+        <v>1022</v>
       </c>
       <c r="C208" s="52" t="s">
         <v>95</v>
@@ -35489,24 +35581,24 @@
         <v>982</v>
       </c>
       <c r="L208" s="55" t="s">
-        <v>1084</v>
+        <v>1082</v>
       </c>
       <c r="M208" s="55"/>
       <c r="N208" s="47" t="s">
         <v>589</v>
       </c>
       <c r="P208" s="47" t="s">
-        <v>1083</v>
+        <v>1081</v>
       </c>
       <c r="S208" s="47"/>
       <c r="T208" s="47"/>
     </row>
     <row r="209" spans="1:20" ht="15" customHeight="1">
       <c r="A209" s="52" t="s">
-        <v>1025</v>
+        <v>1023</v>
       </c>
       <c r="B209" s="55" t="s">
-        <v>1026</v>
+        <v>1024</v>
       </c>
       <c r="C209" s="55" t="s">
         <v>95</v>
@@ -35545,14 +35637,14 @@
         <v>678</v>
       </c>
       <c r="P209" s="47" t="s">
-        <v>1027</v>
+        <v>1025</v>
       </c>
       <c r="S209" s="47"/>
       <c r="T209" s="47"/>
     </row>
     <row r="210" spans="1:20" ht="15" customHeight="1">
       <c r="A210" s="55" t="s">
-        <v>1028</v>
+        <v>1026</v>
       </c>
       <c r="B210" s="52" t="s">
         <v>901</v>
@@ -35594,17 +35686,17 @@
         <v>678</v>
       </c>
       <c r="P210" s="47" t="s">
-        <v>1029</v>
+        <v>1027</v>
       </c>
       <c r="S210" s="47"/>
       <c r="T210" s="47"/>
     </row>
     <row r="211" spans="1:20" ht="15" customHeight="1">
       <c r="A211" s="52" t="s">
-        <v>1030</v>
+        <v>1028</v>
       </c>
       <c r="B211" s="55" t="s">
-        <v>1099</v>
+        <v>1095</v>
       </c>
       <c r="C211" s="55" t="s">
         <v>95</v>
@@ -35638,7 +35730,7 @@
         <v>0</v>
       </c>
       <c r="L211" s="52" t="s">
-        <v>1317</v>
+        <v>1308</v>
       </c>
       <c r="M211" s="52"/>
       <c r="N211" s="47" t="s">
@@ -35649,10 +35741,10 @@
     </row>
     <row r="212" spans="1:20" ht="15" customHeight="1">
       <c r="A212" s="55" t="s">
-        <v>1031</v>
+        <v>1029</v>
       </c>
       <c r="B212" s="52" t="s">
-        <v>1134</v>
+        <v>1130</v>
       </c>
       <c r="C212" s="52" t="s">
         <v>95</v>
@@ -35664,14 +35756,14 @@
         <v>850</v>
       </c>
       <c r="F212" s="64">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G212" s="64">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H212" s="63">
         <f t="shared" si="12"/>
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="I212" s="63">
         <f>IF(D212&lt;&gt;"",D212,IFERROR(E212/(IFERROR(SUM(Sales!C:C),0))*(IFERROR(SUM(Purchases!C:C),0)),0))</f>
@@ -35679,31 +35771,31 @@
       </c>
       <c r="J212" s="63">
         <f t="shared" si="13"/>
-        <v>2220</v>
+        <v>2775</v>
       </c>
       <c r="K212" s="63">
         <f t="shared" si="14"/>
-        <v>2775</v>
+        <v>1665</v>
       </c>
       <c r="L212" s="55" t="s">
-        <v>1320</v>
+        <v>1327</v>
       </c>
       <c r="M212" s="55"/>
       <c r="N212" s="47" t="s">
         <v>589</v>
       </c>
       <c r="P212" s="47" t="s">
-        <v>1321</v>
+        <v>1328</v>
       </c>
       <c r="S212" s="47"/>
       <c r="T212" s="47"/>
     </row>
     <row r="213" spans="1:20" ht="15" customHeight="1">
       <c r="A213" s="52" t="s">
-        <v>1032</v>
+        <v>1030</v>
       </c>
       <c r="B213" s="52" t="s">
-        <v>1138</v>
+        <v>1134</v>
       </c>
       <c r="C213" s="52" t="s">
         <v>95</v>
@@ -35715,10 +35807,10 @@
         <v>1250</v>
       </c>
       <c r="F213" s="66">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G213" s="66">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H213" s="65">
         <f t="shared" si="12"/>
@@ -35730,29 +35822,31 @@
       </c>
       <c r="J213" s="65">
         <f t="shared" si="13"/>
-        <v>0</v>
+        <v>835</v>
       </c>
       <c r="K213" s="65">
         <f t="shared" si="14"/>
-        <v>4175</v>
-      </c>
-      <c r="L213" s="52"/>
+        <v>3340</v>
+      </c>
+      <c r="L213" s="52" t="s">
+        <v>1338</v>
+      </c>
       <c r="M213" s="52"/>
       <c r="N213" s="47" t="s">
-        <v>678</v>
+        <v>589</v>
       </c>
       <c r="P213" s="47" t="s">
-        <v>1139</v>
+        <v>1135</v>
       </c>
       <c r="S213" s="47"/>
       <c r="T213" s="47"/>
     </row>
     <row r="214" spans="1:20" ht="15" customHeight="1">
       <c r="A214" s="55" t="s">
-        <v>1033</v>
+        <v>1031</v>
       </c>
       <c r="B214" s="55" t="s">
-        <v>1140</v>
+        <v>1136</v>
       </c>
       <c r="C214" s="55" t="s">
         <v>95</v>
@@ -35786,21 +35880,21 @@
         <v>2976</v>
       </c>
       <c r="L214" s="55" t="s">
-        <v>1227</v>
+        <v>1221</v>
       </c>
       <c r="M214" s="55"/>
       <c r="N214" s="47" t="s">
         <v>589</v>
       </c>
       <c r="P214" s="47" t="s">
-        <v>1141</v>
+        <v>1137</v>
       </c>
       <c r="S214" s="47"/>
       <c r="T214" s="47"/>
     </row>
     <row r="215" spans="1:20" ht="30">
       <c r="A215" s="52" t="s">
-        <v>1034</v>
+        <v>1032</v>
       </c>
       <c r="B215" s="52" t="s">
         <v>994</v>
@@ -35815,10 +35909,10 @@
         <v>899</v>
       </c>
       <c r="F215" s="66">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G215" s="66">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H215" s="65">
         <f t="shared" si="12"/>
@@ -35830,31 +35924,29 @@
       </c>
       <c r="J215" s="65">
         <f t="shared" si="13"/>
-        <v>576</v>
+        <v>0</v>
       </c>
       <c r="K215" s="65">
         <f t="shared" si="14"/>
-        <v>2880</v>
-      </c>
-      <c r="L215" s="52" t="s">
-        <v>1179</v>
-      </c>
+        <v>3456</v>
+      </c>
+      <c r="L215" s="52"/>
       <c r="M215" s="52"/>
       <c r="N215" s="47" t="s">
-        <v>589</v>
+        <v>678</v>
       </c>
       <c r="P215" s="47" t="s">
-        <v>1180</v>
+        <v>1175</v>
       </c>
       <c r="S215" s="47"/>
       <c r="T215" s="47"/>
     </row>
     <row r="216" spans="1:20" ht="15" customHeight="1">
       <c r="A216" s="55" t="s">
-        <v>1035</v>
+        <v>1033</v>
       </c>
       <c r="B216" s="55" t="s">
-        <v>1142</v>
+        <v>1138</v>
       </c>
       <c r="C216" s="55" t="s">
         <v>95</v>
@@ -35888,24 +35980,24 @@
         <v>0</v>
       </c>
       <c r="L216" s="55" t="s">
-        <v>1275</v>
+        <v>1269</v>
       </c>
       <c r="M216" s="55"/>
       <c r="N216" s="47" t="s">
         <v>504</v>
       </c>
       <c r="P216" s="47" t="s">
-        <v>1143</v>
+        <v>1139</v>
       </c>
       <c r="S216" s="47"/>
       <c r="T216" s="47"/>
     </row>
     <row r="217" spans="1:20" ht="15">
       <c r="A217" s="52" t="s">
-        <v>1036</v>
+        <v>1034</v>
       </c>
       <c r="B217" s="52" t="s">
-        <v>1144</v>
+        <v>1140</v>
       </c>
       <c r="C217" s="52" t="s">
         <v>95</v>
@@ -35939,24 +36031,24 @@
         <v>828</v>
       </c>
       <c r="L217" s="52" t="s">
-        <v>1177</v>
+        <v>1173</v>
       </c>
       <c r="M217" s="52"/>
       <c r="N217" s="47" t="s">
         <v>589</v>
       </c>
       <c r="P217" s="47" t="s">
-        <v>1178</v>
+        <v>1174</v>
       </c>
       <c r="S217" s="47"/>
       <c r="T217" s="47"/>
     </row>
     <row r="218" spans="1:20" ht="15" customHeight="1">
       <c r="A218" s="55" t="s">
-        <v>1037</v>
+        <v>1035</v>
       </c>
       <c r="B218" s="55" t="s">
-        <v>1145</v>
+        <v>1141</v>
       </c>
       <c r="C218" s="55" t="s">
         <v>95</v>
@@ -35990,24 +36082,24 @@
         <v>2283</v>
       </c>
       <c r="L218" s="55" t="s">
-        <v>1186</v>
+        <v>1181</v>
       </c>
       <c r="M218" s="55"/>
       <c r="N218" s="47" t="s">
         <v>678</v>
       </c>
       <c r="P218" s="47" t="s">
-        <v>1185</v>
+        <v>1180</v>
       </c>
       <c r="S218" s="47"/>
       <c r="T218" s="47"/>
     </row>
     <row r="219" spans="1:20" ht="15">
       <c r="A219" s="52" t="s">
-        <v>1038</v>
+        <v>1036</v>
       </c>
       <c r="B219" s="52" t="s">
-        <v>1146</v>
+        <v>1142</v>
       </c>
       <c r="C219" s="52" t="s">
         <v>95</v>
@@ -36041,24 +36133,24 @@
         <v>3805</v>
       </c>
       <c r="L219" s="52" t="s">
-        <v>1173</v>
+        <v>1169</v>
       </c>
       <c r="M219" s="52"/>
       <c r="N219" s="47" t="s">
         <v>589</v>
       </c>
       <c r="P219" s="47" t="s">
-        <v>1174</v>
+        <v>1170</v>
       </c>
       <c r="S219" s="47"/>
       <c r="T219" s="47"/>
     </row>
     <row r="220" spans="1:20" ht="15" customHeight="1">
       <c r="A220" s="55" t="s">
-        <v>1039</v>
+        <v>1037</v>
       </c>
       <c r="B220" s="55" t="s">
-        <v>1170</v>
+        <v>1166</v>
       </c>
       <c r="C220" s="55" t="s">
         <v>95</v>
@@ -36097,17 +36189,17 @@
         <v>678</v>
       </c>
       <c r="P220" s="47" t="s">
-        <v>1171</v>
+        <v>1167</v>
       </c>
       <c r="S220" s="47"/>
       <c r="T220" s="47"/>
     </row>
     <row r="221" spans="1:20" ht="17">
       <c r="A221" s="52" t="s">
-        <v>1040</v>
+        <v>1038</v>
       </c>
       <c r="B221" s="52" t="s">
-        <v>1187</v>
+        <v>1182</v>
       </c>
       <c r="C221" s="52" t="s">
         <v>96</v>
@@ -36146,17 +36238,17 @@
         <v>678</v>
       </c>
       <c r="P221" s="86" t="s">
-        <v>1214</v>
+        <v>1209</v>
       </c>
       <c r="S221" s="47"/>
       <c r="T221" s="47"/>
     </row>
     <row r="222" spans="1:20" ht="15" customHeight="1">
       <c r="A222" s="55" t="s">
-        <v>1041</v>
+        <v>1039</v>
       </c>
       <c r="B222" s="55" t="s">
-        <v>1188</v>
+        <v>1183</v>
       </c>
       <c r="C222" s="55" t="s">
         <v>95</v>
@@ -36195,17 +36287,17 @@
         <v>678</v>
       </c>
       <c r="P222" s="86" t="s">
-        <v>1215</v>
+        <v>1210</v>
       </c>
       <c r="S222" s="47"/>
       <c r="T222" s="47"/>
     </row>
     <row r="223" spans="1:20" ht="15" customHeight="1">
       <c r="A223" s="52" t="s">
-        <v>1042</v>
+        <v>1040</v>
       </c>
       <c r="B223" s="52" t="s">
-        <v>1189</v>
+        <v>1184</v>
       </c>
       <c r="C223" s="52" t="s">
         <v>95</v>
@@ -36239,24 +36331,24 @@
         <v>942</v>
       </c>
       <c r="L223" s="52" t="s">
-        <v>1230</v>
+        <v>1224</v>
       </c>
       <c r="M223" s="52"/>
       <c r="N223" s="47" t="s">
         <v>589</v>
       </c>
       <c r="P223" s="86" t="s">
-        <v>1232</v>
+        <v>1226</v>
       </c>
       <c r="S223" s="47"/>
       <c r="T223" s="47"/>
     </row>
     <row r="224" spans="1:20" ht="15" customHeight="1">
       <c r="A224" s="55" t="s">
-        <v>1043</v>
+        <v>1041</v>
       </c>
       <c r="B224" s="55" t="s">
-        <v>1190</v>
+        <v>1185</v>
       </c>
       <c r="C224" s="55" t="s">
         <v>95</v>
@@ -36297,17 +36389,17 @@
         <v>504</v>
       </c>
       <c r="P224" s="86" t="s">
-        <v>1216</v>
+        <v>1211</v>
       </c>
       <c r="S224" s="47"/>
       <c r="T224" s="47"/>
     </row>
     <row r="225" spans="1:20" ht="15" customHeight="1">
       <c r="A225" s="52" t="s">
-        <v>1044</v>
+        <v>1042</v>
       </c>
       <c r="B225" s="52" t="s">
-        <v>1191</v>
+        <v>1186</v>
       </c>
       <c r="C225" s="52" t="s">
         <v>95</v>
@@ -36319,10 +36411,10 @@
         <v>1500</v>
       </c>
       <c r="F225" s="66">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G225" s="66">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H225" s="65">
         <f t="shared" si="12"/>
@@ -36334,29 +36426,31 @@
       </c>
       <c r="J225" s="65">
         <f t="shared" si="13"/>
-        <v>0</v>
+        <v>940</v>
       </c>
       <c r="K225" s="65">
         <f t="shared" si="14"/>
-        <v>1880</v>
-      </c>
-      <c r="L225" s="52"/>
+        <v>940</v>
+      </c>
+      <c r="L225" s="52" t="s">
+        <v>1334</v>
+      </c>
       <c r="M225" s="52"/>
       <c r="N225" s="47" t="s">
-        <v>678</v>
+        <v>589</v>
       </c>
       <c r="P225" s="86" t="s">
-        <v>1217</v>
+        <v>1335</v>
       </c>
       <c r="S225" s="47"/>
       <c r="T225" s="47"/>
     </row>
     <row r="226" spans="1:20" ht="17">
       <c r="A226" s="52" t="s">
-        <v>1202</v>
+        <v>1197</v>
       </c>
       <c r="B226" s="55" t="s">
-        <v>1192</v>
+        <v>1187</v>
       </c>
       <c r="C226" s="55" t="s">
         <v>95</v>
@@ -36390,24 +36484,24 @@
         <v>1338</v>
       </c>
       <c r="L226" s="55" t="s">
-        <v>1184</v>
+        <v>1179</v>
       </c>
       <c r="M226" s="55"/>
       <c r="N226" s="47" t="s">
         <v>678</v>
       </c>
       <c r="P226" s="86" t="s">
-        <v>1218</v>
+        <v>1212</v>
       </c>
       <c r="S226" s="47"/>
       <c r="T226" s="47"/>
     </row>
     <row r="227" spans="1:20" ht="17">
       <c r="A227" s="55" t="s">
-        <v>1203</v>
+        <v>1198</v>
       </c>
       <c r="B227" s="52" t="s">
-        <v>1193</v>
+        <v>1188</v>
       </c>
       <c r="C227" s="52" t="s">
         <v>95</v>
@@ -36446,17 +36540,17 @@
         <v>678</v>
       </c>
       <c r="P227" s="86" t="s">
-        <v>1219</v>
+        <v>1213</v>
       </c>
       <c r="S227" s="47"/>
       <c r="T227" s="47"/>
     </row>
     <row r="228" spans="1:20" ht="17">
       <c r="A228" s="52" t="s">
-        <v>1204</v>
+        <v>1199</v>
       </c>
       <c r="B228" s="55" t="s">
-        <v>1194</v>
+        <v>1189</v>
       </c>
       <c r="C228" s="55" t="s">
         <v>95</v>
@@ -36490,24 +36584,24 @@
         <v>2775</v>
       </c>
       <c r="L228" s="55" t="s">
-        <v>1304</v>
+        <v>1295</v>
       </c>
       <c r="M228" s="55"/>
       <c r="N228" s="47" t="s">
         <v>589</v>
       </c>
       <c r="P228" s="86" t="s">
-        <v>1305</v>
+        <v>1296</v>
       </c>
       <c r="S228" s="47"/>
       <c r="T228" s="47"/>
     </row>
     <row r="229" spans="1:20" ht="17">
       <c r="A229" s="55" t="s">
-        <v>1205</v>
+        <v>1200</v>
       </c>
       <c r="B229" s="52" t="s">
-        <v>1195</v>
+        <v>1190</v>
       </c>
       <c r="C229" s="52" t="s">
         <v>95</v>
@@ -36541,24 +36635,24 @@
         <v>782</v>
       </c>
       <c r="L229" s="52" t="s">
-        <v>1272</v>
+        <v>1266</v>
       </c>
       <c r="M229" s="52"/>
       <c r="N229" s="47" t="s">
         <v>589</v>
       </c>
       <c r="P229" s="86" t="s">
-        <v>1273</v>
+        <v>1267</v>
       </c>
       <c r="S229" s="47"/>
       <c r="T229" s="47"/>
     </row>
     <row r="230" spans="1:20" ht="17">
       <c r="A230" s="52" t="s">
-        <v>1206</v>
+        <v>1201</v>
       </c>
       <c r="B230" s="55" t="s">
-        <v>1194</v>
+        <v>1189</v>
       </c>
       <c r="C230" s="55" t="s">
         <v>95</v>
@@ -36599,17 +36693,17 @@
         <v>589</v>
       </c>
       <c r="P230" s="86" t="s">
-        <v>1220</v>
+        <v>1214</v>
       </c>
       <c r="S230" s="47"/>
       <c r="T230" s="47"/>
     </row>
     <row r="231" spans="1:20" ht="17">
       <c r="A231" s="52" t="s">
-        <v>1207</v>
+        <v>1202</v>
       </c>
       <c r="B231" s="52" t="s">
-        <v>1196</v>
+        <v>1191</v>
       </c>
       <c r="C231" s="52" t="s">
         <v>95</v>
@@ -36648,17 +36742,17 @@
         <v>678</v>
       </c>
       <c r="P231" s="86" t="s">
-        <v>1171</v>
+        <v>1167</v>
       </c>
       <c r="S231" s="47"/>
       <c r="T231" s="47"/>
     </row>
     <row r="232" spans="1:20" ht="17">
       <c r="A232" s="55" t="s">
-        <v>1208</v>
+        <v>1203</v>
       </c>
       <c r="B232" s="55" t="s">
-        <v>1197</v>
+        <v>1192</v>
       </c>
       <c r="C232" s="55" t="s">
         <v>95</v>
@@ -36692,24 +36786,24 @@
         <v>0</v>
       </c>
       <c r="L232" s="55" t="s">
-        <v>1224</v>
+        <v>1218</v>
       </c>
       <c r="M232" s="55"/>
       <c r="N232" s="47" t="s">
         <v>504</v>
       </c>
       <c r="P232" s="86" t="s">
-        <v>1221</v>
+        <v>1215</v>
       </c>
       <c r="S232" s="47"/>
       <c r="T232" s="47"/>
     </row>
     <row r="233" spans="1:20" ht="17">
       <c r="A233" s="52" t="s">
-        <v>1209</v>
+        <v>1204</v>
       </c>
       <c r="B233" s="52" t="s">
-        <v>1198</v>
+        <v>1193</v>
       </c>
       <c r="C233" s="52" t="s">
         <v>95</v>
@@ -36743,24 +36837,24 @@
         <v>1048</v>
       </c>
       <c r="L233" s="52" t="s">
-        <v>1274</v>
+        <v>1268</v>
       </c>
       <c r="M233" s="52"/>
       <c r="N233" s="47" t="s">
         <v>678</v>
       </c>
       <c r="P233" s="86" t="s">
-        <v>1222</v>
+        <v>1216</v>
       </c>
       <c r="S233" s="47"/>
       <c r="T233" s="47"/>
     </row>
     <row r="234" spans="1:20" ht="17">
       <c r="A234" s="55" t="s">
-        <v>1210</v>
+        <v>1205</v>
       </c>
       <c r="B234" s="55" t="s">
-        <v>1199</v>
+        <v>1194</v>
       </c>
       <c r="C234" s="55" t="s">
         <v>95</v>
@@ -36794,21 +36888,21 @@
         <v>891</v>
       </c>
       <c r="L234" s="55" t="s">
-        <v>1294</v>
+        <v>1285</v>
       </c>
       <c r="M234" s="55"/>
       <c r="N234" s="47" t="s">
         <v>589</v>
       </c>
       <c r="P234" s="86" t="s">
-        <v>1223</v>
+        <v>1217</v>
       </c>
       <c r="S234" s="47"/>
       <c r="T234" s="47"/>
     </row>
     <row r="235" spans="1:20" ht="17">
       <c r="A235" s="52" t="s">
-        <v>1211</v>
+        <v>1206</v>
       </c>
       <c r="B235" s="52" t="s">
         <v>510</v>
@@ -36823,10 +36917,10 @@
         <v>1380</v>
       </c>
       <c r="F235" s="66">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G235" s="66">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H235" s="65">
         <f t="shared" si="15"/>
@@ -36838,31 +36932,31 @@
       </c>
       <c r="J235" s="65">
         <f t="shared" si="16"/>
-        <v>912</v>
+        <v>1824</v>
       </c>
       <c r="K235" s="65">
         <f t="shared" si="17"/>
-        <v>2736</v>
+        <v>1824</v>
       </c>
       <c r="L235" s="52" t="s">
-        <v>1284</v>
+        <v>1330</v>
       </c>
       <c r="M235" s="52"/>
       <c r="N235" s="47" t="s">
         <v>589</v>
       </c>
       <c r="P235" s="86" t="s">
-        <v>1285</v>
+        <v>1331</v>
       </c>
       <c r="S235" s="47"/>
       <c r="T235" s="47"/>
     </row>
     <row r="236" spans="1:20" ht="17">
       <c r="A236" s="52" t="s">
-        <v>1212</v>
+        <v>1207</v>
       </c>
       <c r="B236" s="55" t="s">
-        <v>1200</v>
+        <v>1195</v>
       </c>
       <c r="C236" s="55" t="s">
         <v>95</v>
@@ -36896,24 +36990,24 @@
         <v>1468</v>
       </c>
       <c r="L236" s="55" t="s">
-        <v>1270</v>
+        <v>1264</v>
       </c>
       <c r="M236" s="55"/>
       <c r="N236" s="47" t="s">
         <v>678</v>
       </c>
       <c r="P236" s="86" t="s">
-        <v>1271</v>
+        <v>1265</v>
       </c>
       <c r="S236" s="47"/>
       <c r="T236" s="47"/>
     </row>
     <row r="237" spans="1:20" ht="17">
       <c r="A237" s="55" t="s">
-        <v>1213</v>
+        <v>1208</v>
       </c>
       <c r="B237" s="52" t="s">
-        <v>1201</v>
+        <v>1196</v>
       </c>
       <c r="C237" s="52" t="s">
         <v>95</v>
@@ -36947,24 +37041,24 @@
         <v>872</v>
       </c>
       <c r="L237" s="52" t="s">
-        <v>1269</v>
+        <v>1263</v>
       </c>
       <c r="M237" s="52"/>
       <c r="N237" s="47" t="s">
         <v>678</v>
       </c>
       <c r="P237" s="86" t="s">
-        <v>1268</v>
+        <v>1262</v>
       </c>
       <c r="S237" s="47"/>
       <c r="T237" s="47"/>
     </row>
     <row r="238" spans="1:20" ht="16">
       <c r="A238" s="55" t="s">
-        <v>1236</v>
+        <v>1230</v>
       </c>
       <c r="B238" s="55" t="s">
-        <v>1197</v>
+        <v>1192</v>
       </c>
       <c r="C238" s="55" t="s">
         <v>95</v>
@@ -36998,7 +37092,7 @@
         <v>0</v>
       </c>
       <c r="L238" s="55" t="s">
-        <v>1237</v>
+        <v>1231</v>
       </c>
       <c r="M238" s="55"/>
       <c r="N238" s="47" t="s">
@@ -37010,10 +37104,10 @@
     </row>
     <row r="239" spans="1:20" ht="17">
       <c r="A239" s="52" t="s">
-        <v>1239</v>
+        <v>1233</v>
       </c>
       <c r="B239" s="52" t="s">
-        <v>1249</v>
+        <v>1243</v>
       </c>
       <c r="C239" s="52" t="s">
         <v>95</v>
@@ -37052,17 +37146,17 @@
         <v>678</v>
       </c>
       <c r="P239" s="86" t="s">
-        <v>1260</v>
+        <v>1254</v>
       </c>
       <c r="S239" s="47"/>
       <c r="T239" s="47"/>
     </row>
     <row r="240" spans="1:20" ht="17">
       <c r="A240" s="55" t="s">
-        <v>1240</v>
+        <v>1234</v>
       </c>
       <c r="B240" s="55" t="s">
-        <v>1258</v>
+        <v>1252</v>
       </c>
       <c r="C240" s="55" t="s">
         <v>95</v>
@@ -37096,7 +37190,7 @@
         <v>0</v>
       </c>
       <c r="L240" s="55" t="s">
-        <v>1259</v>
+        <v>1253</v>
       </c>
       <c r="M240" s="55"/>
       <c r="N240" s="47" t="s">
@@ -37110,10 +37204,10 @@
     </row>
     <row r="241" spans="1:20" ht="17">
       <c r="A241" s="52" t="s">
-        <v>1241</v>
+        <v>1235</v>
       </c>
       <c r="B241" s="52" t="s">
-        <v>1250</v>
+        <v>1244</v>
       </c>
       <c r="C241" s="52" t="s">
         <v>95</v>
@@ -37147,24 +37241,24 @@
         <v>1124</v>
       </c>
       <c r="L241" s="52" t="s">
-        <v>1296</v>
+        <v>1287</v>
       </c>
       <c r="M241" s="52"/>
       <c r="N241" s="47" t="s">
         <v>589</v>
       </c>
       <c r="P241" s="86" t="s">
-        <v>1261</v>
+        <v>1255</v>
       </c>
       <c r="S241" s="47"/>
       <c r="T241" s="47"/>
     </row>
     <row r="242" spans="1:20" ht="17">
       <c r="A242" s="55" t="s">
-        <v>1242</v>
+        <v>1236</v>
       </c>
       <c r="B242" s="55" t="s">
-        <v>1251</v>
+        <v>1245</v>
       </c>
       <c r="C242" s="55" t="s">
         <v>95</v>
@@ -37205,17 +37299,17 @@
         <v>678</v>
       </c>
       <c r="P242" s="86" t="s">
-        <v>1262</v>
+        <v>1256</v>
       </c>
       <c r="S242" s="47"/>
       <c r="T242" s="47"/>
     </row>
     <row r="243" spans="1:20" ht="17">
       <c r="A243" s="52" t="s">
-        <v>1243</v>
+        <v>1237</v>
       </c>
       <c r="B243" s="52" t="s">
-        <v>1252</v>
+        <v>1246</v>
       </c>
       <c r="C243" s="52" t="s">
         <v>95</v>
@@ -37249,24 +37343,24 @@
         <v>545</v>
       </c>
       <c r="L243" s="52" t="s">
-        <v>1289</v>
+        <v>1280</v>
       </c>
       <c r="M243" s="52"/>
       <c r="N243" s="47" t="s">
         <v>589</v>
       </c>
       <c r="P243" s="86" t="s">
-        <v>1263</v>
+        <v>1257</v>
       </c>
       <c r="S243" s="47"/>
       <c r="T243" s="47"/>
     </row>
     <row r="244" spans="1:20" ht="17">
       <c r="A244" s="55" t="s">
-        <v>1244</v>
+        <v>1238</v>
       </c>
       <c r="B244" s="55" t="s">
-        <v>1253</v>
+        <v>1247</v>
       </c>
       <c r="C244" s="55" t="s">
         <v>95</v>
@@ -37305,17 +37399,17 @@
         <v>678</v>
       </c>
       <c r="P244" s="86" t="s">
-        <v>1264</v>
+        <v>1258</v>
       </c>
       <c r="S244" s="47"/>
       <c r="T244" s="47"/>
     </row>
     <row r="245" spans="1:20" ht="16">
       <c r="A245" s="52" t="s">
-        <v>1245</v>
+        <v>1239</v>
       </c>
       <c r="B245" s="52" t="s">
-        <v>1254</v>
+        <v>1248</v>
       </c>
       <c r="C245" s="52" t="s">
         <v>95</v>
@@ -37359,10 +37453,10 @@
     </row>
     <row r="246" spans="1:20" ht="17">
       <c r="A246" s="55" t="s">
-        <v>1246</v>
+        <v>1240</v>
       </c>
       <c r="B246" s="55" t="s">
-        <v>1255</v>
+        <v>1249</v>
       </c>
       <c r="C246" s="55" t="s">
         <v>95</v>
@@ -37401,17 +37495,17 @@
         <v>504</v>
       </c>
       <c r="P246" s="86" t="s">
-        <v>1265</v>
+        <v>1259</v>
       </c>
       <c r="S246" s="47"/>
       <c r="T246" s="47"/>
     </row>
     <row r="247" spans="1:20" ht="16">
       <c r="A247" s="52" t="s">
-        <v>1247</v>
+        <v>1241</v>
       </c>
       <c r="B247" s="52" t="s">
-        <v>1256</v>
+        <v>1250</v>
       </c>
       <c r="C247" s="52" t="s">
         <v>95</v>
@@ -37455,10 +37549,10 @@
     </row>
     <row r="248" spans="1:20" ht="17">
       <c r="A248" s="55" t="s">
-        <v>1248</v>
+        <v>1242</v>
       </c>
       <c r="B248" s="55" t="s">
-        <v>1257</v>
+        <v>1251</v>
       </c>
       <c r="C248" s="55" t="s">
         <v>95</v>
@@ -37497,7 +37591,7 @@
         <v>678</v>
       </c>
       <c r="P248" s="86" t="s">
-        <v>1266</v>
+        <v>1260</v>
       </c>
       <c r="S248" s="47"/>
       <c r="T248" s="47"/>
@@ -43674,7 +43768,7 @@
   <sheetData>
     <row r="1" spans="1:8" ht="15" customHeight="1">
       <c r="A1" s="88" t="s">
-        <v>1045</v>
+        <v>1043</v>
       </c>
       <c r="B1" s="88"/>
     </row>
@@ -43683,7 +43777,7 @@
         <v>42</v>
       </c>
       <c r="B2" s="8" t="s">
-        <v>1046</v>
+        <v>1044</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="13.5" customHeight="1">
@@ -43715,25 +43809,25 @@
         <v>42</v>
       </c>
       <c r="B7" s="71" t="s">
+        <v>1045</v>
+      </c>
+      <c r="C7" s="71" t="s">
+        <v>1046</v>
+      </c>
+      <c r="D7" s="71" t="s">
         <v>1047</v>
       </c>
-      <c r="C7" s="71" t="s">
+      <c r="E7" s="71" t="s">
         <v>1048</v>
       </c>
-      <c r="D7" s="71" t="s">
+      <c r="F7" s="71" t="s">
         <v>1049</v>
       </c>
-      <c r="E7" s="71" t="s">
+      <c r="G7" s="71" t="s">
         <v>1050</v>
       </c>
-      <c r="F7" s="71" t="s">
+      <c r="H7" s="71" t="s">
         <v>1051</v>
-      </c>
-      <c r="G7" s="71" t="s">
-        <v>1052</v>
-      </c>
-      <c r="H7" s="71" t="s">
-        <v>1053</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="13.5" customHeight="1">
@@ -43837,7 +43931,7 @@
     </row>
     <row r="12" spans="1:8" s="75" customFormat="1" ht="15.75" customHeight="1">
       <c r="A12" s="89" t="s">
-        <v>1054</v>
+        <v>1052</v>
       </c>
       <c r="B12" s="89"/>
       <c r="C12" s="89"/>
@@ -43850,13 +43944,13 @@
         <v>98</v>
       </c>
       <c r="B13" s="71" t="s">
+        <v>1053</v>
+      </c>
+      <c r="C13" s="71" t="s">
+        <v>1054</v>
+      </c>
+      <c r="D13" s="71" t="s">
         <v>1055</v>
-      </c>
-      <c r="C13" s="71" t="s">
-        <v>1056</v>
-      </c>
-      <c r="D13" s="71" t="s">
-        <v>1057</v>
       </c>
       <c r="E13" s="71" t="s">
         <v>99</v>
@@ -43870,7 +43964,7 @@
         <v>45952</v>
       </c>
       <c r="B14" s="9" t="s">
-        <v>1058</v>
+        <v>1056</v>
       </c>
       <c r="C14" s="9" t="s">
         <v>51</v>
@@ -43888,7 +43982,7 @@
         <v>45952</v>
       </c>
       <c r="B15" s="11" t="s">
-        <v>1058</v>
+        <v>1056</v>
       </c>
       <c r="C15" s="11" t="s">
         <v>51</v>
@@ -43942,7 +44036,7 @@
         <v>45970</v>
       </c>
       <c r="B18" s="9" t="s">
-        <v>1058</v>
+        <v>1056</v>
       </c>
       <c r="C18" s="9" t="s">
         <v>50</v>
@@ -43960,7 +44054,7 @@
         <v>45970</v>
       </c>
       <c r="B19" s="11" t="s">
-        <v>1058</v>
+        <v>1056</v>
       </c>
       <c r="C19" s="11" t="s">
         <v>50</v>
@@ -43978,7 +44072,7 @@
         <v>45973</v>
       </c>
       <c r="B20" s="9" t="s">
-        <v>1058</v>
+        <v>1056</v>
       </c>
       <c r="C20" s="9" t="s">
         <v>50</v>
@@ -43996,7 +44090,7 @@
         <v>45973</v>
       </c>
       <c r="B21" s="11" t="s">
-        <v>1058</v>
+        <v>1056</v>
       </c>
       <c r="C21" s="11" t="s">
         <v>49</v>
@@ -44014,7 +44108,7 @@
         <v>46058</v>
       </c>
       <c r="B22" s="9" t="s">
-        <v>1058</v>
+        <v>1056</v>
       </c>
       <c r="C22" s="9" t="s">
         <v>51</v>
@@ -44050,7 +44144,7 @@
         <v>46059</v>
       </c>
       <c r="B24" s="9" t="s">
-        <v>1058</v>
+        <v>1056</v>
       </c>
       <c r="C24" s="9" t="s">
         <v>49</v>
@@ -44086,7 +44180,7 @@
         <v>46093</v>
       </c>
       <c r="B26" s="9" t="s">
-        <v>1058</v>
+        <v>1056</v>
       </c>
       <c r="C26" s="9" t="s">
         <v>50</v>
@@ -44104,7 +44198,7 @@
         <v>46093</v>
       </c>
       <c r="B27" s="11" t="s">
-        <v>1058</v>
+        <v>1056</v>
       </c>
       <c r="C27" s="11" t="s">
         <v>51</v>
@@ -44187,7 +44281,7 @@
     </row>
     <row r="58" spans="2:2" ht="13.5" customHeight="1">
       <c r="B58" s="6" t="s">
-        <v>1059</v>
+        <v>1057</v>
       </c>
     </row>
   </sheetData>
@@ -44217,7 +44311,7 @@
   <sheetData>
     <row r="1" spans="1:7" ht="13.5" customHeight="1">
       <c r="A1" s="78" t="s">
-        <v>1060</v>
+        <v>1058</v>
       </c>
     </row>
     <row r="3" spans="1:7" s="72" customFormat="1" ht="13.5" customHeight="1">
@@ -44225,22 +44319,22 @@
         <v>42</v>
       </c>
       <c r="B3" s="71" t="s">
+        <v>1059</v>
+      </c>
+      <c r="C3" s="71" t="s">
+        <v>1044</v>
+      </c>
+      <c r="D3" s="71" t="s">
+        <v>1060</v>
+      </c>
+      <c r="E3" s="71" t="s">
         <v>1061</v>
       </c>
-      <c r="C3" s="71" t="s">
-        <v>1046</v>
-      </c>
-      <c r="D3" s="71" t="s">
+      <c r="F3" s="71" t="s">
         <v>1062</v>
       </c>
-      <c r="E3" s="71" t="s">
+      <c r="G3" s="71" t="s">
         <v>1063</v>
-      </c>
-      <c r="F3" s="71" t="s">
-        <v>1064</v>
-      </c>
-      <c r="G3" s="71" t="s">
-        <v>1065</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="13.5" customHeight="1">
@@ -44249,7 +44343,7 @@
       </c>
       <c r="B4" s="9">
         <f>IFERROR(SUMIFS(Sales!$C:$C,Sales!$E:$E,$A4,Sales!$I:$I,"Completed"),0)</f>
-        <v>469208</v>
+        <v>472938</v>
       </c>
       <c r="C4" s="9">
         <f>VLOOKUP($A4,PartnerShares!$A$3:$B$5,2,FALSE())</f>
@@ -44257,11 +44351,11 @@
       </c>
       <c r="D4" s="9">
         <f>Summary!$B$4*C4</f>
-        <v>179156.4908</v>
+        <v>180400.07279999999</v>
       </c>
       <c r="E4" s="9">
         <f>B4-D4</f>
-        <v>290051.50919999997</v>
+        <v>292537.92720000003</v>
       </c>
       <c r="F4" s="9">
         <f>IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$D$13:$D$499,$A4,PartnerShares!$B$13:$B$499,"Cash"),0)-IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$C$13:$C$499,$A4,PartnerShares!$B$13:$B$499,"Cash"),0)</f>
@@ -44269,7 +44363,7 @@
       </c>
       <c r="G4" s="73">
         <f>E4+F4</f>
-        <v>152741.48319999996</v>
+        <v>155227.90120000002</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="13.5" customHeight="1">
@@ -44286,11 +44380,11 @@
       </c>
       <c r="D5" s="11">
         <f>Summary!$B$4*C5</f>
-        <v>179049.0184</v>
+        <v>180291.85440000001</v>
       </c>
       <c r="E5" s="11">
         <f>B5-D5</f>
-        <v>-124425.0184</v>
+        <v>-125667.85440000001</v>
       </c>
       <c r="F5" s="11">
         <f>IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$D$13:$D$499,$A5,PartnerShares!$B$13:$B$499,"Cash"),0)-IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$C$13:$C$499,$A5,PartnerShares!$B$13:$B$499,"Cash"),0)</f>
@@ -44298,7 +44392,7 @@
       </c>
       <c r="G5" s="74">
         <f>E5+F5</f>
-        <v>-52837.9764</v>
+        <v>-54080.81240000001</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="13.5" customHeight="1">
@@ -44315,11 +44409,11 @@
       </c>
       <c r="D6" s="9">
         <f>Summary!$B$4*C6</f>
-        <v>179156.4908</v>
+        <v>180400.07279999999</v>
       </c>
       <c r="E6" s="9">
         <f>B6-D6</f>
-        <v>-166626.4908</v>
+        <v>-167870.07279999999</v>
       </c>
       <c r="F6" s="9">
         <f>IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$D$13:$D$499,$A6,PartnerShares!$B$13:$B$499,"Cash"),0)-IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$C$13:$C$499,$A6,PartnerShares!$B$13:$B$499,"Cash"),0)</f>
@@ -44327,7 +44421,7 @@
       </c>
       <c r="G6" s="73">
         <f>E6+F6</f>
-        <v>-100903.50679999999</v>
+        <v>-102147.08879999998</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="13.5" customHeight="1">
@@ -44337,27 +44431,27 @@
     </row>
     <row r="10" spans="1:7" ht="13.5" customHeight="1">
       <c r="A10" s="6" t="s">
-        <v>1066</v>
+        <v>1064</v>
       </c>
     </row>
     <row r="11" spans="1:7" ht="13.5" customHeight="1">
       <c r="A11" s="6" t="s">
-        <v>1067</v>
+        <v>1065</v>
       </c>
     </row>
     <row r="12" spans="1:7" ht="13.5" customHeight="1">
       <c r="A12" s="6" t="s">
-        <v>1068</v>
+        <v>1066</v>
       </c>
     </row>
     <row r="13" spans="1:7" ht="13.5" customHeight="1">
       <c r="A13" s="6" t="s">
-        <v>1069</v>
+        <v>1067</v>
       </c>
     </row>
     <row r="14" spans="1:7" ht="13.5" customHeight="1">
       <c r="A14" s="6" t="s">
-        <v>1070</v>
+        <v>1068</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Kuthanpully purchases, Komappa purchases, Sales - Onam week
</commit_message>
<xml_diff>
--- a/docs/Chiraath-Summary-Aug26.xlsx
+++ b/docs/Chiraath-Summary-Aug26.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/anooppremachandran/Desktop/CHIRAATH/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63805685-D5E2-F64D-8AAE-58F5C469B1FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CAD0F0D8-6843-AD42-B565-17AC8A3C5383}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" tabRatio="500" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3381" uniqueCount="1339">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3418" uniqueCount="1355">
   <si>
     <t>Notes:</t>
   </si>
@@ -4080,6 +4080,54 @@
   </si>
   <si>
     <t>Hima B S</t>
+  </si>
+  <si>
+    <t>Kuthanpully</t>
+  </si>
+  <si>
+    <t>CHR-249</t>
+  </si>
+  <si>
+    <t>CHR-250</t>
+  </si>
+  <si>
+    <t>Purple with silver zari</t>
+  </si>
+  <si>
+    <t>Peacock blue/Royal blue, Purple/Pink, Lime Green/Wine Purple</t>
+  </si>
+  <si>
+    <t>426363 Churidar Set</t>
+  </si>
+  <si>
+    <t>L, XL, XXL</t>
+  </si>
+  <si>
+    <t>CHR-251</t>
+  </si>
+  <si>
+    <t>425677 Churidar Set</t>
+  </si>
+  <si>
+    <t>M, L, XL, XXL</t>
+  </si>
+  <si>
+    <t>CHR-252</t>
+  </si>
+  <si>
+    <t>417278 Churidar Set</t>
+  </si>
+  <si>
+    <t>CHR-253</t>
+  </si>
+  <si>
+    <t>424938 Churidar Set</t>
+  </si>
+  <si>
+    <t>Soft Silk Saree Collection (Kuthanpully)</t>
+  </si>
+  <si>
+    <t>Semi Silk (Kuthanpully)</t>
   </si>
 </sst>
 </file>
@@ -4091,7 +4139,7 @@
     <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd;@"/>
     <numFmt numFmtId="166" formatCode="m/d/yyyy"/>
   </numFmts>
-  <fonts count="32">
+  <fonts count="33">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -4322,6 +4370,13 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
     </font>
+    <font>
+      <strike/>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="9">
     <fill>
@@ -4437,7 +4492,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="90">
+  <cellXfs count="95">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -4677,6 +4732,21 @@
     </xf>
     <xf numFmtId="0" fontId="29" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -5068,10 +5138,10 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>173</c:v>
+                  <c:v>177</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>51</c:v>
+                  <c:v>65</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>3</c:v>
@@ -5398,10 +5468,10 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>53945</c:v>
+                  <c:v>69573</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>122683.14666666667</c:v>
+                  <c:v>125729.14666666667</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>1062</c:v>
@@ -5737,7 +5807,7 @@
                   <c:v>102200</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>10461</c:v>
+                  <c:v>45517</c:v>
                 </c:pt>
                 <c:pt idx="8">
                   <c:v>0</c:v>
@@ -5897,7 +5967,7 @@
                   <c:v>63906</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>72908</c:v>
+                  <c:v>72808</c:v>
                 </c:pt>
                 <c:pt idx="8">
                   <c:v>0</c:v>
@@ -6337,7 +6407,7 @@
                   <c:v>-38294</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>62447</c:v>
+                  <c:v>27291</c:v>
                 </c:pt>
                 <c:pt idx="8">
                   <c:v>0</c:v>
@@ -7958,7 +8028,7 @@
     <col min="4" max="4" width="30.1640625" style="6" customWidth="1"/>
     <col min="5" max="5" width="22.1640625" style="6" customWidth="1"/>
     <col min="6" max="6" width="31.1640625" style="6" customWidth="1"/>
-    <col min="7" max="7" width="14.6640625" style="6" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.6640625" style="6" bestFit="1" customWidth="1"/>
     <col min="8" max="16384" width="8.83203125" style="6"/>
   </cols>
   <sheetData>
@@ -7973,7 +8043,7 @@
       </c>
       <c r="B3" s="8">
         <f>SUM(Purchases!C:C)</f>
-        <v>566808</v>
+        <v>601864</v>
       </c>
       <c r="E3" s="8" t="s">
         <v>42</v>
@@ -7988,7 +8058,7 @@
       </c>
       <c r="B4" s="10">
         <f>SUMIFS(Sales!C:C, Sales!I:I, "Completed")</f>
-        <v>541092</v>
+        <v>544692</v>
       </c>
       <c r="E4" s="9" t="str">
         <f>PartnerShares!A3</f>
@@ -8005,7 +8075,7 @@
       </c>
       <c r="B5" s="12">
         <f>SUM(Sales!C:C)</f>
-        <v>565312</v>
+        <v>565212</v>
       </c>
       <c r="E5" s="11" t="str">
         <f>PartnerShares!A4</f>
@@ -8022,7 +8092,7 @@
       </c>
       <c r="B6" s="10">
         <f>B4-B3</f>
-        <v>-25716</v>
+        <v>-57172</v>
       </c>
       <c r="E6" s="9" t="str">
         <f>PartnerShares!A5</f>
@@ -8057,7 +8127,7 @@
       </c>
       <c r="B10" s="13">
         <f>PartnerShares!H8</f>
-        <v>55651.66</v>
+        <v>44016.32666666666</v>
       </c>
       <c r="C10" s="9"/>
     </row>
@@ -8067,7 +8137,7 @@
       </c>
       <c r="B11" s="14">
         <f>PartnerShares!H9</f>
-        <v>40741.67</v>
+        <v>64062.336666666655</v>
       </c>
       <c r="C11" s="11"/>
     </row>
@@ -8077,7 +8147,7 @@
       </c>
       <c r="B12" s="13">
         <f>PartnerShares!H10</f>
-        <v>-96393.33</v>
+        <v>-108078.66333333334</v>
       </c>
       <c r="C12" s="9"/>
     </row>
@@ -8116,15 +8186,15 @@
       </c>
       <c r="B18" s="10">
         <f>PartnerShares!B8</f>
-        <v>262891</v>
+        <v>262941</v>
       </c>
       <c r="C18" s="10">
         <f>PartnerShares!C8</f>
-        <v>188936</v>
+        <v>200621.33333333334</v>
       </c>
       <c r="D18" s="10">
         <f>PartnerShares!D8</f>
-        <v>73955</v>
+        <v>62319.666666666657</v>
       </c>
       <c r="E18" s="10">
         <f>IFERROR(SUMIFS(PartnerShares!$E$14:$E$500,PartnerShares!$D$14:$D$500,$A18,PartnerShares!$B$14:$B$500,"Contribution"),0)-IFERROR(SUMIFS(PartnerShares!$E$14:$E$500,PartnerShares!$C$14:$C$500,$A18,PartnerShares!$B$14:$B$500,"Contribution"),0)</f>
@@ -8132,11 +8202,11 @@
       </c>
       <c r="F18" s="13">
         <f>D18-E18</f>
-        <v>55651.66</v>
+        <v>44016.32666666666</v>
       </c>
       <c r="G18" s="16" t="str">
         <f>IF(ROUND(F18,0)&gt;0,"Receive ₹"&amp;TEXT(ABS(F18),"#,##0"),IF(ROUND(F18,0)&lt;0,"Pay ₹"&amp;TEXT(ABS(F18),"#,##0"),"✓ Settled"))</f>
-        <v>Receive ₹55,652</v>
+        <v>Receive ₹44,016</v>
       </c>
     </row>
     <row r="19" spans="1:7" ht="13.5" customHeight="1">
@@ -8146,15 +8216,15 @@
       </c>
       <c r="B19" s="12">
         <f>PartnerShares!B9</f>
-        <v>271317</v>
+        <v>306323</v>
       </c>
       <c r="C19" s="12">
         <f>PartnerShares!C9</f>
-        <v>188936</v>
+        <v>200621.33333333334</v>
       </c>
       <c r="D19" s="12">
         <f>PartnerShares!D9</f>
-        <v>82381</v>
+        <v>105701.66666666666</v>
       </c>
       <c r="E19" s="12">
         <f>IFERROR(SUMIFS(PartnerShares!$E$14:$E$500,PartnerShares!$D$14:$D$500,$A19,PartnerShares!$B$14:$B$500,"Contribution"),0)-IFERROR(SUMIFS(PartnerShares!$E$14:$E$500,PartnerShares!$C$14:$C$500,$A19,PartnerShares!$B$14:$B$500,"Contribution"),0)</f>
@@ -8162,11 +8232,11 @@
       </c>
       <c r="F19" s="14">
         <f>D19-E19</f>
-        <v>40741.67</v>
+        <v>64062.336666666655</v>
       </c>
       <c r="G19" s="17" t="str">
         <f>IF(ROUND(F19,0)&gt;0,"Receive ₹"&amp;TEXT(ABS(F19),"#,##0"),IF(ROUND(F19,0)&lt;0,"Pay ₹"&amp;TEXT(ABS(F19),"#,##0"),"✓ Settled"))</f>
-        <v>Receive ₹40,742</v>
+        <v>Receive ₹64,062</v>
       </c>
     </row>
     <row r="20" spans="1:7" ht="13.5" customHeight="1">
@@ -8180,11 +8250,11 @@
       </c>
       <c r="C20" s="10">
         <f>PartnerShares!C10</f>
-        <v>188936</v>
+        <v>200621.33333333334</v>
       </c>
       <c r="D20" s="10">
         <f>PartnerShares!D10</f>
-        <v>-156336</v>
+        <v>-168021.33333333334</v>
       </c>
       <c r="E20" s="10">
         <f>IFERROR(SUMIFS(PartnerShares!$E$14:$E$500,PartnerShares!$D$14:$D$500,$A20,PartnerShares!$B$14:$B$500,"Contribution"),0)-IFERROR(SUMIFS(PartnerShares!$E$14:$E$500,PartnerShares!$C$14:$C$500,$A20,PartnerShares!$B$14:$B$500,"Contribution"),0)</f>
@@ -8192,11 +8262,11 @@
       </c>
       <c r="F20" s="13">
         <f>D20-E20</f>
-        <v>-96393.33</v>
+        <v>-108078.66333333334</v>
       </c>
       <c r="G20" s="17" t="str">
         <f>IF(ROUND(F20,0)&gt;0,"Receive ₹"&amp;TEXT(ABS(F20),"#,##0"),IF(ROUND(F20,0)&lt;0,"Pay ₹"&amp;TEXT(ABS(F20),"#,##0"),"✓ Settled"))</f>
-        <v>Pay ₹96,393</v>
+        <v>Pay ₹108,079</v>
       </c>
     </row>
     <row r="24" spans="1:7" ht="15.75" customHeight="1">
@@ -8234,15 +8304,15 @@
       </c>
       <c r="B26" s="10">
         <f>'Cash Pool'!B4</f>
-        <v>472938</v>
+        <v>476538</v>
       </c>
       <c r="C26" s="10">
         <f>'Cash Pool'!D4</f>
-        <v>180400.07279999999</v>
+        <v>181600.31279999999</v>
       </c>
       <c r="D26" s="10">
         <f>'Cash Pool'!E4</f>
-        <v>292537.92720000003</v>
+        <v>294937.68720000004</v>
       </c>
       <c r="E26" s="10">
         <f>'Cash Pool'!F4</f>
@@ -8250,11 +8320,11 @@
       </c>
       <c r="F26" s="13">
         <f>'Cash Pool'!G4</f>
-        <v>155227.90120000002</v>
+        <v>157627.66120000003</v>
       </c>
       <c r="G26" s="17" t="str">
         <f>IF(ROUND(F26,0)&gt;0,"Pay ₹"&amp;TEXT(ABS(F26),"#,##0"),IF(ROUND(F26,0)&lt;0,"Receive ₹"&amp;TEXT(ABS(F26),"#,##0"),"✓ Settled"))</f>
-        <v>Pay ₹155,228</v>
+        <v>Pay ₹157,628</v>
       </c>
     </row>
     <row r="27" spans="1:7" ht="13.5" customHeight="1">
@@ -8268,11 +8338,11 @@
       </c>
       <c r="C27" s="12">
         <f>'Cash Pool'!D5</f>
-        <v>180291.85440000001</v>
+        <v>181491.3744</v>
       </c>
       <c r="D27" s="12">
         <f>'Cash Pool'!E5</f>
-        <v>-125667.85440000001</v>
+        <v>-126867.3744</v>
       </c>
       <c r="E27" s="12">
         <f>'Cash Pool'!F5</f>
@@ -8280,11 +8350,11 @@
       </c>
       <c r="F27" s="14">
         <f>'Cash Pool'!G5</f>
-        <v>-54080.81240000001</v>
+        <v>-55280.332399999999</v>
       </c>
       <c r="G27" s="18" t="str">
         <f>IF(ROUND(F27,0)&gt;0,"Pay ₹"&amp;TEXT(ABS(F27),"#,##0"),IF(ROUND(F27,0)&lt;0,"Receive ₹"&amp;TEXT(ABS(F27),"#,##0"),"✓ Settled"))</f>
-        <v>Receive ₹54,081</v>
+        <v>Receive ₹55,280</v>
       </c>
     </row>
     <row r="28" spans="1:7" ht="13.5" customHeight="1">
@@ -8298,11 +8368,11 @@
       </c>
       <c r="C28" s="10">
         <f>'Cash Pool'!D6</f>
-        <v>180400.07279999999</v>
+        <v>181600.31279999999</v>
       </c>
       <c r="D28" s="10">
         <f>'Cash Pool'!E6</f>
-        <v>-167870.07279999999</v>
+        <v>-169070.31279999999</v>
       </c>
       <c r="E28" s="10">
         <f>'Cash Pool'!F6</f>
@@ -8310,11 +8380,11 @@
       </c>
       <c r="F28" s="13">
         <f>'Cash Pool'!G6</f>
-        <v>-102147.08879999998</v>
+        <v>-103347.32879999997</v>
       </c>
       <c r="G28" s="16" t="str">
         <f>IF(ROUND(F28,0)&gt;0,"Pay ₹"&amp;TEXT(ABS(F28),"#,##0"),IF(ROUND(F28,0)&lt;0,"Receive ₹"&amp;TEXT(ABS(F28),"#,##0"),"✓ Settled"))</f>
-        <v>Receive ₹102,147</v>
+        <v>Receive ₹103,347</v>
       </c>
     </row>
     <row r="32" spans="1:7" ht="15.75" customHeight="1">
@@ -8426,7 +8496,7 @@
       </c>
       <c r="B3" s="20">
         <f ca="1">TODAY()</f>
-        <v>46261</v>
+        <v>46263</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="15" customHeight="1">
@@ -8435,14 +8505,14 @@
       </c>
       <c r="B5" s="21">
         <f>Summary!B3</f>
-        <v>566808</v>
+        <v>601864</v>
       </c>
       <c r="D5" s="19" t="s">
         <v>69</v>
       </c>
       <c r="E5" s="21">
         <f>Summary!B4</f>
-        <v>541092</v>
+        <v>544692</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="15" customHeight="1">
@@ -8451,14 +8521,14 @@
       </c>
       <c r="B6" s="21">
         <f>Summary!B6</f>
-        <v>-25716</v>
+        <v>-57172</v>
       </c>
       <c r="D6" s="19" t="s">
         <v>71</v>
       </c>
       <c r="E6" s="21">
         <f>SUMIFS(INVENTORY!K:K, INVENTORY!N:N, "&lt;&gt;Sold Out")</f>
-        <v>168031.34666666665</v>
+        <v>186705.34666666665</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="15.75" customHeight="1">
@@ -8628,15 +8698,15 @@
       </c>
       <c r="B17" s="27">
         <f>IFERROR(SUMPRODUCT((TEXT(Purchases!$A$2:$A$998,"MMM")=$A17)*(YEAR(Purchases!$A$2:$A$998)=$B$7)*Purchases!$C$2:$C$998),0)</f>
-        <v>10461</v>
+        <v>45517</v>
       </c>
       <c r="C17" s="27">
         <f>IFERROR(SUMPRODUCT((TEXT(Sales!$A$2:$A$993,"MMM")=$A17)*(YEAR(Sales!$A$2:$A$993)=$B$7)*Sales!$C$2:$C$993),0)</f>
-        <v>72908</v>
+        <v>72808</v>
       </c>
       <c r="D17" s="27">
         <f t="shared" si="0"/>
-        <v>62447</v>
+        <v>27291</v>
       </c>
     </row>
     <row r="18" spans="1:4" ht="15" customHeight="1">
@@ -8734,14 +8804,14 @@
       </c>
       <c r="H47" s="30">
         <f>SUMIF(INVENTORY!C:C, F47, INVENTORY!G:G)</f>
-        <v>173</v>
+        <v>177</v>
       </c>
       <c r="J47" s="30" t="s">
         <v>96</v>
       </c>
       <c r="K47" s="31">
         <f t="array" ref="K47">SUMPRODUCT((INVENTORY!$C$2:$C$476=J47)*(INVENTORY!$D$2:$D$476)*(INVENTORY!$G$2:$G$476))</f>
-        <v>53945</v>
+        <v>69573</v>
       </c>
     </row>
     <row r="48" spans="6:11" ht="15" customHeight="1">
@@ -8754,14 +8824,14 @@
       </c>
       <c r="H48" s="30">
         <f>SUMIF(INVENTORY!C:C, F48, INVENTORY!G:G)</f>
-        <v>51</v>
+        <v>65</v>
       </c>
       <c r="J48" s="30" t="s">
         <v>95</v>
       </c>
       <c r="K48" s="31">
         <f t="array" ref="K48">SUMPRODUCT((INVENTORY!$C$2:$C$476=J48)*(INVENTORY!$D$2:$D$476)*(INVENTORY!$G$2:$G$476))</f>
-        <v>122683.14666666667</v>
+        <v>125729.14666666667</v>
       </c>
     </row>
     <row r="49" spans="5:12" ht="15" customHeight="1">
@@ -10390,22 +10460,46 @@
       </c>
     </row>
     <row r="110" spans="1:4" ht="15" customHeight="1">
-      <c r="A110" s="35"/>
-      <c r="B110" s="36"/>
-      <c r="C110" s="37"/>
-      <c r="D110" s="36"/>
+      <c r="A110" s="35">
+        <v>46259</v>
+      </c>
+      <c r="B110" s="36" t="s">
+        <v>50</v>
+      </c>
+      <c r="C110" s="37">
+        <v>3046</v>
+      </c>
+      <c r="D110" s="36" t="s">
+        <v>1339</v>
+      </c>
     </row>
     <row r="111" spans="1:4" ht="15" customHeight="1">
-      <c r="A111" s="38"/>
-      <c r="B111" s="39"/>
-      <c r="C111" s="40"/>
-      <c r="D111" s="39"/>
+      <c r="A111" s="38">
+        <v>46262</v>
+      </c>
+      <c r="B111" s="39" t="s">
+        <v>49</v>
+      </c>
+      <c r="C111" s="40">
+        <v>50</v>
+      </c>
+      <c r="D111" s="39" t="s">
+        <v>119</v>
+      </c>
     </row>
     <row r="112" spans="1:4" ht="15" customHeight="1">
-      <c r="A112" s="35"/>
-      <c r="B112" s="36"/>
-      <c r="C112" s="37"/>
-      <c r="D112" s="36"/>
+      <c r="A112" s="35">
+        <v>46262</v>
+      </c>
+      <c r="B112" s="36" t="s">
+        <v>50</v>
+      </c>
+      <c r="C112" s="37">
+        <v>31960</v>
+      </c>
+      <c r="D112" s="36" t="s">
+        <v>118</v>
+      </c>
     </row>
     <row r="113" spans="1:4" ht="15" customHeight="1">
       <c r="A113" s="38"/>
@@ -20291,19 +20385,21 @@
         <v>175</v>
       </c>
       <c r="C319" s="85">
-        <v>2200</v>
+        <v>2100</v>
       </c>
       <c r="D319" s="45" t="s">
         <v>162</v>
       </c>
-      <c r="E319" s="45"/>
+      <c r="E319" s="45" t="s">
+        <v>49</v>
+      </c>
       <c r="F319" s="46"/>
       <c r="G319" s="46"/>
       <c r="H319" s="46" t="s">
         <v>1323</v>
       </c>
       <c r="I319" s="45" t="s">
-        <v>356</v>
+        <v>148</v>
       </c>
     </row>
     <row r="320" spans="1:9" ht="14">
@@ -20353,7 +20449,7 @@
         <v>1333</v>
       </c>
       <c r="I321" s="45" t="s">
-        <v>356</v>
+        <v>148</v>
       </c>
     </row>
     <row r="322" spans="1:9" ht="14">
@@ -37202,7 +37298,7 @@
       <c r="S240" s="47"/>
       <c r="T240" s="47"/>
     </row>
-    <row r="241" spans="1:20" ht="17">
+    <row r="241" spans="1:246" ht="17">
       <c r="A241" s="52" t="s">
         <v>1235</v>
       </c>
@@ -37253,7 +37349,7 @@
       <c r="S241" s="47"/>
       <c r="T241" s="47"/>
     </row>
-    <row r="242" spans="1:20" ht="17">
+    <row r="242" spans="1:246" ht="17">
       <c r="A242" s="55" t="s">
         <v>1236</v>
       </c>
@@ -37304,7 +37400,7 @@
       <c r="S242" s="47"/>
       <c r="T242" s="47"/>
     </row>
-    <row r="243" spans="1:20" ht="17">
+    <row r="243" spans="1:246" ht="17">
       <c r="A243" s="52" t="s">
         <v>1237</v>
       </c>
@@ -37355,7 +37451,7 @@
       <c r="S243" s="47"/>
       <c r="T243" s="47"/>
     </row>
-    <row r="244" spans="1:20" ht="17">
+    <row r="244" spans="1:246" ht="17">
       <c r="A244" s="55" t="s">
         <v>1238</v>
       </c>
@@ -37404,7 +37500,7 @@
       <c r="S244" s="47"/>
       <c r="T244" s="47"/>
     </row>
-    <row r="245" spans="1:20" ht="16">
+    <row r="245" spans="1:246" ht="16">
       <c r="A245" s="52" t="s">
         <v>1239</v>
       </c>
@@ -37451,58 +37547,282 @@
       <c r="S245" s="47"/>
       <c r="T245" s="47"/>
     </row>
-    <row r="246" spans="1:20" ht="17">
-      <c r="A246" s="55" t="s">
+    <row r="246" spans="1:246" s="62" customFormat="1" ht="17">
+      <c r="A246" s="90" t="s">
         <v>1240</v>
       </c>
-      <c r="B246" s="55" t="s">
+      <c r="B246" s="90" t="s">
         <v>1249</v>
       </c>
-      <c r="C246" s="55" t="s">
+      <c r="C246" s="90" t="s">
         <v>95</v>
       </c>
-      <c r="D246" s="56">
+      <c r="D246" s="91">
         <v>629</v>
       </c>
-      <c r="E246" s="56"/>
-      <c r="F246" s="64">
+      <c r="E246" s="91"/>
+      <c r="F246" s="92">
         <v>0</v>
       </c>
-      <c r="G246" s="64">
+      <c r="G246" s="92">
         <v>0</v>
       </c>
-      <c r="H246" s="63">
+      <c r="H246" s="93">
         <f t="shared" si="18"/>
         <v>0</v>
       </c>
-      <c r="I246" s="63">
+      <c r="I246" s="93">
         <f>IF(D246&lt;&gt;"",D246,IFERROR(E246/(IFERROR(SUM(Sales!C:C),0))*(IFERROR(SUM(Purchases!C:C),0)),0))</f>
         <v>629</v>
       </c>
-      <c r="J246" s="63">
+      <c r="J246" s="93">
         <f t="shared" si="19"/>
         <v>0</v>
       </c>
-      <c r="K246" s="63">
+      <c r="K246" s="93">
         <f t="shared" si="20"/>
         <v>0</v>
       </c>
-      <c r="L246" s="55" t="s">
+      <c r="L246" s="90" t="s">
         <v>608</v>
       </c>
-      <c r="M246" s="55"/>
-      <c r="N246" s="47" t="s">
+      <c r="M246" s="90"/>
+      <c r="N246" s="62" t="s">
         <v>504</v>
       </c>
-      <c r="P246" s="86" t="s">
+      <c r="P246" s="94" t="s">
         <v>1259</v>
       </c>
-      <c r="S246" s="47"/>
-      <c r="T246" s="47"/>
-    </row>
-    <row r="247" spans="1:20" ht="16">
+      <c r="U246" s="61"/>
+      <c r="V246" s="61"/>
+      <c r="W246" s="61"/>
+      <c r="X246" s="61"/>
+      <c r="Y246" s="61"/>
+      <c r="Z246" s="61"/>
+      <c r="AA246" s="61"/>
+      <c r="AB246" s="61"/>
+      <c r="AC246" s="61"/>
+      <c r="AD246" s="61"/>
+      <c r="AE246" s="61"/>
+      <c r="AF246" s="61"/>
+      <c r="AG246" s="61"/>
+      <c r="AH246" s="61"/>
+      <c r="AI246" s="61"/>
+      <c r="AJ246" s="61"/>
+      <c r="AK246" s="61"/>
+      <c r="AL246" s="61"/>
+      <c r="AM246" s="61"/>
+      <c r="AN246" s="61"/>
+      <c r="AO246" s="61"/>
+      <c r="AP246" s="61"/>
+      <c r="AQ246" s="61"/>
+      <c r="AR246" s="61"/>
+      <c r="AS246" s="61"/>
+      <c r="AT246" s="61"/>
+      <c r="AU246" s="61"/>
+      <c r="AV246" s="61"/>
+      <c r="AW246" s="61"/>
+      <c r="AX246" s="61"/>
+      <c r="AY246" s="61"/>
+      <c r="AZ246" s="61"/>
+      <c r="BA246" s="61"/>
+      <c r="BB246" s="61"/>
+      <c r="BC246" s="61"/>
+      <c r="BD246" s="61"/>
+      <c r="BE246" s="61"/>
+      <c r="BF246" s="61"/>
+      <c r="BG246" s="61"/>
+      <c r="BH246" s="61"/>
+      <c r="BI246" s="61"/>
+      <c r="BJ246" s="61"/>
+      <c r="BK246" s="61"/>
+      <c r="BL246" s="61"/>
+      <c r="BM246" s="61"/>
+      <c r="BN246" s="61"/>
+      <c r="BO246" s="61"/>
+      <c r="BP246" s="61"/>
+      <c r="BQ246" s="61"/>
+      <c r="BR246" s="61"/>
+      <c r="BS246" s="61"/>
+      <c r="BT246" s="61"/>
+      <c r="BU246" s="61"/>
+      <c r="BV246" s="61"/>
+      <c r="BW246" s="61"/>
+      <c r="BX246" s="61"/>
+      <c r="BY246" s="61"/>
+      <c r="BZ246" s="61"/>
+      <c r="CA246" s="61"/>
+      <c r="CB246" s="61"/>
+      <c r="CC246" s="61"/>
+      <c r="CD246" s="61"/>
+      <c r="CE246" s="61"/>
+      <c r="CF246" s="61"/>
+      <c r="CG246" s="61"/>
+      <c r="CH246" s="61"/>
+      <c r="CI246" s="61"/>
+      <c r="CJ246" s="61"/>
+      <c r="CK246" s="61"/>
+      <c r="CL246" s="61"/>
+      <c r="CM246" s="61"/>
+      <c r="CN246" s="61"/>
+      <c r="CO246" s="61"/>
+      <c r="CP246" s="61"/>
+      <c r="CQ246" s="61"/>
+      <c r="CR246" s="61"/>
+      <c r="CS246" s="61"/>
+      <c r="CT246" s="61"/>
+      <c r="CU246" s="61"/>
+      <c r="CV246" s="61"/>
+      <c r="CW246" s="61"/>
+      <c r="CX246" s="61"/>
+      <c r="CY246" s="61"/>
+      <c r="CZ246" s="61"/>
+      <c r="DA246" s="61"/>
+      <c r="DB246" s="61"/>
+      <c r="DC246" s="61"/>
+      <c r="DD246" s="61"/>
+      <c r="DE246" s="61"/>
+      <c r="DF246" s="61"/>
+      <c r="DG246" s="61"/>
+      <c r="DH246" s="61"/>
+      <c r="DI246" s="61"/>
+      <c r="DJ246" s="61"/>
+      <c r="DK246" s="61"/>
+      <c r="DL246" s="61"/>
+      <c r="DM246" s="61"/>
+      <c r="DN246" s="61"/>
+      <c r="DO246" s="61"/>
+      <c r="DP246" s="61"/>
+      <c r="DQ246" s="61"/>
+      <c r="DR246" s="61"/>
+      <c r="DS246" s="61"/>
+      <c r="DT246" s="61"/>
+      <c r="DU246" s="61"/>
+      <c r="DV246" s="61"/>
+      <c r="DW246" s="61"/>
+      <c r="DX246" s="61"/>
+      <c r="DY246" s="61"/>
+      <c r="DZ246" s="61"/>
+      <c r="EA246" s="61"/>
+      <c r="EB246" s="61"/>
+      <c r="EC246" s="61"/>
+      <c r="ED246" s="61"/>
+      <c r="EE246" s="61"/>
+      <c r="EF246" s="61"/>
+      <c r="EG246" s="61"/>
+      <c r="EH246" s="61"/>
+      <c r="EI246" s="61"/>
+      <c r="EJ246" s="61"/>
+      <c r="EK246" s="61"/>
+      <c r="EL246" s="61"/>
+      <c r="EM246" s="61"/>
+      <c r="EN246" s="61"/>
+      <c r="EO246" s="61"/>
+      <c r="EP246" s="61"/>
+      <c r="EQ246" s="61"/>
+      <c r="ER246" s="61"/>
+      <c r="ES246" s="61"/>
+      <c r="ET246" s="61"/>
+      <c r="EU246" s="61"/>
+      <c r="EV246" s="61"/>
+      <c r="EW246" s="61"/>
+      <c r="EX246" s="61"/>
+      <c r="EY246" s="61"/>
+      <c r="EZ246" s="61"/>
+      <c r="FA246" s="61"/>
+      <c r="FB246" s="61"/>
+      <c r="FC246" s="61"/>
+      <c r="FD246" s="61"/>
+      <c r="FE246" s="61"/>
+      <c r="FF246" s="61"/>
+      <c r="FG246" s="61"/>
+      <c r="FH246" s="61"/>
+      <c r="FI246" s="61"/>
+      <c r="FJ246" s="61"/>
+      <c r="FK246" s="61"/>
+      <c r="FL246" s="61"/>
+      <c r="FM246" s="61"/>
+      <c r="FN246" s="61"/>
+      <c r="FO246" s="61"/>
+      <c r="FP246" s="61"/>
+      <c r="FQ246" s="61"/>
+      <c r="FR246" s="61"/>
+      <c r="FS246" s="61"/>
+      <c r="FT246" s="61"/>
+      <c r="FU246" s="61"/>
+      <c r="FV246" s="61"/>
+      <c r="FW246" s="61"/>
+      <c r="FX246" s="61"/>
+      <c r="FY246" s="61"/>
+      <c r="FZ246" s="61"/>
+      <c r="GA246" s="61"/>
+      <c r="GB246" s="61"/>
+      <c r="GC246" s="61"/>
+      <c r="GD246" s="61"/>
+      <c r="GE246" s="61"/>
+      <c r="GF246" s="61"/>
+      <c r="GG246" s="61"/>
+      <c r="GH246" s="61"/>
+      <c r="GI246" s="61"/>
+      <c r="GJ246" s="61"/>
+      <c r="GK246" s="61"/>
+      <c r="GL246" s="61"/>
+      <c r="GM246" s="61"/>
+      <c r="GN246" s="61"/>
+      <c r="GO246" s="61"/>
+      <c r="GP246" s="61"/>
+      <c r="GQ246" s="61"/>
+      <c r="GR246" s="61"/>
+      <c r="GS246" s="61"/>
+      <c r="GT246" s="61"/>
+      <c r="GU246" s="61"/>
+      <c r="GV246" s="61"/>
+      <c r="GW246" s="61"/>
+      <c r="GX246" s="61"/>
+      <c r="GY246" s="61"/>
+      <c r="GZ246" s="61"/>
+      <c r="HA246" s="61"/>
+      <c r="HB246" s="61"/>
+      <c r="HC246" s="61"/>
+      <c r="HD246" s="61"/>
+      <c r="HE246" s="61"/>
+      <c r="HF246" s="61"/>
+      <c r="HG246" s="61"/>
+      <c r="HH246" s="61"/>
+      <c r="HI246" s="61"/>
+      <c r="HJ246" s="61"/>
+      <c r="HK246" s="61"/>
+      <c r="HL246" s="61"/>
+      <c r="HM246" s="61"/>
+      <c r="HN246" s="61"/>
+      <c r="HO246" s="61"/>
+      <c r="HP246" s="61"/>
+      <c r="HQ246" s="61"/>
+      <c r="HR246" s="61"/>
+      <c r="HS246" s="61"/>
+      <c r="HT246" s="61"/>
+      <c r="HU246" s="61"/>
+      <c r="HV246" s="61"/>
+      <c r="HW246" s="61"/>
+      <c r="HX246" s="61"/>
+      <c r="HY246" s="61"/>
+      <c r="HZ246" s="61"/>
+      <c r="IA246" s="61"/>
+      <c r="IB246" s="61"/>
+      <c r="IC246" s="61"/>
+      <c r="ID246" s="61"/>
+      <c r="IE246" s="61"/>
+      <c r="IF246" s="61"/>
+      <c r="IG246" s="61"/>
+      <c r="IH246" s="61"/>
+      <c r="II246" s="61"/>
+      <c r="IJ246" s="61"/>
+      <c r="IK246" s="61"/>
+      <c r="IL246" s="61"/>
+    </row>
+    <row r="247" spans="1:246" ht="16">
       <c r="A247" s="52" t="s">
-        <v>1241</v>
+        <v>1240</v>
       </c>
       <c r="B247" s="52" t="s">
         <v>1250</v>
@@ -37547,9 +37867,9 @@
       <c r="S247" s="47"/>
       <c r="T247" s="47"/>
     </row>
-    <row r="248" spans="1:20" ht="17">
+    <row r="248" spans="1:246" ht="17">
       <c r="A248" s="55" t="s">
-        <v>1242</v>
+        <v>1241</v>
       </c>
       <c r="B248" s="55" t="s">
         <v>1251</v>
@@ -37596,12 +37916,22 @@
       <c r="S248" s="47"/>
       <c r="T248" s="47"/>
     </row>
-    <row r="249" spans="1:20" ht="16">
-      <c r="A249" s="52"/>
-      <c r="B249" s="52"/>
-      <c r="C249" s="52"/>
-      <c r="D249" s="53"/>
-      <c r="E249" s="53"/>
+    <row r="249" spans="1:246" ht="17">
+      <c r="A249" s="52" t="s">
+        <v>1242</v>
+      </c>
+      <c r="B249" s="52" t="s">
+        <v>1353</v>
+      </c>
+      <c r="C249" s="52" t="s">
+        <v>95</v>
+      </c>
+      <c r="D249" s="53">
+        <v>882</v>
+      </c>
+      <c r="E249" s="53">
+        <v>1380</v>
+      </c>
       <c r="F249" s="66">
         <v>0</v>
       </c>
@@ -37614,7 +37944,7 @@
       </c>
       <c r="I249" s="65">
         <f>IF(D249&lt;&gt;"",D249,IFERROR(E249/(IFERROR(SUM(Sales!C:C),0))*(IFERROR(SUM(Purchases!C:C),0)),0))</f>
-        <v>0</v>
+        <v>882</v>
       </c>
       <c r="J249" s="65">
         <f t="shared" si="19"/>
@@ -37622,33 +37952,48 @@
       </c>
       <c r="K249" s="65">
         <f t="shared" si="20"/>
-        <v>0</v>
+        <v>2646</v>
       </c>
       <c r="L249" s="52"/>
       <c r="M249" s="52"/>
-      <c r="P249" s="86"/>
+      <c r="N249" s="47" t="s">
+        <v>678</v>
+      </c>
+      <c r="P249" s="86" t="s">
+        <v>1343</v>
+      </c>
       <c r="S249" s="47"/>
       <c r="T249" s="47"/>
     </row>
-    <row r="250" spans="1:20" ht="16">
-      <c r="A250" s="55"/>
-      <c r="B250" s="55"/>
-      <c r="C250" s="55"/>
-      <c r="D250" s="56"/>
-      <c r="E250" s="56"/>
+    <row r="250" spans="1:246" ht="17">
+      <c r="A250" s="55" t="s">
+        <v>1340</v>
+      </c>
+      <c r="B250" s="55" t="s">
+        <v>1354</v>
+      </c>
+      <c r="C250" s="55" t="s">
+        <v>95</v>
+      </c>
+      <c r="D250" s="56">
+        <v>400</v>
+      </c>
+      <c r="E250" s="56">
+        <v>699</v>
+      </c>
       <c r="F250" s="64">
         <v>0</v>
       </c>
       <c r="G250" s="64">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H250" s="63">
         <f t="shared" si="18"/>
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I250" s="63">
         <f>IF(D250&lt;&gt;"",D250,IFERROR(E250/(IFERROR(SUM(Sales!C:C),0))*(IFERROR(SUM(Purchases!C:C),0)),0))</f>
-        <v>0</v>
+        <v>400</v>
       </c>
       <c r="J250" s="63">
         <f t="shared" si="19"/>
@@ -37656,19 +38001,32 @@
       </c>
       <c r="K250" s="63">
         <f t="shared" si="20"/>
-        <v>0</v>
+        <v>400</v>
       </c>
       <c r="L250" s="55"/>
       <c r="M250" s="55"/>
-      <c r="P250" s="86"/>
+      <c r="N250" s="47" t="s">
+        <v>678</v>
+      </c>
+      <c r="P250" s="86" t="s">
+        <v>1342</v>
+      </c>
       <c r="S250" s="47"/>
       <c r="T250" s="47"/>
     </row>
-    <row r="251" spans="1:20" ht="16">
-      <c r="A251" s="52"/>
-      <c r="B251" s="52"/>
-      <c r="C251" s="52"/>
-      <c r="D251" s="53"/>
+    <row r="251" spans="1:246" ht="16">
+      <c r="A251" s="52" t="s">
+        <v>1341</v>
+      </c>
+      <c r="B251" s="52" t="s">
+        <v>1344</v>
+      </c>
+      <c r="C251" s="52" t="s">
+        <v>96</v>
+      </c>
+      <c r="D251" s="53">
+        <v>1090</v>
+      </c>
       <c r="E251" s="53"/>
       <c r="F251" s="66">
         <v>0</v>
@@ -37682,7 +38040,7 @@
       </c>
       <c r="I251" s="65">
         <f>IF(D251&lt;&gt;"",D251,IFERROR(E251/(IFERROR(SUM(Sales!C:C),0))*(IFERROR(SUM(Purchases!C:C),0)),0))</f>
-        <v>0</v>
+        <v>1090</v>
       </c>
       <c r="J251" s="65">
         <f t="shared" si="19"/>
@@ -37690,33 +38048,47 @@
       </c>
       <c r="K251" s="65">
         <f t="shared" si="20"/>
-        <v>0</v>
+        <v>3270</v>
       </c>
       <c r="L251" s="52"/>
       <c r="M251" s="52"/>
+      <c r="N251" s="47" t="s">
+        <v>678</v>
+      </c>
+      <c r="O251" s="47" t="s">
+        <v>1345</v>
+      </c>
       <c r="P251" s="86"/>
       <c r="S251" s="47"/>
       <c r="T251" s="47"/>
     </row>
-    <row r="252" spans="1:20" ht="16">
-      <c r="A252" s="55"/>
-      <c r="B252" s="55"/>
-      <c r="C252" s="55"/>
-      <c r="D252" s="56"/>
+    <row r="252" spans="1:246" ht="16">
+      <c r="A252" s="55" t="s">
+        <v>1346</v>
+      </c>
+      <c r="B252" s="55" t="s">
+        <v>1347</v>
+      </c>
+      <c r="C252" s="55" t="s">
+        <v>96</v>
+      </c>
+      <c r="D252" s="56">
+        <v>1049</v>
+      </c>
       <c r="E252" s="56"/>
       <c r="F252" s="64">
         <v>0</v>
       </c>
       <c r="G252" s="64">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H252" s="63">
         <f t="shared" si="18"/>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I252" s="63">
         <f>IF(D252&lt;&gt;"",D252,IFERROR(E252/(IFERROR(SUM(Sales!C:C),0))*(IFERROR(SUM(Purchases!C:C),0)),0))</f>
-        <v>0</v>
+        <v>1049</v>
       </c>
       <c r="J252" s="63">
         <f t="shared" si="19"/>
@@ -37724,33 +38096,47 @@
       </c>
       <c r="K252" s="63">
         <f t="shared" si="20"/>
-        <v>0</v>
+        <v>4196</v>
       </c>
       <c r="L252" s="55"/>
       <c r="M252" s="55"/>
+      <c r="N252" s="47" t="s">
+        <v>678</v>
+      </c>
+      <c r="O252" s="47" t="s">
+        <v>1348</v>
+      </c>
       <c r="P252" s="86"/>
       <c r="S252" s="47"/>
       <c r="T252" s="47"/>
     </row>
-    <row r="253" spans="1:20" ht="16">
-      <c r="A253" s="52"/>
-      <c r="B253" s="52"/>
-      <c r="C253" s="52"/>
-      <c r="D253" s="53"/>
+    <row r="253" spans="1:246" ht="16">
+      <c r="A253" s="52" t="s">
+        <v>1349</v>
+      </c>
+      <c r="B253" s="52" t="s">
+        <v>1350</v>
+      </c>
+      <c r="C253" s="52" t="s">
+        <v>96</v>
+      </c>
+      <c r="D253" s="53">
+        <v>1049</v>
+      </c>
       <c r="E253" s="53"/>
       <c r="F253" s="66">
         <v>0</v>
       </c>
       <c r="G253" s="66">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H253" s="65">
         <f t="shared" si="18"/>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I253" s="65">
         <f>IF(D253&lt;&gt;"",D253,IFERROR(E253/(IFERROR(SUM(Sales!C:C),0))*(IFERROR(SUM(Purchases!C:C),0)),0))</f>
-        <v>0</v>
+        <v>1049</v>
       </c>
       <c r="J253" s="65">
         <f t="shared" si="19"/>
@@ -37758,19 +38144,33 @@
       </c>
       <c r="K253" s="65">
         <f t="shared" si="20"/>
-        <v>0</v>
+        <v>4196</v>
       </c>
       <c r="L253" s="52"/>
       <c r="M253" s="52"/>
+      <c r="N253" s="47" t="s">
+        <v>678</v>
+      </c>
+      <c r="O253" s="47" t="s">
+        <v>1348</v>
+      </c>
       <c r="P253" s="86"/>
       <c r="S253" s="47"/>
       <c r="T253" s="47"/>
     </row>
-    <row r="254" spans="1:20" ht="16">
-      <c r="A254" s="55"/>
-      <c r="B254" s="55"/>
-      <c r="C254" s="55"/>
-      <c r="D254" s="56"/>
+    <row r="254" spans="1:246" ht="16">
+      <c r="A254" s="55" t="s">
+        <v>1351</v>
+      </c>
+      <c r="B254" s="55" t="s">
+        <v>1352</v>
+      </c>
+      <c r="C254" s="55" t="s">
+        <v>96</v>
+      </c>
+      <c r="D254" s="56">
+        <v>1322</v>
+      </c>
       <c r="E254" s="56"/>
       <c r="F254" s="64">
         <v>0</v>
@@ -37784,7 +38184,7 @@
       </c>
       <c r="I254" s="63">
         <f>IF(D254&lt;&gt;"",D254,IFERROR(E254/(IFERROR(SUM(Sales!C:C),0))*(IFERROR(SUM(Purchases!C:C),0)),0))</f>
-        <v>0</v>
+        <v>1322</v>
       </c>
       <c r="J254" s="63">
         <f t="shared" si="19"/>
@@ -37792,15 +38192,21 @@
       </c>
       <c r="K254" s="63">
         <f t="shared" si="20"/>
-        <v>0</v>
+        <v>3966</v>
       </c>
       <c r="L254" s="55"/>
       <c r="M254" s="55"/>
+      <c r="N254" s="47" t="s">
+        <v>678</v>
+      </c>
+      <c r="O254" s="47" t="s">
+        <v>1345</v>
+      </c>
       <c r="P254" s="86"/>
       <c r="S254" s="47"/>
       <c r="T254" s="47"/>
     </row>
-    <row r="255" spans="1:20" ht="16">
+    <row r="255" spans="1:246" ht="16">
       <c r="A255" s="52"/>
       <c r="B255" s="52"/>
       <c r="C255" s="52"/>
@@ -37834,7 +38240,7 @@
       <c r="S255" s="47"/>
       <c r="T255" s="47"/>
     </row>
-    <row r="256" spans="1:20" ht="16">
+    <row r="256" spans="1:246" ht="16">
       <c r="A256" s="55"/>
       <c r="B256" s="55"/>
       <c r="C256" s="55"/>
@@ -43836,15 +44242,15 @@
       </c>
       <c r="B8" s="9">
         <f>IFERROR(SUMIF(Purchases!$B:$B,$A8,Purchases!$C:$C),0)</f>
-        <v>262891</v>
+        <v>262941</v>
       </c>
       <c r="C8" s="9">
         <f>SUM($B$8:$B$10)/3</f>
-        <v>188936</v>
+        <v>200621.33333333334</v>
       </c>
       <c r="D8" s="9">
         <f>B8-C8</f>
-        <v>73955</v>
+        <v>62319.666666666657</v>
       </c>
       <c r="E8" s="9">
         <f>IF(Summary!$B$6&gt;0, Summary!$B$6*VLOOKUP($A8,$A$3:$B$5,2,FALSE()),0)</f>
@@ -43852,7 +44258,7 @@
       </c>
       <c r="F8" s="9">
         <f>D8+E8</f>
-        <v>73955</v>
+        <v>62319.666666666657</v>
       </c>
       <c r="G8" s="9">
         <f>IFERROR(SUMIFS($E$13:$E$499,$D$13:$D$499,$A8,$B$13:$B$499,"Contribution"),0)+IFERROR(SUMIFS($E$13:$E$499,$D$13:$D$499,$A8,$B$13:$B$499,"Profit"),0)-IFERROR(SUMIFS($E$13:$E$499,$C$13:$C$499,$A8,$B$13:$B$499,"Contribution"),0)-IFERROR(SUMIFS($E$13:$E$499,$C$13:$C$499,$A8,$B$13:$B$499,"Profit"),0)</f>
@@ -43860,7 +44266,7 @@
       </c>
       <c r="H8" s="73">
         <f>F8-G8</f>
-        <v>55651.66</v>
+        <v>44016.32666666666</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="13.5" customHeight="1">
@@ -43869,15 +44275,15 @@
       </c>
       <c r="B9" s="11">
         <f>IFERROR(SUMIF(Purchases!$B:$B,$A9,Purchases!$C:$C),0)</f>
-        <v>271317</v>
+        <v>306323</v>
       </c>
       <c r="C9" s="11">
         <f>SUM($B$8:$B$10)/3</f>
-        <v>188936</v>
+        <v>200621.33333333334</v>
       </c>
       <c r="D9" s="11">
         <f>B9-C9</f>
-        <v>82381</v>
+        <v>105701.66666666666</v>
       </c>
       <c r="E9" s="11">
         <f>IF(Summary!$B$6&gt;0, Summary!$B$6*VLOOKUP($A9,$A$3:$B$5,2,FALSE()),0)</f>
@@ -43885,7 +44291,7 @@
       </c>
       <c r="F9" s="11">
         <f>D9+E9</f>
-        <v>82381</v>
+        <v>105701.66666666666</v>
       </c>
       <c r="G9" s="11">
         <f>IFERROR(SUMIFS($E$13:$E$499,$D$13:$D$499,$A9,$B$13:$B$499,"Contribution"),0)+IFERROR(SUMIFS($E$13:$E$499,$D$13:$D$499,$A9,$B$13:$B$499,"Profit"),0)-IFERROR(SUMIFS($E$13:$E$499,$C$13:$C$499,$A9,$B$13:$B$499,"Contribution"),0)-IFERROR(SUMIFS($E$13:$E$499,$C$13:$C$499,$A9,$B$13:$B$499,"Profit"),0)</f>
@@ -43893,7 +44299,7 @@
       </c>
       <c r="H9" s="74">
         <f>F9-G9</f>
-        <v>40741.67</v>
+        <v>64062.336666666655</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="13.5" customHeight="1">
@@ -43906,11 +44312,11 @@
       </c>
       <c r="C10" s="9">
         <f>SUM($B$8:$B$10)/3</f>
-        <v>188936</v>
+        <v>200621.33333333334</v>
       </c>
       <c r="D10" s="9">
         <f>B10-C10</f>
-        <v>-156336</v>
+        <v>-168021.33333333334</v>
       </c>
       <c r="E10" s="9">
         <f>IF(Summary!$B$6&gt;0, Summary!$B$6*VLOOKUP($A10,$A$3:$B$5,2,FALSE()),0)</f>
@@ -43918,7 +44324,7 @@
       </c>
       <c r="F10" s="9">
         <f>D10+E10</f>
-        <v>-156336</v>
+        <v>-168021.33333333334</v>
       </c>
       <c r="G10" s="9">
         <f>IFERROR(SUMIFS($E$13:$E$499,$D$13:$D$499,$A10,$B$13:$B$499,"Contribution"),0)+IFERROR(SUMIFS($E$13:$E$499,$D$13:$D$499,$A10,$B$13:$B$499,"Profit"),0)-IFERROR(SUMIFS($E$13:$E$499,$C$13:$C$499,$A10,$B$13:$B$499,"Contribution"),0)-IFERROR(SUMIFS($E$13:$E$499,$C$13:$C$499,$A10,$B$13:$B$499,"Profit"),0)</f>
@@ -43926,7 +44332,7 @@
       </c>
       <c r="H10" s="73">
         <f>F10-G10</f>
-        <v>-96393.33</v>
+        <v>-108078.66333333334</v>
       </c>
     </row>
     <row r="12" spans="1:8" s="75" customFormat="1" ht="15.75" customHeight="1">
@@ -44343,7 +44749,7 @@
       </c>
       <c r="B4" s="9">
         <f>IFERROR(SUMIFS(Sales!$C:$C,Sales!$E:$E,$A4,Sales!$I:$I,"Completed"),0)</f>
-        <v>472938</v>
+        <v>476538</v>
       </c>
       <c r="C4" s="9">
         <f>VLOOKUP($A4,PartnerShares!$A$3:$B$5,2,FALSE())</f>
@@ -44351,11 +44757,11 @@
       </c>
       <c r="D4" s="9">
         <f>Summary!$B$4*C4</f>
-        <v>180400.07279999999</v>
+        <v>181600.31279999999</v>
       </c>
       <c r="E4" s="9">
         <f>B4-D4</f>
-        <v>292537.92720000003</v>
+        <v>294937.68720000004</v>
       </c>
       <c r="F4" s="9">
         <f>IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$D$13:$D$499,$A4,PartnerShares!$B$13:$B$499,"Cash"),0)-IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$C$13:$C$499,$A4,PartnerShares!$B$13:$B$499,"Cash"),0)</f>
@@ -44363,7 +44769,7 @@
       </c>
       <c r="G4" s="73">
         <f>E4+F4</f>
-        <v>155227.90120000002</v>
+        <v>157627.66120000003</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="13.5" customHeight="1">
@@ -44380,11 +44786,11 @@
       </c>
       <c r="D5" s="11">
         <f>Summary!$B$4*C5</f>
-        <v>180291.85440000001</v>
+        <v>181491.3744</v>
       </c>
       <c r="E5" s="11">
         <f>B5-D5</f>
-        <v>-125667.85440000001</v>
+        <v>-126867.3744</v>
       </c>
       <c r="F5" s="11">
         <f>IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$D$13:$D$499,$A5,PartnerShares!$B$13:$B$499,"Cash"),0)-IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$C$13:$C$499,$A5,PartnerShares!$B$13:$B$499,"Cash"),0)</f>
@@ -44392,7 +44798,7 @@
       </c>
       <c r="G5" s="74">
         <f>E5+F5</f>
-        <v>-54080.81240000001</v>
+        <v>-55280.332399999999</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="13.5" customHeight="1">
@@ -44409,11 +44815,11 @@
       </c>
       <c r="D6" s="9">
         <f>Summary!$B$4*C6</f>
-        <v>180400.07279999999</v>
+        <v>181600.31279999999</v>
       </c>
       <c r="E6" s="9">
         <f>B6-D6</f>
-        <v>-167870.07279999999</v>
+        <v>-169070.31279999999</v>
       </c>
       <c r="F6" s="9">
         <f>IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$D$13:$D$499,$A6,PartnerShares!$B$13:$B$499,"Cash"),0)-IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$C$13:$C$499,$A6,PartnerShares!$B$13:$B$499,"Cash"),0)</f>
@@ -44421,7 +44827,7 @@
       </c>
       <c r="G6" s="73">
         <f>E6+F6</f>
-        <v>-102147.08879999998</v>
+        <v>-103347.32879999997</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="13.5" customHeight="1">

</xml_diff>